<commit_message>
Track ADIF TCI split and diagnostic export stages
</commit_message>
<xml_diff>
--- a/outputs/feature-matrix-2026-10-16/OM0RX-xLog_Feature_Comparison_2026-10-16.xlsx
+++ b/outputs/feature-matrix-2026-10-16/OM0RX-xLog_Feature_Comparison_2026-10-16.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Matrix" sheetId="1" r:id="R36b729aae38642c1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Outstanding" sheetId="2" r:id="R4ff2ab3bfc414949"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enhancement Review" sheetId="3" r:id="R41c86d4ff0554ba5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="4" r:id="R9ab3f7bf71fa43c2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Matrix" sheetId="1" r:id="Rda3195638bfa4672"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Outstanding" sheetId="2" r:id="Rdcc0c94b16b44760"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enhancement Review" sheetId="3" r:id="Rec41ba8b89fc44af"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="4" r:id="Rb76840bd2dd04850"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -852,12 +852,12 @@
       <x:c r="E9" s="59"/>
       <x:c r="F9" s="59"/>
     </x:row>
-    <x:row r="10" ht="48" hidden="0" customHeight="1">
+    <x:row r="10" ht="60" hidden="0" customHeight="1">
       <x:c r="A10" s="66" t="str">
         <x:v>ADIF field preservation</x:v>
       </x:c>
       <x:c r="B10" s="67" t="str">
-        <x:v>Source complete for the reviewed compatibility stage — local records retain a JSON field bag; unknown/custom fields, Unicode, station/contact and RX/TX data survive supported ADI/ADX round trips. UTF-8 byte scanning and FT4/FT2/JTTY MFSK-submode export are fixed; the full 3.1.8 enum/deprecation audit remains open and ADIF_VER stays 3.1.7.</x:v>
+        <x:v>Source complete for three reviewed compatibility stages — local records retain a JSON field bag; unknown/custom fields, Unicode, station/contact and RX/TX data survive supported ADI/ADX round trips. UTF-8 byte scanning, FT4/FT2/JTTY MFSK-submode export and C4FM/DSTAR DIGITALVOICE-submode export are fixed. Strict raw deprecated-mode ADX import and the remaining 3.1.8 enum/deprecation audit remain open; ADIF_VER stays 3.1.7.</x:v>
       </x:c>
       <x:c r="C10" s="67" t="str">
         <x:v>Documented — import/export plus four user-definable logging fields.</x:v>
@@ -980,12 +980,12 @@
       <x:c r="E17" s="59"/>
       <x:c r="F17" s="59"/>
     </x:row>
-    <x:row r="18" ht="48" hidden="0" customHeight="1">
+    <x:row r="18" ht="60" hidden="0" customHeight="1">
       <x:c r="A18" s="66" t="str">
         <x:v>Connection Doctor and support preview</x:v>
       </x:c>
       <x:c r="B18" s="67" t="str">
-        <x:v>Passive native window complete — fixed provider/configuration/connection/freshness/capability stages consume only already-retained allowlisted state. The typed preview cannot represent secrets, endpoints, identifiers, raw errors, radio values, timestamps or log contents. Opt-in redacted export and exact-package/provider acceptance remain open.</x:v>
+        <x:v>Passive native window plus click-only redacted export source complete — fixed provider/configuration/connection/freshness/capability stages consume only already-retained allowlisted state. The typed preview and exported JSON cannot represent secrets, endpoints, identifiers, raw errors, radio values, timestamps or log contents. Exact-package Save/Cancel/overwrite and retained-provider acceptance remain open.</x:v>
       </x:c>
       <x:c r="C18" s="67" t="str">
         <x:v>Not established as a comparable product surface in reviewed primary evidence.</x:v>
@@ -1300,12 +1300,12 @@
       <x:c r="E37" s="59"/>
       <x:c r="F37" s="59"/>
     </x:row>
-    <x:row r="38" ht="72" hidden="0" customHeight="1">
+    <x:row r="38" ht="84" hidden="0" customHeight="1">
       <x:c r="A38" s="66" t="str">
         <x:v>TCI rig control — SunSDR/ExpertSDR and compatible servers</x:v>
       </x:c>
       <x:c r="B38" s="67" t="str">
-        <x:v>Source complete through observed receive-frequency/mode tuning and TRX-wide receive-filter adjustment — bounded protocol/session, exact discovery, producer-time freshness, saved credential-free ws/wss setup and stale-aware UI. Explicit controls use the existing connection, durable no-replay receipts and newer exact readback. The filter has an app-local ±24 kHz bound and no longer misuses IF_LIMITS. Transmit/PTT, split/TX-VFO, spots, audio/IQ and package/live-server acceptance remain open.</x:v>
+        <x:v>Source complete through observed receive-frequency/mode tuning, TRX-wide receive-filter adjustment and configured-TRX split observation — bounded protocol/session, exact discovery, producer-time freshness, saved credential-free ws/wss setup and stale-aware UI. Explicit controls use the existing connection, durable no-replay receipts and newer exact readback. The filter has an app-local ±24 kHz bound and no longer misuses IF_LIMITS. The pinned protocol exposes no authoritative TX-VFO/frequency report, so neither is inferred. Transmit/PTT, split/TX-VFO controls, spots, audio/IQ and package/live-server acceptance remain open.</x:v>
       </x:c>
       <x:c r="C38" s="67" t="str">
         <x:v>Not established in the reviewed primary RUMlogNG evidence.</x:v>
@@ -2730,7 +2730,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6717d7c22a524002"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R88b11e46e9054047"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2914,7 +2914,7 @@
         <x:v>RUMlogNG edit/search/export workflow</x:v>
       </x:c>
     </x:row>
-    <x:row r="12" ht="24" hidden="0" customHeight="1">
+    <x:row r="12" ht="36" hidden="0" customHeight="1">
       <x:c r="A12" s="66" t="str">
         <x:v>P0</x:v>
       </x:c>
@@ -2922,10 +2922,10 @@
         <x:v>ADIF 3.1.8 conformance</x:v>
       </x:c>
       <x:c r="C12" s="67" t="str">
-        <x:v>First compatibility fixes complete</x:v>
+        <x:v>Three compatibility fixes complete</x:v>
       </x:c>
       <x:c r="D12" s="67" t="str">
-        <x:v>Complete enum/deprecation and MODE/SUBMODE audit before changing ADIF_VER; run copied-log/package and service-specific interoperability acceptance.</x:v>
+        <x:v>Add strict raw deprecated-mode ADX import coverage and complete the remaining enum/deprecation and MODE/SUBMODE audit before changing ADIF_VER; run copied-log/package and service-specific interoperability acceptance.</x:v>
       </x:c>
       <x:c r="E12" s="67" t="str">
         <x:v>Pinned official fixtures, copied-log round trip and exact package</x:v>
@@ -2962,10 +2962,10 @@
         <x:v>Full TCI radio provider</x:v>
       </x:c>
       <x:c r="C14" s="67" t="str">
-        <x:v>Observed receive tune and filter source complete</x:v>
+        <x:v>Receive tune/filter and passive split observation source complete</x:v>
       </x:c>
       <x:c r="D14" s="67" t="str">
-        <x:v>Extend the existing no-replay owner with separately reviewed split/TX-VFO, urgent release, spots and optional audio/IQ slices; transmit/PTT requires its own explicit authority.</x:v>
+        <x:v>Extend the existing no-replay owner with separately reviewed split/TX-VFO controls, urgent release, spots and optional audio/IQ slices; do not infer unavailable TX-VFO telemetry and keep transmit/PTT behind its own explicit authority.</x:v>
       </x:c>
       <x:c r="E14" s="67" t="str">
         <x:v>Simulated-server races, package tests, then operator-controlled SunSDR acceptance</x:v>
@@ -3102,10 +3102,10 @@
         <x:v>Connection Doctor surface</x:v>
       </x:c>
       <x:c r="C21" s="67" t="str">
-        <x:v>Read-only native source window complete</x:v>
+        <x:v>Native window and redacted export source complete</x:v>
       </x:c>
       <x:c r="D21" s="67" t="str">
-        <x:v>Add only explicit opt-in redacted export, then verify exact package and real retained-provider states.</x:v>
+        <x:v>Verify native Save/Cancel/overwrite in the exact package and real retained-provider states; preserve the closed allowlist and no-action boundary.</x:v>
       </x:c>
       <x:c r="E21" s="67" t="str">
         <x:v>Privacy review, exact-package and retained-provider acceptance</x:v>
@@ -4620,7 +4620,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2701b1497ad3417d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7280f261a56d461d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4755,7 +4755,7 @@
       </x:c>
       <x:c r="F9" s="59"/>
     </x:row>
-    <x:row r="10" ht="15" hidden="0" customHeight="1">
+    <x:row r="10" ht="24" hidden="0" customHeight="1">
       <x:c r="A10" s="66" t="str">
         <x:v>R04</x:v>
       </x:c>
@@ -4763,13 +4763,13 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="C10" s="67" t="str">
-        <x:v>First compatibility fixes complete</x:v>
+        <x:v>Three compatibility fixes complete</x:v>
       </x:c>
       <x:c r="D10" s="67" t="str">
         <x:v>ADIF parser/writer and frontend transfer</x:v>
       </x:c>
       <x:c r="E10" s="67" t="str">
-        <x:v>Finish 3.1.8 enum/deprecation audit before header bump.</x:v>
+        <x:v>Add strict raw deprecated-mode ADX import coverage and finish the remaining 3.1.8 enum/deprecation audit before header bump.</x:v>
       </x:c>
       <x:c r="F10" s="59"/>
     </x:row>
@@ -4979,13 +4979,13 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="C22" s="67" t="str">
-        <x:v>Retained read-only native window complete; export/package open</x:v>
+        <x:v>Native window and click-only redacted export source complete; package open</x:v>
       </x:c>
       <x:c r="D22" s="67" t="str">
         <x:v>Retained station diagnostics only</x:v>
       </x:c>
       <x:c r="E22" s="67" t="str">
-        <x:v>Add only explicit opt-in allowlist export; package-test retained states.</x:v>
+        <x:v>Package-test Save/Cancel/overwrite and real retained states; preserve the closed allowlist.</x:v>
       </x:c>
       <x:c r="F22" s="59"/>
     </x:row>
@@ -6507,7 +6507,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R20b008ca4cce48d8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R41bd2164c09243d5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6587,7 +6587,7 @@
         <x:v>OM0RX-xLog</x:v>
       </x:c>
       <x:c r="B7" s="65" t="str">
-        <x:v>Current source checkpoint 31f2f2880de55e72ace5cd44a8ad0c68aa79d443</x:v>
+        <x:v>Current implementation checkpoint c27dec859f211524ddea68658c500d4388ca6ffc</x:v>
       </x:c>
       <x:c r="C7" s="65" t="str">
         <x:v>2026-10-16</x:v>
@@ -6598,18 +6598,18 @@
       <x:c r="E7" s="59"/>
       <x:c r="F7" s="59"/>
     </x:row>
-    <x:row r="8" ht="36" hidden="0" customHeight="1">
+    <x:row r="8" ht="48" hidden="0" customHeight="1">
       <x:c r="A8" s="66" t="str">
         <x:v>OM0RX-xLog</x:v>
       </x:c>
       <x:c r="B8" s="67" t="str">
-        <x:v>https://github.com/oliverbross/OM0RX-xLog/commit/31f2f2880de55e72ace5cd44a8ad0c68aa79d443</x:v>
+        <x:v>https://github.com/oliverbross/OM0RX-xLog/commit/c27dec859f211524ddea68658c500d4388ca6ffc</x:v>
       </x:c>
       <x:c r="C8" s="67" t="str">
         <x:v>2026-10-16</x:v>
       </x:c>
       <x:c r="D8" s="67" t="str">
-        <x:v>Exact committed baseline including observed TCI receive tuning/filter control, native Operating Goals and Connection Doctor windows, cloneable saved filters, responsive alert/reference-window improvements, PJ/DXCC preview and ADIF fixes, and the independent Previous QSOs window.</x:v>
+        <x:v>Exact committed implementation baseline including observed TCI receive tune/filter and split telemetry, native Operating Goals, Connection Doctor with redacted export, cloneable saved filters, responsive alert/reference-window improvements, PJ/DXCC preview, three bounded ADIF compatibility fixes, and the independent Previous QSOs window.</x:v>
       </x:c>
       <x:c r="E8" s="59"/>
       <x:c r="F8" s="59"/>
@@ -8236,7 +8236,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re3bb9d0a8c79437c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rafceee808e204629"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Track ADX build and TCI telemetry follow-ups
</commit_message>
<xml_diff>
--- a/outputs/feature-matrix-2026-10-16/OM0RX-xLog_Feature_Comparison_2026-10-16.xlsx
+++ b/outputs/feature-matrix-2026-10-16/OM0RX-xLog_Feature_Comparison_2026-10-16.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Matrix" sheetId="1" r:id="Rda3195638bfa4672"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Outstanding" sheetId="2" r:id="Rdcc0c94b16b44760"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enhancement Review" sheetId="3" r:id="Rec41ba8b89fc44af"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="4" r:id="Rb76840bd2dd04850"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Matrix" sheetId="1" r:id="R143da979c0c545cc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Outstanding" sheetId="2" r:id="R28315ee573654dbd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enhancement Review" sheetId="3" r:id="R43da29c98b6044d7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="4" r:id="Rd80ede5ba6d94201"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -857,7 +857,7 @@
         <x:v>ADIF field preservation</x:v>
       </x:c>
       <x:c r="B10" s="67" t="str">
-        <x:v>Source complete for three reviewed compatibility stages — local records retain a JSON field bag; unknown/custom fields, Unicode, station/contact and RX/TX data survive supported ADI/ADX round trips. UTF-8 byte scanning, FT4/FT2/JTTY MFSK-submode export and C4FM/DSTAR DIGITALVOICE-submode export are fixed. Strict raw deprecated-mode ADX import and the remaining 3.1.8 enum/deprecation audit remain open; ADIF_VER stays 3.1.7.</x:v>
+        <x:v>Source complete for four reviewed compatibility stages — local records retain a JSON field bag; unknown/custom fields, Unicode, station/contact and RX/TX data survive supported ADI/ADX round trips. UTF-8 byte scanning, FT4/FT2/JTTY MFSK-submode export, C4FM/DSTAR DIGITALVOICE-submode export and import-only raw deprecated-mode ADX acceptance are fixed. The remaining 3.1.8 enum/deprecation audit remains open; ADIF_VER stays 3.1.7.</x:v>
       </x:c>
       <x:c r="C10" s="67" t="str">
         <x:v>Documented — import/export plus four user-definable logging fields.</x:v>
@@ -980,12 +980,12 @@
       <x:c r="E17" s="59"/>
       <x:c r="F17" s="59"/>
     </x:row>
-    <x:row r="18" ht="60" hidden="0" customHeight="1">
+    <x:row r="18" ht="72" hidden="0" customHeight="1">
       <x:c r="A18" s="66" t="str">
         <x:v>Connection Doctor and support preview</x:v>
       </x:c>
       <x:c r="B18" s="67" t="str">
-        <x:v>Passive native window plus click-only redacted export source complete — fixed provider/configuration/connection/freshness/capability stages consume only already-retained allowlisted state. The typed preview and exported JSON cannot represent secrets, endpoints, identifiers, raw errors, radio values, timestamps or log contents. Exact-package Save/Cancel/overwrite and retained-provider acceptance remain open.</x:v>
+        <x:v>Passive native window plus click-only redacted export source complete — fixed provider/configuration/connection/freshness/capability stages consume only already-retained allowlisted state. The typed preview and exported JSON cannot represent secrets, endpoints, identifiers, raw errors, radio values, timestamps or log contents. The former late-CSS bundle gate is fixed; exact-package Save/Cancel/overwrite and retained-provider acceptance remain open.</x:v>
       </x:c>
       <x:c r="C18" s="67" t="str">
         <x:v>Not established as a comparable product surface in reviewed primary evidence.</x:v>
@@ -1252,12 +1252,12 @@
       <x:c r="E34" s="59"/>
       <x:c r="F34" s="59"/>
     </x:row>
-    <x:row r="35" ht="48" hidden="0" customHeight="1">
+    <x:row r="35" ht="60" hidden="0" customHeight="1">
       <x:c r="A35" s="66" t="str">
         <x:v>Responsive detached windows</x:v>
       </x:c>
       <x:c r="B35" s="67" t="str">
-        <x:v>Partial — common chrome removal and targeted fixes cover many roles. Detached Propagation rows now align at compact widths; Station Status and Rotor use the shared inset and Rotor starts at the top. Focused 31/31 UI plus rendered-geometry checks pass; the full packaged all-window resolution/scale matrix remains outstanding.</x:v>
+        <x:v>Partial — common chrome removal and targeted fixes cover many roles. Detached Propagation rows align; Station Status and Rotor use the shared inset; Rotor starts at the top. Focused 31/31 UI, rendered geometry, Band Map 380×1100, Callsign Intelligence 680×500 and Rotor 676×500/400×600 browser checks pass without page overflow. The packaged all-window resolution/scale matrix remains outstanding.</x:v>
       </x:c>
       <x:c r="C35" s="67" t="str">
         <x:v>Mature native macOS window behavior is the reference; exact responsive tests were not obtained.</x:v>
@@ -1300,12 +1300,12 @@
       <x:c r="E37" s="59"/>
       <x:c r="F37" s="59"/>
     </x:row>
-    <x:row r="38" ht="84" hidden="0" customHeight="1">
+    <x:row r="38" ht="96" hidden="0" customHeight="1">
       <x:c r="A38" s="66" t="str">
         <x:v>TCI rig control — SunSDR/ExpertSDR and compatible servers</x:v>
       </x:c>
       <x:c r="B38" s="67" t="str">
-        <x:v>Source complete through observed receive-frequency/mode tuning, TRX-wide receive-filter adjustment and configured-TRX split observation — bounded protocol/session, exact discovery, producer-time freshness, saved credential-free ws/wss setup and stale-aware UI. Explicit controls use the existing connection, durable no-replay receipts and newer exact readback. The filter has an app-local ±24 kHz bound and no longer misuses IF_LIMITS. The pinned protocol exposes no authoritative TX-VFO/frequency report, so neither is inferred. Transmit/PTT, split/TX-VFO controls, spots, audio/IQ and package/live-server acceptance remain open.</x:v>
+        <x:v>Source complete through observed receive-frequency/mode tuning, TRX-wide receive-filter adjustment, configured-TRX split observation and server-global TX-frequency telemetry — bounded protocol/session, exact discovery, producer-time freshness, saved credential-free ws/wss setup and stale-aware UI. Explicit controls use the existing connection, durable no-replay receipts and newer exact readback. The filter has an app-local ±24 kHz bound and no longer misuses IF_LIMITS. Global TX frequency has no TRX/channel/VFO identity and is never promoted to configured evidence or authority. Transmit/PTT, split/TX-VFO controls, spots, audio/IQ and package/live-server acceptance remain open.</x:v>
       </x:c>
       <x:c r="C38" s="67" t="str">
         <x:v>Not established in the reviewed primary RUMlogNG evidence.</x:v>
@@ -2730,7 +2730,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R88b11e46e9054047"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd07c3420df4c49c4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2922,10 +2922,10 @@
         <x:v>ADIF 3.1.8 conformance</x:v>
       </x:c>
       <x:c r="C12" s="67" t="str">
-        <x:v>Three compatibility fixes complete</x:v>
+        <x:v>Four compatibility fixes complete</x:v>
       </x:c>
       <x:c r="D12" s="67" t="str">
-        <x:v>Add strict raw deprecated-mode ADX import coverage and complete the remaining enum/deprecation and MODE/SUBMODE audit before changing ADIF_VER; run copied-log/package and service-specific interoperability acceptance.</x:v>
+        <x:v>Complete the remaining enum/deprecation and MODE/SUBMODE audit before changing ADIF_VER; run copied-log/package and service-specific interoperability acceptance.</x:v>
       </x:c>
       <x:c r="E12" s="67" t="str">
         <x:v>Pinned official fixtures, copied-log round trip and exact package</x:v>
@@ -2954,7 +2954,7 @@
         <x:v>Official/date-qualified CTY rules</x:v>
       </x:c>
     </x:row>
-    <x:row r="14" ht="36" hidden="0" customHeight="1">
+    <x:row r="14" ht="48" hidden="0" customHeight="1">
       <x:c r="A14" s="66" t="str">
         <x:v>P1</x:v>
       </x:c>
@@ -2962,10 +2962,10 @@
         <x:v>Full TCI radio provider</x:v>
       </x:c>
       <x:c r="C14" s="67" t="str">
-        <x:v>Receive tune/filter and passive split observation source complete</x:v>
+        <x:v>Receive tune/filter, passive split and global TX-frequency observation source complete</x:v>
       </x:c>
       <x:c r="D14" s="67" t="str">
-        <x:v>Extend the existing no-replay owner with separately reviewed split/TX-VFO controls, urgent release, spots and optional audio/IQ slices; do not infer unavailable TX-VFO telemetry and keep transmit/PTT behind its own explicit authority.</x:v>
+        <x:v>Extend the existing no-replay owner with separately reviewed split/TX-VFO controls, urgent release and optional audio/IQ slices; do not assign global TX frequency to a TRX/VFO. The pinned protocol has no received spot inventory, and transmit/PTT keeps its own explicit authority.</x:v>
       </x:c>
       <x:c r="E14" s="67" t="str">
         <x:v>Simulated-server races, package tests, then operator-controlled SunSDR acceptance</x:v>
@@ -4620,7 +4620,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7280f261a56d461d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra4950aa38de4490e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4755,7 +4755,7 @@
       </x:c>
       <x:c r="F9" s="59"/>
     </x:row>
-    <x:row r="10" ht="24" hidden="0" customHeight="1">
+    <x:row r="10" ht="15" hidden="0" customHeight="1">
       <x:c r="A10" s="66" t="str">
         <x:v>R04</x:v>
       </x:c>
@@ -4763,13 +4763,13 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="C10" s="67" t="str">
-        <x:v>Three compatibility fixes complete</x:v>
+        <x:v>Four compatibility fixes complete</x:v>
       </x:c>
       <x:c r="D10" s="67" t="str">
         <x:v>ADIF parser/writer and frontend transfer</x:v>
       </x:c>
       <x:c r="E10" s="67" t="str">
-        <x:v>Add strict raw deprecated-mode ADX import coverage and finish the remaining 3.1.8 enum/deprecation audit before header bump.</x:v>
+        <x:v>Finish the remaining 3.1.8 enum/deprecation audit before header bump.</x:v>
       </x:c>
       <x:c r="F10" s="59"/>
     </x:row>
@@ -4781,7 +4781,7 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="C11" s="67" t="str">
-        <x:v>Detached geometry follow-up source complete; acceptance open</x:v>
+        <x:v>Detached geometry and targeted browser checks complete; package acceptance open</x:v>
       </x:c>
       <x:c r="D11" s="67" t="str">
         <x:v>Native window geometry and Canvas/Separate Windows owner</x:v>
@@ -6507,7 +6507,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R41bd2164c09243d5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2c1c7876e6a34170"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6587,7 +6587,7 @@
         <x:v>OM0RX-xLog</x:v>
       </x:c>
       <x:c r="B7" s="65" t="str">
-        <x:v>Current implementation checkpoint c27dec859f211524ddea68658c500d4388ca6ffc</x:v>
+        <x:v>Current implementation checkpoint b6bf7c1b36e2a8175b468719d4cf4c390316b2ec</x:v>
       </x:c>
       <x:c r="C7" s="65" t="str">
         <x:v>2026-10-16</x:v>
@@ -6603,13 +6603,13 @@
         <x:v>OM0RX-xLog</x:v>
       </x:c>
       <x:c r="B8" s="67" t="str">
-        <x:v>https://github.com/oliverbross/OM0RX-xLog/commit/c27dec859f211524ddea68658c500d4388ca6ffc</x:v>
+        <x:v>https://github.com/oliverbross/OM0RX-xLog/commit/b6bf7c1b36e2a8175b468719d4cf4c390316b2ec</x:v>
       </x:c>
       <x:c r="C8" s="67" t="str">
         <x:v>2026-10-16</x:v>
       </x:c>
       <x:c r="D8" s="67" t="str">
-        <x:v>Exact committed implementation baseline including observed TCI receive tune/filter and split telemetry, native Operating Goals, Connection Doctor with redacted export, cloneable saved filters, responsive alert/reference-window improvements, PJ/DXCC preview, three bounded ADIF compatibility fixes, and the independent Previous QSOs window.</x:v>
+        <x:v>Exact committed implementation baseline including observed TCI receive tune/filter, split and global TX-frequency telemetry, native Operating Goals, Connection Doctor with redacted export, cloneable saved filters, responsive window improvements, PJ/DXCC preview, four bounded ADIF compatibility fixes, and the independent Previous QSOs window.</x:v>
       </x:c>
       <x:c r="E8" s="59"/>
       <x:c r="F8" s="59"/>
@@ -8236,7 +8236,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rafceee808e204629"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0c492a533f194b84"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Track online log ADIF and TCI follow-ups
</commit_message>
<xml_diff>
--- a/outputs/feature-matrix-2026-10-16/OM0RX-xLog_Feature_Comparison_2026-10-16.xlsx
+++ b/outputs/feature-matrix-2026-10-16/OM0RX-xLog_Feature_Comparison_2026-10-16.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Matrix" sheetId="1" r:id="R143da979c0c545cc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Outstanding" sheetId="2" r:id="R28315ee573654dbd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enhancement Review" sheetId="3" r:id="R43da29c98b6044d7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="4" r:id="Rd80ede5ba6d94201"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Matrix" sheetId="1" r:id="R392661c588cb4fc7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Outstanding" sheetId="2" r:id="Rceb75a0f3e32431e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enhancement Review" sheetId="3" r:id="R236656e92ce84aff"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="4" r:id="R86507dcab7304199"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -482,7 +482,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="FeatureComparisonTable" displayName="FeatureComparisonTable" ref="A6:D51" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="FeatureComparisonTable" displayName="FeatureComparisonTable" ref="A6:D52" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="4">
     <x:tableColumn id="1" name="Feature"/>
     <x:tableColumn id="2" name="OM0RX-xLog"/>
@@ -494,7 +494,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="OutstandingWorkTable" displayName="OutstandingWorkTable" ref="A6:F26" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="OutstandingWorkTable" displayName="OutstandingWorkTable" ref="A6:F27" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="6">
     <x:tableColumn id="1" name="Priority"/>
     <x:tableColumn id="2" name="Feature or decision"/>
@@ -857,7 +857,7 @@
         <x:v>ADIF field preservation</x:v>
       </x:c>
       <x:c r="B10" s="67" t="str">
-        <x:v>Source complete for four reviewed compatibility stages — local records retain a JSON field bag; unknown/custom fields, Unicode, station/contact and RX/TX data survive supported ADI/ADX round trips. UTF-8 byte scanning, FT4/FT2/JTTY MFSK-submode export, C4FM/DSTAR DIGITALVOICE-submode export and import-only raw deprecated-mode ADX acceptance are fixed. The remaining 3.1.8 enum/deprecation audit remains open; ADIF_VER stays 3.1.7.</x:v>
+        <x:v>Source complete for five reviewed compatibility stages — local records retain a JSON field bag; unknown/custom fields, Unicode, station/contact and RX/TX data survive supported ADI/ADX round trips. UTF-8 byte scanning, FT4/FT2/JTTY MFSK-submode export, C4FM/DSTAR DIGITALVOICE-submode handling and import-only PSK31 to PSK/PSK31 normalization are fixed. The remaining 3.1.8 enum/deprecation audit remains open; ADIF_VER stays 3.1.7.</x:v>
       </x:c>
       <x:c r="C10" s="67" t="str">
         <x:v>Documented — import/export plus four user-definable logging fields.</x:v>
@@ -1076,459 +1076,467 @@
       <x:c r="E23" s="59"/>
       <x:c r="F23" s="59"/>
     </x:row>
-    <x:row r="24" ht="24" hidden="0" customHeight="1">
+    <x:row r="24" ht="48" hidden="0" customHeight="1">
       <x:c r="A24" s="66" t="str">
-        <x:v>HRDLog.net upload</x:v>
+        <x:v>Online-log follow-up evidence</x:v>
       </x:c>
       <x:c r="B24" s="67" t="str">
-        <x:v>Outstanding — deferred until the current official service contract is verified and implemented behind the same vault/receipt/no-replay boundary.</x:v>
+        <x:v>Core projection source complete — canonical QRZ/Club Log receipts expose delivery state, revision currency and attempt age while retained paper/LoTW/eQSL confirmations remain separate. Provider acceptance/match age and sponsor credit stay explicitly unknown; route/UI and live-account acceptance remain open.</x:v>
       </x:c>
       <x:c r="C24" s="67" t="str">
-        <x:v>Documented via the separate real-time upload utility.</x:v>
+        <x:v>Documented service status and confirmation workflows; exact evidence boundaries were not audited.</x:v>
       </x:c>
       <x:c r="D24" s="67" t="str">
-        <x:v>Documented — HRDLog.net integration.</x:v>
+        <x:v>Documented online-log integrations; exact evidence boundaries were not audited.</x:v>
       </x:c>
       <x:c r="E24" s="59"/>
       <x:c r="F24" s="59"/>
     </x:row>
     <x:row r="25" ht="24" hidden="0" customHeight="1">
       <x:c r="A25" s="66" t="str">
-        <x:v>Direct LoTW and eQSL workflows</x:v>
+        <x:v>HRDLog.net upload</x:v>
       </x:c>
       <x:c r="B25" s="67" t="str">
-        <x:v>Outstanding as independent providers — confirmation fields and Wavelog refresh are supported, but direct credential/upload/download owners remain separate programmes.</x:v>
+        <x:v>Outstanding — deferred until the current official service contract is verified and implemented behind the same vault/receipt/no-replay boundary.</x:v>
       </x:c>
       <x:c r="C25" s="67" t="str">
-        <x:v>Documented — direct upload/download, QSL statistics and paper-QSL workflows.</x:v>
+        <x:v>Documented via the separate real-time upload utility.</x:v>
       </x:c>
       <x:c r="D25" s="67" t="str">
-        <x:v>Documented — LoTW and eQSL integration; TQSL is optional for LoTW and eQSL can download QSL pictures.</x:v>
+        <x:v>Documented — HRDLog.net integration.</x:v>
       </x:c>
       <x:c r="E25" s="59"/>
       <x:c r="F25" s="59"/>
     </x:row>
     <x:row r="26" ht="24" hidden="0" customHeight="1">
       <x:c r="A26" s="66" t="str">
-        <x:v>WSJT-X Logged ADIF UDP intake</x:v>
+        <x:v>Direct LoTW and eQSL workflows</x:v>
       </x:c>
       <x:c r="B26" s="67" t="str">
-        <x:v>Source complete — explicit default-off receive-only listener for official Logged ADIF messages; loopback/multicast validation and duplicate-safe local save; live WSJT-X acceptance open.</x:v>
+        <x:v>Outstanding as independent providers — confirmation fields and Wavelog refresh are supported, but direct credential/upload/download owners remain separate programmes.</x:v>
       </x:c>
       <x:c r="C26" s="67" t="str">
-        <x:v>Documented / locally inventoried — configurable WSJT-X UDP logging and save choices.</x:v>
+        <x:v>Documented — direct upload/download, QSL statistics and paper-QSL workflows.</x:v>
       </x:c>
       <x:c r="D26" s="67" t="str">
-        <x:v>Documented — WSJT-X integration; source audit shows one configurable unicast/multicast receiver and QSO Logged/Logged ADIF parsing.</x:v>
+        <x:v>Documented — LoTW and eQSL integration; TQSL is optional for LoTW and eQSL can download QSL pictures.</x:v>
       </x:c>
       <x:c r="E26" s="59"/>
       <x:c r="F26" s="59"/>
     </x:row>
     <x:row r="27" ht="24" hidden="0" customHeight="1">
       <x:c r="A27" s="66" t="str">
-        <x:v>WSJT-X CQ activity and novelty</x:v>
+        <x:v>WSJT-X Logged ADIF UDP intake</x:v>
       </x:c>
       <x:c r="B27" s="67" t="str">
-        <x:v>Source complete — bounded receive-only FT8/FT4 CQ activity feeds named alerts with current local call/DXCC novelty; no reply, CAT, PTT or save authority.</x:v>
+        <x:v>Source complete — explicit default-off receive-only listener for official Logged ADIF messages; loopback/multicast validation and duplicate-safe local save; live WSJT-X acceptance open.</x:v>
       </x:c>
       <x:c r="C27" s="67" t="str">
-        <x:v>Documented / locally inventoried — WSJT-X activity-window and callsign-checking choices.</x:v>
+        <x:v>Documented / locally inventoried — configurable WSJT-X UDP logging and save choices.</x:v>
       </x:c>
       <x:c r="D27" s="67" t="str">
-        <x:v>Documented — WSJT-X activity can feed its alert evaluator.</x:v>
+        <x:v>Documented — WSJT-X integration; source audit shows one configurable unicast/multicast receiver and QSO Logged/Logged ADIF parsing.</x:v>
       </x:c>
       <x:c r="E27" s="59"/>
       <x:c r="F27" s="59"/>
     </x:row>
     <x:row r="28" ht="24" hidden="0" customHeight="1">
       <x:c r="A28" s="66" t="str">
-        <x:v>DX Cluster</x:v>
+        <x:v>WSJT-X CQ activity and novelty</x:v>
       </x:c>
       <x:c r="B28" s="67" t="str">
-        <x:v>Implemented — native shared cluster owner, profiles, filters, console paths and retained spot state; configuration and display remain separated.</x:v>
+        <x:v>Source complete — bounded receive-only FT8/FT4 CQ activity feeds named alerts with current local call/DXCC novelty; no reply, CAT, PTT or save authority.</x:v>
       </x:c>
       <x:c r="C28" s="67" t="str">
-        <x:v>Documented — internet/local-skimmer cluster, terminal and separated/alerted spots.</x:v>
+        <x:v>Documented / locally inventoried — WSJT-X activity-window and callsign-checking choices.</x:v>
       </x:c>
       <x:c r="D28" s="67" t="str">
-        <x:v>Documented — DX cluster integration.</x:v>
+        <x:v>Documented — WSJT-X activity can feed its alert evaluator.</x:v>
       </x:c>
       <x:c r="E28" s="59"/>
       <x:c r="F28" s="59"/>
     </x:row>
     <x:row r="29" ht="24" hidden="0" customHeight="1">
       <x:c r="A29" s="66" t="str">
-        <x:v>Spot History</x:v>
+        <x:v>DX Cluster</x:v>
       </x:c>
       <x:c r="B29" s="67" t="str">
-        <x:v>Source complete — separate retained local reports, search/filter/statistics and read-only review. Detached column controls exist; packaged/live retention acceptance remains open.</x:v>
+        <x:v>Implemented — native shared cluster owner, profiles, filters, console paths and retained spot state; configuration and display remain separated.</x:v>
       </x:c>
       <x:c r="C29" s="67" t="str">
-        <x:v>Documented — incoming cluster data and spot/search workflows; exact retained-history model differs.</x:v>
+        <x:v>Documented — internet/local-skimmer cluster, terminal and separated/alerted spots.</x:v>
       </x:c>
       <x:c r="D29" s="67" t="str">
-        <x:v>Documented alert/history tables; exact long-term raw report retention was not established in the reviewed README.</x:v>
+        <x:v>Documented — DX cluster integration.</x:v>
       </x:c>
       <x:c r="E29" s="59"/>
       <x:c r="F29" s="59"/>
     </x:row>
-    <x:row r="30" ht="48" hidden="0" customHeight="1">
+    <x:row r="30" ht="24" hidden="0" customHeight="1">
       <x:c r="A30" s="66" t="str">
-        <x:v>Named DX/WSJT-X alert rules</x:v>
+        <x:v>Spot History</x:v>
       </x:c>
       <x:c r="B30" s="67" t="str">
-        <x:v>Source complete — independently enabled structured rules, all matching names, bounded dedup/rate limiting and passive recent-alert dashboard. Each retained event explains its call/DXCC/band/mode/special evidence and first-to-last report history; compact windows use cards instead of horizontal scrolling.</x:v>
+        <x:v>Source complete — separate retained local reports, search/filter/statistics and read-only review. Detached column controls exist; packaged/live retention acceptance remains open.</x:v>
       </x:c>
       <x:c r="C30" s="67" t="str">
-        <x:v>Documented — DXCC/band/mode/IOTA novelty, confirmation source choices, wildcard station watches and optional spoken delivery.</x:v>
+        <x:v>Documented — incoming cluster data and spot/search workflows; exact retained-history model differs.</x:v>
       </x:c>
       <x:c r="D30" s="67" t="str">
-        <x:v>Documented — named cloneable rules combining source, callsign, entity, novelty, geography, comment, band, mode, memberships and activity references.</x:v>
+        <x:v>Documented alert/history tables; exact long-term raw report retention was not established in the reviewed README.</x:v>
       </x:c>
       <x:c r="E30" s="59"/>
       <x:c r="F30" s="59"/>
     </x:row>
-    <x:row r="31" ht="24" hidden="0" customHeight="1">
+    <x:row r="31" ht="48" hidden="0" customHeight="1">
       <x:c r="A31" s="66" t="str">
-        <x:v>Alert delivery without RF authority</x:v>
+        <x:v>Named DX/WSJT-X alert rules</x:v>
       </x:c>
       <x:c r="B31" s="67" t="str">
-        <x:v>Source complete — native default-off popup plus optional sound, no action button or station authority; installed live-cluster popup/sound acceptance open.</x:v>
+        <x:v>Source complete — independently enabled structured rules, all matching names, bounded dedup/rate limiting and passive recent-alert dashboard. Each retained event explains its call/DXCC/band/mode/special evidence and first-to-last report history; compact windows use cards instead of horizontal scrolling.</x:v>
       </x:c>
       <x:c r="C31" s="67" t="str">
-        <x:v>Documented — color-only or opt-in spoken alarm delivery.</x:v>
+        <x:v>Documented — DXCC/band/mode/IOTA novelty, confirmation source choices, wildcard station watches and optional spoken delivery.</x:v>
       </x:c>
       <x:c r="D31" s="67" t="str">
-        <x:v>Documented — optional bell and outbound UDP; QLog may also tune/reply from alert UI, which OM0RX-xLog intentionally does not copy.</x:v>
+        <x:v>Documented — named cloneable rules combining source, callsign, entity, novelty, geography, comment, band, mode, memberships and activity references.</x:v>
       </x:c>
       <x:c r="E31" s="59"/>
       <x:c r="F31" s="59"/>
     </x:row>
     <x:row r="32" ht="24" hidden="0" customHeight="1">
       <x:c r="A32" s="66" t="str">
-        <x:v>World map and grayline</x:v>
+        <x:v>Alert delivery without RF authority</x:v>
       </x:c>
       <x:c r="B32" s="67" t="str">
-        <x:v>Implemented — online hybrid/satellite/standard map, spot and DXCC layers, route/grayline/sun overlays and semantic labels; prolonged operator observation remains.</x:v>
+        <x:v>Source complete — native default-off popup plus optional sound, no action button or station authority; installed live-cluster popup/sound acceptance open.</x:v>
       </x:c>
       <x:c r="C32" s="67" t="str">
-        <x:v>Documented — maps/grayline and DXCC/spot workflows.</x:v>
+        <x:v>Documented — color-only or opt-in spoken alarm delivery.</x:v>
       </x:c>
       <x:c r="D32" s="67" t="str">
-        <x:v>Documented — online and offline map.</x:v>
+        <x:v>Documented — optional bell and outbound UDP; QLog may also tune/reply from alert UI, which OM0RX-xLog intentionally does not copy.</x:v>
       </x:c>
       <x:c r="E32" s="59"/>
       <x:c r="F32" s="59"/>
     </x:row>
     <x:row r="33" ht="24" hidden="0" customHeight="1">
       <x:c r="A33" s="66" t="str">
-        <x:v>Band maps</x:v>
+        <x:v>World map and grayline</x:v>
       </x:c>
       <x:c r="B33" s="67" t="str">
-        <x:v>Implemented — multiple independently keyed band maps, follow-radio behavior and detached windows; final mixed-size/multi-display packaged acceptance remains.</x:v>
+        <x:v>Implemented — online hybrid/satellite/standard map, spot and DXCC layers, route/grayline/sun overlays and semantic labels; prolonged operator observation remains.</x:v>
       </x:c>
       <x:c r="C33" s="67" t="str">
-        <x:v>Documented / locally observed — multiple independent band-map windows.</x:v>
+        <x:v>Documented — maps/grayline and DXCC/spot workflows.</x:v>
       </x:c>
       <x:c r="D33" s="67" t="str">
-        <x:v>Documented — bandmap.</x:v>
+        <x:v>Documented — online and offline map.</x:v>
       </x:c>
       <x:c r="E33" s="59"/>
       <x:c r="F33" s="59"/>
     </x:row>
-    <x:row r="34" ht="36" hidden="0" customHeight="1">
+    <x:row r="34" ht="24" hidden="0" customHeight="1">
       <x:c r="A34" s="66" t="str">
-        <x:v>Canvas and separate-window modes</x:v>
+        <x:v>Band maps</x:v>
       </x:c>
       <x:c r="B34" s="67" t="str">
-        <x:v>Source complete — persistent Canvas/Separate Windows choice, named native task windows and geometry recovery. Switching to Canvas closes child windows; simultaneous multi-display packaged acceptance remains.</x:v>
+        <x:v>Implemented — multiple independently keyed band maps, follow-radio behavior and detached windows; final mixed-size/multi-display packaged acceptance remains.</x:v>
       </x:c>
       <x:c r="C34" s="67" t="str">
-        <x:v>Documented / locally observed — many named native windows with saved placement conventions.</x:v>
+        <x:v>Documented / locally observed — multiple independent band-map windows.</x:v>
       </x:c>
       <x:c r="D34" s="67" t="str">
-        <x:v>Documented — customizable GUI and saved layout profiles; macOS is experimental.</x:v>
+        <x:v>Documented — bandmap.</x:v>
       </x:c>
       <x:c r="E34" s="59"/>
       <x:c r="F34" s="59"/>
     </x:row>
-    <x:row r="35" ht="60" hidden="0" customHeight="1">
+    <x:row r="35" ht="36" hidden="0" customHeight="1">
       <x:c r="A35" s="66" t="str">
-        <x:v>Responsive detached windows</x:v>
+        <x:v>Canvas and separate-window modes</x:v>
       </x:c>
       <x:c r="B35" s="67" t="str">
-        <x:v>Partial — common chrome removal and targeted fixes cover many roles. Detached Propagation rows align; Station Status and Rotor use the shared inset; Rotor starts at the top. Focused 31/31 UI, rendered geometry, Band Map 380×1100, Callsign Intelligence 680×500 and Rotor 676×500/400×600 browser checks pass without page overflow. The packaged all-window resolution/scale matrix remains outstanding.</x:v>
+        <x:v>Source complete — persistent Canvas/Separate Windows choice, named native task windows and geometry recovery. Switching to Canvas closes child windows; simultaneous multi-display packaged acceptance remains.</x:v>
       </x:c>
       <x:c r="C35" s="67" t="str">
-        <x:v>Mature native macOS window behavior is the reference; exact responsive tests were not obtained.</x:v>
+        <x:v>Documented / locally observed — many named native windows with saved placement conventions.</x:v>
       </x:c>
       <x:c r="D35" s="67" t="str">
-        <x:v>Recommended resolution is 1920×1080; cross-platform GUI is customizable, but compact-window behavior was not established.</x:v>
+        <x:v>Documented — customizable GUI and saved layout profiles; macOS is experimental.</x:v>
       </x:c>
       <x:c r="E35" s="59"/>
       <x:c r="F35" s="59"/>
     </x:row>
-    <x:row r="36" ht="24" hidden="0" customHeight="1">
+    <x:row r="36" ht="60" hidden="0" customHeight="1">
       <x:c r="A36" s="66" t="str">
-        <x:v>Custom canvas panel move/resize</x:v>
+        <x:v>Responsive detached windows</x:v>
       </x:c>
       <x:c r="B36" s="67" t="str">
-        <x:v>Source complete for traditional unlock/edit interaction — panel arrow enters edit mode, title drags position and edges/corners resize; broader mixed-size acceptance remains.</x:v>
+        <x:v>Partial — common chrome removal and targeted fixes cover many roles. Detached Propagation rows align; Station Status and Rotor use the shared inset; Rotor starts at the top. Focused 31/31 UI, rendered geometry, Band Map 380×1100, Callsign Intelligence 680×500 and Rotor 676×500/400×600 browser checks pass without page overflow. The packaged all-window resolution/scale matrix remains outstanding.</x:v>
       </x:c>
       <x:c r="C36" s="67" t="str">
-        <x:v>Not a directly comparable canvas workflow in reviewed evidence.</x:v>
+        <x:v>Mature native macOS window behavior is the reference; exact responsive tests were not obtained.</x:v>
       </x:c>
       <x:c r="D36" s="67" t="str">
-        <x:v>Documented saved layout profiles; exact freeform canvas resize interaction differs.</x:v>
+        <x:v>Recommended resolution is 1920×1080; cross-platform GUI is customizable, but compact-window behavior was not established.</x:v>
       </x:c>
       <x:c r="E36" s="59"/>
       <x:c r="F36" s="59"/>
     </x:row>
     <x:row r="37" ht="24" hidden="0" customHeight="1">
       <x:c r="A37" s="66" t="str">
-        <x:v>Radio control providers</x:v>
+        <x:v>Custom canvas panel move/resize</x:v>
       </x:c>
       <x:c r="B37" s="67" t="str">
-        <x:v>Implemented — Remote Agent, direct FLEX LAN and local Hamlib paths are capability-separated with explicit selection/connect and retained observed state.</x:v>
+        <x:v>Source complete for traditional unlock/edit interaction — panel arrow enters edit mode, title drags position and edges/corners resize; broader mixed-size acceptance remains.</x:v>
       </x:c>
       <x:c r="C37" s="67" t="str">
-        <x:v>Documented — Kenwood, Elecraft, Yaesu and Icom support, with deeper controls for selected models.</x:v>
+        <x:v>Not a directly comparable canvas workflow in reviewed evidence.</x:v>
       </x:c>
       <x:c r="D37" s="67" t="str">
-        <x:v>Documented — Hamlib, OmniRig, TCI and FLRig.</x:v>
+        <x:v>Documented saved layout profiles; exact freeform canvas resize interaction differs.</x:v>
       </x:c>
       <x:c r="E37" s="59"/>
       <x:c r="F37" s="59"/>
     </x:row>
-    <x:row r="38" ht="96" hidden="0" customHeight="1">
+    <x:row r="38" ht="24" hidden="0" customHeight="1">
       <x:c r="A38" s="66" t="str">
-        <x:v>TCI rig control — SunSDR/ExpertSDR and compatible servers</x:v>
+        <x:v>Radio control providers</x:v>
       </x:c>
       <x:c r="B38" s="67" t="str">
-        <x:v>Source complete through observed receive-frequency/mode tuning, TRX-wide receive-filter adjustment, configured-TRX split observation and server-global TX-frequency telemetry — bounded protocol/session, exact discovery, producer-time freshness, saved credential-free ws/wss setup and stale-aware UI. Explicit controls use the existing connection, durable no-replay receipts and newer exact readback. The filter has an app-local ±24 kHz bound and no longer misuses IF_LIMITS. Global TX frequency has no TRX/channel/VFO identity and is never promoted to configured evidence or authority. Transmit/PTT, split/TX-VFO controls, spots, audio/IQ and package/live-server acceptance remain open.</x:v>
+        <x:v>Implemented — Remote Agent, direct FLEX LAN and local Hamlib paths are capability-separated with explicit selection/connect and retained observed state.</x:v>
       </x:c>
       <x:c r="C38" s="67" t="str">
-        <x:v>Not established in the reviewed primary RUMlogNG evidence.</x:v>
+        <x:v>Documented — Kenwood, Elecraft, Yaesu and Icom support, with deeper controls for selected models.</x:v>
       </x:c>
       <x:c r="D38" s="67" t="str">
-        <x:v>Documented — QLog supports all TCI-compatible rigs through its native TCI provider.</x:v>
+        <x:v>Documented — Hamlib, OmniRig, TCI and FLRig.</x:v>
       </x:c>
       <x:c r="E38" s="59"/>
       <x:c r="F38" s="59"/>
     </x:row>
-    <x:row r="39" ht="24" hidden="0" customHeight="1">
+    <x:row r="39" ht="96" hidden="0" customHeight="1">
       <x:c r="A39" s="66" t="str">
-        <x:v>Safe simplex tuning and Tune/Cancel</x:v>
+        <x:v>TCI rig control — SunSDR/ExpertSDR and compatible servers</x:v>
       </x:c>
       <x:c r="B39" s="67" t="str">
-        <x:v>Source complete — durable exact-owner transactions, one existing-worker dispatch, no replay and authoritative readback where available; packaged/hardware acceptance open.</x:v>
+        <x:v>Source complete through observed receive-frequency/mode tuning, TRX-wide receive-filter adjustment, configured-TRX split observation, server-global TX-frequency telemetry and passive server spot-click events — bounded protocol/session, exact discovery, producer-time freshness, saved credential-free ws/wss setup and stale-aware UI. Explicit controls use the existing connection, durable no-replay receipts and newer exact readback. Global TX frequency and spot clicks remain separate telemetry and never become configured evidence, inventory or authority. Transmit/PTT, split/TX-VFO controls, outbound spot management, audio/IQ and package/live-server acceptance remain open.</x:v>
       </x:c>
       <x:c r="C39" s="67" t="str">
-        <x:v>Documented — CAT can set transceiver parameters from the logbook and vice versa; safety contract was not audited.</x:v>
+        <x:v>Not established in the reviewed primary RUMlogNG evidence.</x:v>
       </x:c>
       <x:c r="D39" s="67" t="str">
-        <x:v>Documented — rig control and cluster/bandmap integration; safety contract was not audited.</x:v>
+        <x:v>Documented — QLog supports all TCI-compatible rigs through its native TCI provider.</x:v>
       </x:c>
       <x:c r="E39" s="59"/>
       <x:c r="F39" s="59"/>
     </x:row>
-    <x:row r="40" ht="48" hidden="0" customHeight="1">
+    <x:row r="40" ht="24" hidden="0" customHeight="1">
       <x:c r="A40" s="66" t="str">
-        <x:v>Amplifier Operate/Standby</x:v>
+        <x:v>Safe simplex tuning and Tune/Cancel</x:v>
       </x:c>
       <x:c r="B40" s="67" t="str">
-        <x:v>Source complete — one shared Agent-only durable owner provides separate Operate and urgent Standby lanes, exact identity/freshness fences, one-attempt journal-before-send dispatch and explicit unknown-receipt recovery. Packaged Agent, amplifier-readback, hardware and RF acceptance remain.</x:v>
+        <x:v>Source complete — durable exact-owner transactions, one existing-worker dispatch, no replay and authoritative readback where available; packaged/hardware acceptance open.</x:v>
       </x:c>
       <x:c r="C40" s="67" t="str">
-        <x:v>Model/device controls exist for supported station equipment; exact KPA-style workflow was not established.</x:v>
+        <x:v>Documented — CAT can set transceiver parameters from the logbook and vice versa; safety contract was not audited.</x:v>
       </x:c>
       <x:c r="D40" s="67" t="str">
-        <x:v>No comparable amplifier owner was established in reviewed evidence.</x:v>
+        <x:v>Documented — rig control and cluster/bandmap integration; safety contract was not audited.</x:v>
       </x:c>
       <x:c r="E40" s="59"/>
       <x:c r="F40" s="59"/>
     </x:row>
-    <x:row r="41" ht="24" hidden="0" customHeight="1">
+    <x:row r="41" ht="48" hidden="0" customHeight="1">
       <x:c r="A41" s="66" t="str">
-        <x:v>Rotor control</x:v>
+        <x:v>Amplifier Operate/Standby</x:v>
       </x:c>
       <x:c r="B41" s="67" t="str">
-        <x:v>Source complete — shared manual Goto, native urgent Stop and standalone Auto/Stop with exact owner/generation fences; packaged/hardware acceptance open.</x:v>
+        <x:v>Source complete — one shared Agent-only durable owner provides separate Operate and urgent Standby lanes, exact identity/freshness fences, one-attempt journal-before-send dispatch and explicit unknown-receipt recovery. Packaged Agent, amplifier-readback, hardware and RF acceptance remain.</x:v>
       </x:c>
       <x:c r="C41" s="67" t="str">
-        <x:v>Documented through a companion advanced Rotor application interacting with RUMlogNG and WSJT-X.</x:v>
+        <x:v>Model/device controls exist for supported station equipment; exact KPA-style workflow was not established.</x:v>
       </x:c>
       <x:c r="D41" s="67" t="str">
-        <x:v>Documented — Hamlib and PSTRotator control.</x:v>
+        <x:v>No comparable amplifier owner was established in reviewed evidence.</x:v>
       </x:c>
       <x:c r="E41" s="59"/>
       <x:c r="F41" s="59"/>
     </x:row>
     <x:row r="42" ht="24" hidden="0" customHeight="1">
       <x:c r="A42" s="66" t="str">
-        <x:v>CW keyer and console</x:v>
+        <x:v>Rotor control</x:v>
       </x:c>
       <x:c r="B42" s="67" t="str">
-        <x:v>Implemented foundation — shared saved macros/new-QSO context plus explicit selected-radio and independent WinKeyer ownership; remaining end-to-end hardware acceptance is open.</x:v>
+        <x:v>Source complete — shared manual Goto, native urgent Stop and standalone Auto/Stop with exact owner/generation fences; packaged/hardware acceptance open.</x:v>
       </x:c>
       <x:c r="C42" s="67" t="str">
-        <x:v>Documented — K1EL WinKeyer, CW keyer and RTTY application.</x:v>
+        <x:v>Documented through a companion advanced Rotor application interacting with RUMlogNG and WSJT-X.</x:v>
       </x:c>
       <x:c r="D42" s="67" t="str">
-        <x:v>Documented — CWDaemon, FLDigi, Morse over CAT, WinKey v1/v2 and CW Console.</x:v>
+        <x:v>Documented — Hamlib and PSTRotator control.</x:v>
       </x:c>
       <x:c r="E42" s="59"/>
       <x:c r="F42" s="59"/>
     </x:row>
     <x:row r="43" ht="24" hidden="0" customHeight="1">
       <x:c r="A43" s="66" t="str">
-        <x:v>Propagation display</x:v>
+        <x:v>CW keyer and console</x:v>
       </x:c>
       <x:c r="B43" s="67" t="str">
-        <x:v>Source complete with live provider proof — bounded HamQSL/N0NBH refresh and correct freshness semantics; final packaged outage/freshness observation remains.</x:v>
+        <x:v>Implemented foundation — shared saved macros/new-QSO context plus explicit selected-radio and independent WinKeyer ownership; remaining end-to-end hardware acceptance is open.</x:v>
       </x:c>
       <x:c r="C43" s="67" t="str">
-        <x:v>Not highlighted in reviewed primary feature listing.</x:v>
+        <x:v>Documented — K1EL WinKeyer, CW keyer and RTTY application.</x:v>
       </x:c>
       <x:c r="D43" s="67" t="str">
-        <x:v>Not highlighted in reviewed primary feature listing.</x:v>
+        <x:v>Documented — CWDaemon, FLDigi, Morse over CAT, WinKey v1/v2 and CW Console.</x:v>
       </x:c>
       <x:c r="E43" s="59"/>
       <x:c r="F43" s="59"/>
     </x:row>
     <x:row r="44" ht="24" hidden="0" customHeight="1">
       <x:c r="A44" s="66" t="str">
-        <x:v>Awards and statistics</x:v>
+        <x:v>Propagation display</x:v>
       </x:c>
       <x:c r="B44" s="67" t="str">
-        <x:v>Implemented foundation — nine native calculators plus a 192-programme research library; many programmes are tracking/blocked rather than falsely credited.</x:v>
+        <x:v>Source complete with live provider proof — bounded HamQSL/N0NBH refresh and correct freshness semantics; final packaged outage/freshness observation remains.</x:v>
       </x:c>
       <x:c r="C44" s="67" t="str">
-        <x:v>Documented — DXCC plus IOTA, CQ/ITU zones, grids, states, counties, DOKs and detailed QSL statistics.</x:v>
+        <x:v>Not highlighted in reviewed primary feature listing.</x:v>
       </x:c>
       <x:c r="D44" s="67" t="str">
-        <x:v>Documented — basic awards and station statistics.</x:v>
+        <x:v>Not highlighted in reviewed primary feature listing.</x:v>
       </x:c>
       <x:c r="E44" s="59"/>
       <x:c r="F44" s="59"/>
     </x:row>
     <x:row r="45" ht="24" hidden="0" customHeight="1">
       <x:c r="A45" s="66" t="str">
-        <x:v>Contest logging</x:v>
+        <x:v>Awards and statistics</x:v>
       </x:c>
       <x:c r="B45" s="67" t="str">
-        <x:v>Outstanding as a separate programme — ordinary logging remains primary; do not add empty parity UI.</x:v>
+        <x:v>Implemented foundation — nine native calculators plus a 192-programme research library; many programmes are tracking/blocked rather than falsely credited.</x:v>
       </x:c>
       <x:c r="C45" s="67" t="str">
-        <x:v>Documented — specialized contest/DXpedition logger with scoring and ESM.</x:v>
+        <x:v>Documented — DXCC plus IOTA, CQ/ITU zones, grids, states, counties, DOKs and detailed QSL statistics.</x:v>
       </x:c>
       <x:c r="D45" s="67" t="str">
-        <x:v>Documented — basic contest support; QLog states contests are not its current focus.</x:v>
+        <x:v>Documented — basic awards and station statistics.</x:v>
       </x:c>
       <x:c r="E45" s="59"/>
       <x:c r="F45" s="59"/>
     </x:row>
     <x:row r="46" ht="24" hidden="0" customHeight="1">
       <x:c r="A46" s="66" t="str">
-        <x:v>Paper QSL and label printing</x:v>
+        <x:v>Contest logging</x:v>
       </x:c>
       <x:c r="B46" s="67" t="str">
-        <x:v>Outstanding as a dedicated workflow; ADIF QSL fields are preserved and remote confirmations can refresh.</x:v>
+        <x:v>Outstanding as a separate programme — ordinary logging remains primary; do not add empty parity UI.</x:v>
       </x:c>
       <x:c r="C46" s="67" t="str">
-        <x:v>Documented — incoming paper QSL management and QSL label printing.</x:v>
+        <x:v>Documented — specialized contest/DXpedition logger with scoring and ESM.</x:v>
       </x:c>
       <x:c r="D46" s="67" t="str">
-        <x:v>No paper-label workflow established in the reviewed README.</x:v>
+        <x:v>Documented — basic contest support; QLog states contests are not its current focus.</x:v>
       </x:c>
       <x:c r="E46" s="59"/>
       <x:c r="F46" s="59"/>
     </x:row>
     <x:row r="47" ht="24" hidden="0" customHeight="1">
       <x:c r="A47" s="66" t="str">
-        <x:v>Station/location profiles</x:v>
+        <x:v>Paper QSL and label printing</x:v>
       </x:c>
       <x:c r="B47" s="67" t="str">
-        <x:v>Partial — saved station identity/equipment/workspace configuration exists with separate radio, rotor, antenna and activity ownership; profile UX can be improved without unsafe implicit apply.</x:v>
+        <x:v>Outstanding as a dedicated workflow; ADIF QSL fields are preserved and remote confirmations can refresh.</x:v>
       </x:c>
       <x:c r="C47" s="67" t="str">
-        <x:v>Documented / locally observed — operator identity, radios, QRGs, modes/satellites, cluster, QSL and service groups.</x:v>
+        <x:v>Documented — incoming paper QSL management and QSL label printing.</x:v>
       </x:c>
       <x:c r="D47" s="67" t="str">
-        <x:v>Documented — station location profile support.</x:v>
+        <x:v>No paper-label workflow established in the reviewed README.</x:v>
       </x:c>
       <x:c r="E47" s="59"/>
       <x:c r="F47" s="59"/>
     </x:row>
     <x:row r="48" ht="24" hidden="0" customHeight="1">
       <x:c r="A48" s="66" t="str">
-        <x:v>Secure credential storage</x:v>
+        <x:v>Station/location profiles</x:v>
       </x:c>
       <x:c r="B48" s="67" t="str">
-        <x:v>Implemented — Keychain/vault-backed provider credentials with ownership and revision fencing.</x:v>
+        <x:v>Partial — saved station identity/equipment/workspace configuration exists with separate radio, rotor, antenna and activity ownership; profile UX can be improved without unsafe implicit apply.</x:v>
       </x:c>
       <x:c r="C48" s="67" t="str">
-        <x:v>Uses macOS platform storage for supported services; exact architecture was not audited.</x:v>
+        <x:v>Documented / locally observed — operator identity, radios, QRGs, modes/satellites, cluster, QSL and service groups.</x:v>
       </x:c>
       <x:c r="D48" s="67" t="str">
-        <x:v>Documented — system keyring/credential store support on Linux, Windows and macOS.</x:v>
+        <x:v>Documented — station location profile support.</x:v>
       </x:c>
       <x:c r="E48" s="59"/>
       <x:c r="F48" s="59"/>
     </x:row>
     <x:row r="49" ht="24" hidden="0" customHeight="1">
       <x:c r="A49" s="66" t="str">
-        <x:v>Backups</x:v>
+        <x:v>Secure credential storage</x:v>
       </x:c>
       <x:c r="B49" s="67" t="str">
-        <x:v>Partial — local backup/restore safety exists; optional remote FTP/FTPS/SFTP work is active in a separate user-owned change set and is not counted complete here.</x:v>
+        <x:v>Implemented — Keychain/vault-backed provider credentials with ownership and revision fencing.</x:v>
       </x:c>
       <x:c r="C49" s="67" t="str">
-        <x:v>Not established in reviewed primary feature listing.</x:v>
+        <x:v>Uses macOS platform storage for supported services; exact architecture was not audited.</x:v>
       </x:c>
       <x:c r="D49" s="67" t="str">
-        <x:v>Not established in reviewed primary feature listing.</x:v>
+        <x:v>Documented — system keyring/credential store support on Linux, Windows and macOS.</x:v>
       </x:c>
       <x:c r="E49" s="59"/>
       <x:c r="F49" s="59"/>
     </x:row>
     <x:row r="50" ht="24" hidden="0" customHeight="1">
       <x:c r="A50" s="66" t="str">
-        <x:v>Cross-platform delivery</x:v>
+        <x:v>Backups</x:v>
       </x:c>
       <x:c r="B50" s="67" t="str">
-        <x:v>Partial — one shared UI/domain targets macOS, Windows and Linux; Mac is the current acceptance focus and Windows/Linux packaging is intentionally deferred.</x:v>
+        <x:v>Partial — local backup/restore safety exists; optional remote FTP/FTPS/SFTP work is active in a separate user-owned change set and is not counted complete here.</x:v>
       </x:c>
       <x:c r="C50" s="67" t="str">
-        <x:v>Mac only.</x:v>
+        <x:v>Not established in reviewed primary feature listing.</x:v>
       </x:c>
       <x:c r="D50" s="67" t="str">
-        <x:v>Linux and Windows supported; macOS is documented as experimental/developer-only.</x:v>
+        <x:v>Not established in reviewed primary feature listing.</x:v>
       </x:c>
       <x:c r="E50" s="59"/>
       <x:c r="F50" s="59"/>
     </x:row>
     <x:row r="51" ht="24" hidden="0" customHeight="1">
       <x:c r="A51" s="66" t="str">
-        <x:v>Privacy and telemetry</x:v>
+        <x:v>Cross-platform delivery</x:v>
       </x:c>
       <x:c r="B51" s="67" t="str">
-        <x:v>Implemented by design — local-first operation, explicit external-service enrollment and no hidden station/network actions in source acceptance tests.</x:v>
+        <x:v>Partial — one shared UI/domain targets macOS, Windows and Linux; Mac is the current acceptance focus and Windows/Linux packaging is intentionally deferred.</x:v>
       </x:c>
       <x:c r="C51" s="67" t="str">
-        <x:v>Current App Store disclosure says data is not collected.</x:v>
+        <x:v>Mac only.</x:v>
       </x:c>
       <x:c r="D51" s="67" t="str">
-        <x:v>Documented — no ads, user tracking or hidden telemetry.</x:v>
+        <x:v>Linux and Windows supported; macOS is documented as experimental/developer-only.</x:v>
       </x:c>
       <x:c r="E51" s="59"/>
       <x:c r="F51" s="59"/>
     </x:row>
-    <x:row r="52" ht="15" hidden="0" customHeight="1">
-      <x:c r="A52" s="59"/>
-      <x:c r="B52" s="59"/>
-      <x:c r="C52" s="59"/>
-      <x:c r="D52" s="59"/>
+    <x:row r="52" ht="24" hidden="0" customHeight="1">
+      <x:c r="A52" s="66" t="str">
+        <x:v>Privacy and telemetry</x:v>
+      </x:c>
+      <x:c r="B52" s="67" t="str">
+        <x:v>Implemented by design — local-first operation, explicit external-service enrollment and no hidden station/network actions in source acceptance tests.</x:v>
+      </x:c>
+      <x:c r="C52" s="67" t="str">
+        <x:v>Current App Store disclosure says data is not collected.</x:v>
+      </x:c>
+      <x:c r="D52" s="67" t="str">
+        <x:v>Documented — no ads, user tracking or hidden telemetry.</x:v>
+      </x:c>
       <x:c r="E52" s="59"/>
       <x:c r="F52" s="59"/>
     </x:row>
@@ -2720,7 +2728,7 @@
   <x:mergeCells>
     <x:mergeCell ref="A3:D3"/>
   </x:mergeCells>
-  <x:conditionalFormatting sqref="B7:B51">
+  <x:conditionalFormatting sqref="B7:B52">
     <x:cfRule type="beginsWith" dxfId="0" priority="1" operator="beginsWith" text="Installed"/>
     <x:cfRule type="beginsWith" dxfId="1" priority="2" operator="beginsWith" text="Implemented"/>
     <x:cfRule type="beginsWith" dxfId="2" priority="3" operator="beginsWith" text="Source complete"/>
@@ -2730,7 +2738,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd07c3420df4c49c4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc1394a2ba5414e01"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2922,7 +2930,7 @@
         <x:v>ADIF 3.1.8 conformance</x:v>
       </x:c>
       <x:c r="C12" s="67" t="str">
-        <x:v>Four compatibility fixes complete</x:v>
+        <x:v>Five compatibility fixes complete</x:v>
       </x:c>
       <x:c r="D12" s="67" t="str">
         <x:v>Complete the remaining enum/deprecation and MODE/SUBMODE audit before changing ADIF_VER; run copied-log/package and service-specific interoperability acceptance.</x:v>
@@ -2962,10 +2970,10 @@
         <x:v>Full TCI radio provider</x:v>
       </x:c>
       <x:c r="C14" s="67" t="str">
-        <x:v>Receive tune/filter, passive split and global TX-frequency observation source complete</x:v>
+        <x:v>Receive tune/filter plus passive split, TX-frequency and spot-click observation source complete</x:v>
       </x:c>
       <x:c r="D14" s="67" t="str">
-        <x:v>Extend the existing no-replay owner with separately reviewed split/TX-VFO controls, urgent release and optional audio/IQ slices; do not assign global TX frequency to a TRX/VFO. The pinned protocol has no received spot inventory, and transmit/PTT keeps its own explicit authority.</x:v>
+        <x:v>Extend the existing no-replay owner with separately reviewed split/TX-VFO controls, urgent release and optional audio/IQ slices; do not assign global TX frequency or spot-click events to configured evidence/inventory. Transmit/PTT keeps its own explicit authority.</x:v>
       </x:c>
       <x:c r="E14" s="67" t="str">
         <x:v>Simulated-server races, package tests, then operator-controlled SunSDR acceptance</x:v>
@@ -3134,44 +3142,44 @@
         <x:v>RUMlogNG alarms/award status; QLog alerts/filters</x:v>
       </x:c>
     </x:row>
-    <x:row r="23" ht="24" hidden="0" customHeight="1">
+    <x:row r="23" ht="36" hidden="0" customHeight="1">
       <x:c r="A23" s="66" t="str">
         <x:v>P1</x:v>
       </x:c>
       <x:c r="B23" s="67" t="str">
-        <x:v>Contest logging</x:v>
+        <x:v>Online-log follow-up UI</x:v>
       </x:c>
       <x:c r="C23" s="67" t="str">
-        <x:v>Programme decision</x:v>
+        <x:v>Core projection source complete</x:v>
       </x:c>
       <x:c r="D23" s="67" t="str">
-        <x:v>Decide whether to build a separate contest engine with scoring, exchange, ESM and Cabrillo/REG1TEST export.</x:v>
+        <x:v>Add a bounded worker/native surface only after the provider acceptance/match timestamp contract is explicit; never infer confirmation or sponsor credit from upload delivery.</x:v>
       </x:c>
       <x:c r="E23" s="67" t="str">
-        <x:v>Rules, performance and contest-specific acceptance plan</x:v>
+        <x:v>Focused route/UI tests, exact package and live-account evidence</x:v>
       </x:c>
       <x:c r="F23" s="67" t="str">
-        <x:v>RUMlogNG mature contest workflow; QLog basic contests</x:v>
+        <x:v>RUMlogNG/QLog online-log status workflows</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="24" hidden="0" customHeight="1">
       <x:c r="A24" s="66" t="str">
-        <x:v>P2</x:v>
+        <x:v>P1</x:v>
       </x:c>
       <x:c r="B24" s="67" t="str">
-        <x:v>Paper QSL and labels</x:v>
+        <x:v>Contest logging</x:v>
       </x:c>
       <x:c r="C24" s="67" t="str">
         <x:v>Programme decision</x:v>
       </x:c>
       <x:c r="D24" s="67" t="str">
-        <x:v>Decide whether paper-QSL tracking and label printing belongs in the product or remains an external workflow.</x:v>
+        <x:v>Decide whether to build a separate contest engine with scoring, exchange, ESM and Cabrillo/REG1TEST export.</x:v>
       </x:c>
       <x:c r="E24" s="67" t="str">
-        <x:v>Printer/template requirements and operator demand</x:v>
+        <x:v>Rules, performance and contest-specific acceptance plan</x:v>
       </x:c>
       <x:c r="F24" s="67" t="str">
-        <x:v>RUMlogNG</x:v>
+        <x:v>RUMlogNG mature contest workflow; QLog basic contests</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="24" hidden="0" customHeight="1">
@@ -3179,19 +3187,19 @@
         <x:v>P2</x:v>
       </x:c>
       <x:c r="B25" s="67" t="str">
-        <x:v>Regional band/allocation guides</x:v>
+        <x:v>Paper QSL and labels</x:v>
       </x:c>
       <x:c r="C25" s="67" t="str">
-        <x:v>Candidate</x:v>
+        <x:v>Programme decision</x:v>
       </x:c>
       <x:c r="D25" s="67" t="str">
-        <x:v>Add only from authoritative regional data with operator-selected region and update provenance.</x:v>
+        <x:v>Decide whether paper-QSL tracking and label printing belongs in the product or remains an external workflow.</x:v>
       </x:c>
       <x:c r="E25" s="67" t="str">
-        <x:v>Authoritative data source and boundary tests</x:v>
+        <x:v>Printer/template requirements and operator demand</x:v>
       </x:c>
       <x:c r="F25" s="67" t="str">
-        <x:v>QLog band guides; RUMlogNG editable QRG segments</x:v>
+        <x:v>RUMlogNG</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="24" hidden="0" customHeight="1">
@@ -3199,28 +3207,40 @@
         <x:v>P2</x:v>
       </x:c>
       <x:c r="B26" s="67" t="str">
+        <x:v>Regional band/allocation guides</x:v>
+      </x:c>
+      <x:c r="C26" s="67" t="str">
+        <x:v>Candidate</x:v>
+      </x:c>
+      <x:c r="D26" s="67" t="str">
+        <x:v>Add only from authoritative regional data with operator-selected region and update provenance.</x:v>
+      </x:c>
+      <x:c r="E26" s="67" t="str">
+        <x:v>Authoritative data source and boundary tests</x:v>
+      </x:c>
+      <x:c r="F26" s="67" t="str">
+        <x:v>QLog band guides; RUMlogNG editable QRG segments</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="24" hidden="0" customHeight="1">
+      <x:c r="A27" s="66" t="str">
+        <x:v>P2</x:v>
+      </x:c>
+      <x:c r="B27" s="67" t="str">
         <x:v>Windows and Linux packages</x:v>
       </x:c>
-      <x:c r="C26" s="67" t="str">
+      <x:c r="C27" s="67" t="str">
         <x:v>Deferred</x:v>
       </x:c>
-      <x:c r="D26" s="67" t="str">
+      <x:c r="D27" s="67" t="str">
         <x:v>Build only after Mac visual and workflow acceptance, then validate platform-specific keyrings, radios and window behavior.</x:v>
       </x:c>
-      <x:c r="E26" s="67" t="str">
+      <x:c r="E27" s="67" t="str">
         <x:v>Native Windows/Linux packages and hardware tests</x:v>
       </x:c>
-      <x:c r="F26" s="67" t="str">
+      <x:c r="F27" s="67" t="str">
         <x:v>QLog cross-platform distribution</x:v>
       </x:c>
-    </x:row>
-    <x:row r="27" ht="15" hidden="0" customHeight="1">
-      <x:c r="A27" s="59"/>
-      <x:c r="B27" s="59"/>
-      <x:c r="C27" s="59"/>
-      <x:c r="D27" s="59"/>
-      <x:c r="E27" s="59"/>
-      <x:c r="F27" s="59"/>
     </x:row>
     <x:row r="28" ht="15" hidden="0" customHeight="1">
       <x:c r="A28" s="59"/>
@@ -4610,7 +4630,7 @@
   <x:mergeCells>
     <x:mergeCell ref="A3:F3"/>
   </x:mergeCells>
-  <x:conditionalFormatting sqref="A7:A26">
+  <x:conditionalFormatting sqref="A7:A27">
     <x:cfRule type="cellIs" dxfId="6" priority="1" operator="equal">
       <x:formula>"P0"</x:formula>
     </x:cfRule>
@@ -4620,7 +4640,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra4950aa38de4490e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rca28128b13914bb3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4763,7 +4783,7 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="C10" s="67" t="str">
-        <x:v>Four compatibility fixes complete</x:v>
+        <x:v>Five compatibility fixes complete</x:v>
       </x:c>
       <x:c r="D10" s="67" t="str">
         <x:v>ADIF parser/writer and frontend transfer</x:v>
@@ -4809,7 +4829,7 @@
       </x:c>
       <x:c r="F12" s="59"/>
     </x:row>
-    <x:row r="13" ht="15" hidden="0" customHeight="1">
+    <x:row r="13" ht="24" hidden="0" customHeight="1">
       <x:c r="A13" s="66" t="str">
         <x:v>R07</x:v>
       </x:c>
@@ -4817,13 +4837,13 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="C13" s="67" t="str">
-        <x:v>Useful extension</x:v>
+        <x:v>Core evidence projection complete; route/UI open</x:v>
       </x:c>
       <x:c r="D13" s="67" t="str">
         <x:v>Sync/delivery/confirmation and award state</x:v>
       </x:c>
       <x:c r="E13" s="67" t="str">
-        <x:v>Provider follow-up queue; keep upload, confirmation and credit distinct.</x:v>
+        <x:v>Expose the bounded projection after provider timestamp and sponsor-rule contracts; keep upload, confirmation and credit distinct.</x:v>
       </x:c>
       <x:c r="F13" s="59"/>
     </x:row>
@@ -6507,7 +6527,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2c1c7876e6a34170"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9919fb6ed1614c66"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6587,7 +6607,7 @@
         <x:v>OM0RX-xLog</x:v>
       </x:c>
       <x:c r="B7" s="65" t="str">
-        <x:v>Current implementation checkpoint b6bf7c1b36e2a8175b468719d4cf4c390316b2ec</x:v>
+        <x:v>Current implementation checkpoint 259b05d37d5d133ff9c3c9a7a659e851d81507e8</x:v>
       </x:c>
       <x:c r="C7" s="65" t="str">
         <x:v>2026-10-16</x:v>
@@ -6603,13 +6623,13 @@
         <x:v>OM0RX-xLog</x:v>
       </x:c>
       <x:c r="B8" s="67" t="str">
-        <x:v>https://github.com/oliverbross/OM0RX-xLog/commit/b6bf7c1b36e2a8175b468719d4cf4c390316b2ec</x:v>
+        <x:v>https://github.com/oliverbross/OM0RX-xLog/commit/259b05d37d5d133ff9c3c9a7a659e851d81507e8</x:v>
       </x:c>
       <x:c r="C8" s="67" t="str">
         <x:v>2026-10-16</x:v>
       </x:c>
       <x:c r="D8" s="67" t="str">
-        <x:v>Exact committed implementation baseline including observed TCI receive tune/filter, split and global TX-frequency telemetry, native Operating Goals, Connection Doctor with redacted export, cloneable saved filters, responsive window improvements, PJ/DXCC preview, four bounded ADIF compatibility fixes, and the independent Previous QSOs window.</x:v>
+        <x:v>Exact committed implementation baseline including passive TCI spot-click telemetry, QRZ/Club Log follow-up evidence, PSK31 deprecation compatibility, the OM0RX-xLog document title, earlier TCI receive tune/filter/split/global-TX stages, Operating Goals, Connection Doctor, saved filters, responsive windows, PJ/DXCC preview and Previous QSOs.</x:v>
       </x:c>
       <x:c r="E8" s="59"/>
       <x:c r="F8" s="59"/>
@@ -8236,7 +8256,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0c492a533f194b84"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9a148ad66f1b49f4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Track ADIF TCI log follow-up and award stages
</commit_message>
<xml_diff>
--- a/outputs/feature-matrix-2026-10-16/OM0RX-xLog_Feature_Comparison_2026-10-16.xlsx
+++ b/outputs/feature-matrix-2026-10-16/OM0RX-xLog_Feature_Comparison_2026-10-16.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Matrix" sheetId="1" r:id="R392661c588cb4fc7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Outstanding" sheetId="2" r:id="Rceb75a0f3e32431e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enhancement Review" sheetId="3" r:id="R236656e92ce84aff"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="4" r:id="R86507dcab7304199"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Matrix" sheetId="1" r:id="Re0b4912c92084d5a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Outstanding" sheetId="2" r:id="R0c8d239aa2034edd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enhancement Review" sheetId="3" r:id="R2f2679c3e7aa4ebc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="4" r:id="R61cd216046194268"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -852,12 +852,12 @@
       <x:c r="E9" s="59"/>
       <x:c r="F9" s="59"/>
     </x:row>
-    <x:row r="10" ht="60" hidden="0" customHeight="1">
+    <x:row r="10" ht="84" hidden="0" customHeight="1">
       <x:c r="A10" s="66" t="str">
         <x:v>ADIF field preservation</x:v>
       </x:c>
       <x:c r="B10" s="67" t="str">
-        <x:v>Source complete for five reviewed compatibility stages — local records retain a JSON field bag; unknown/custom fields, Unicode, station/contact and RX/TX data survive supported ADI/ADX round trips. UTF-8 byte scanning, FT4/FT2/JTTY MFSK-submode export, C4FM/DSTAR DIGITALVOICE-submode handling and import-only PSK31 to PSK/PSK31 normalization are fixed. The remaining 3.1.8 enum/deprecation audit remains open; ADIF_VER stays 3.1.7.</x:v>
+        <x:v>Source complete for seven reviewed compatibility stages — local records retain a JSON field bag; unknown/custom fields, Unicode, station/contact and RX/TX data survive supported ADI/ADX round trips. UTF-8 byte scanning, FT4/FT2/JTTY MFSK-submode export, C4FM/DSTAR DIGITALVOICE-submode handling and import-only PSK31/PSK63/PSK63F to PSK/submode normalization are fixed. Latest Swift 18/18 and frontend 1,170/1,170 pass (CLI-timeout-only retry); current-source TypeScript passes. Remaining 3.1.8 audit and package/real-log acceptance stay open; ADIF_VER stays 3.1.7.</x:v>
       </x:c>
       <x:c r="C10" s="67" t="str">
         <x:v>Documented — import/export plus four user-definable logging fields.</x:v>
@@ -1076,12 +1076,12 @@
       <x:c r="E23" s="59"/>
       <x:c r="F23" s="59"/>
     </x:row>
-    <x:row r="24" ht="48" hidden="0" customHeight="1">
+    <x:row r="24" ht="84" hidden="0" customHeight="1">
       <x:c r="A24" s="66" t="str">
         <x:v>Online-log follow-up evidence</x:v>
       </x:c>
       <x:c r="B24" s="67" t="str">
-        <x:v>Core projection source complete — canonical QRZ/Club Log receipts expose delivery state, revision currency and attempt age while retained paper/LoTW/eQSL confirmations remain separate. Provider acceptance/match age and sponsor credit stay explicitly unknown; route/UI and live-account acceptance remain open.</x:v>
+        <x:v>Source and browser verified — generation-fenced local route and Logbook row panel expose canonical QRZ/Club Log delivery state, receipt revision and attempt age, separately from retained paper/LoTW/eQSL confirmations. Opening performs no fetch; explicit Refresh reads local evidence, and Close/context changes retire pending reads. Swift route 1/1, Rust permission 1/1, frontend 31/31, TypeScript/build/bundle gates and 640x480/1280x800 actual-Logbook browser checks pass. Provider acceptance/match age and sponsor credit remain unknown; exact-package/native and live-account acceptance remain open.</x:v>
       </x:c>
       <x:c r="C24" s="67" t="str">
         <x:v>Documented service status and confirmation workflows; exact evidence boundaries were not audited.</x:v>
@@ -1316,12 +1316,12 @@
       <x:c r="E38" s="59"/>
       <x:c r="F38" s="59"/>
     </x:row>
-    <x:row r="39" ht="96" hidden="0" customHeight="1">
+    <x:row r="39" ht="132" hidden="0" customHeight="1">
       <x:c r="A39" s="66" t="str">
         <x:v>TCI rig control — SunSDR/ExpertSDR and compatible servers</x:v>
       </x:c>
       <x:c r="B39" s="67" t="str">
-        <x:v>Source complete through observed receive-frequency/mode tuning, TRX-wide receive-filter adjustment, configured-TRX split observation, server-global TX-frequency telemetry and passive server spot-click events — bounded protocol/session, exact discovery, producer-time freshness, saved credential-free ws/wss setup and stale-aware UI. Explicit controls use the existing connection, durable no-replay receipts and newer exact readback. Global TX frequency and spot clicks remain separate telemetry and never become configured evidence, inventory or authority. Transmit/PTT, split/TX-VFO controls, outbound spot management, audio/IQ and package/live-server acceptance remain open.</x:v>
+        <x:v>Source complete through receive tune/filter, configured-TRX split, global TX-frequency telemetry, APP_FOCUS, addressed RX_CLICKED_ON_SPOT, legacy CLICKED_ON_SPOT and receipt-only CW_MACROS_EMPTY and opaque CALLSIGN_SEND observations. Passive notifications retain independent producer receipts; legacy clicks infer no TRX/channel/VFO. CW_MACROS_EMPTY proves no queue-empty, TX/RX, CW or RF authority. APP_FOCUS Swift 45/45, legacy-click 50/50 (lifecycle rerun) CW receipt 55/55 and CALLSIGN_SEND 60/60 (34 protocol + 26 session) pass. CALLSIGN_SEND uses strict validation/reconnect clearing and confers no target/contact identity authority, command correlation, TX completion/success or RF inference. Explicit controls retain the existing no-replay/readback owner. Transmit/PTT, split/TX-VFO controls, outbound spots, audio/IQ and package/live-server/RF acceptance remain open.</x:v>
       </x:c>
       <x:c r="C39" s="67" t="str">
         <x:v>Not established in the reviewed primary RUMlogNG evidence.</x:v>
@@ -1412,12 +1412,12 @@
       <x:c r="E44" s="59"/>
       <x:c r="F44" s="59"/>
     </x:row>
-    <x:row r="45" ht="24" hidden="0" customHeight="1">
+    <x:row r="45" ht="84" hidden="0" customHeight="1">
       <x:c r="A45" s="66" t="str">
         <x:v>Awards and statistics</x:v>
       </x:c>
       <x:c r="B45" s="67" t="str">
-        <x:v>Implemented foundation — nine native calculators plus a 192-programme research library; many programmes are tracking/blocked rather than falsely credited.</x:v>
+        <x:v>Implemented foundation — nine native calculators plus a 192-programme research library. 6d9b186 adds pure QRPDXCCPreflightV1 snapshot screening (7/7 Swift) as an R09 dependency only: candidates/exclusions/unknowns and exact retained-power checks. Candidate stored DXCCs are not validated entities, progress, completion or sponsor credit. Measurement, sponsor validity, applicant scope, land/direct-contact eligibility and declaration remain unresolved; executable sponsor rules, application/export, route/UI and package/live acceptance stay open.</x:v>
       </x:c>
       <x:c r="C45" s="67" t="str">
         <x:v>Documented — DXCC plus IOTA, CQ/ITU zones, grids, states, counties, DOKs and detailed QSL statistics.</x:v>
@@ -2738,7 +2738,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc1394a2ba5414e01"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R02c02717c7284122"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2930,7 +2930,7 @@
         <x:v>ADIF 3.1.8 conformance</x:v>
       </x:c>
       <x:c r="C12" s="67" t="str">
-        <x:v>Five compatibility fixes complete</x:v>
+        <x:v>Seven compatibility stages complete</x:v>
       </x:c>
       <x:c r="D12" s="67" t="str">
         <x:v>Complete the remaining enum/deprecation and MODE/SUBMODE audit before changing ADIF_VER; run copied-log/package and service-specific interoperability acceptance.</x:v>
@@ -2962,7 +2962,7 @@
         <x:v>Official/date-qualified CTY rules</x:v>
       </x:c>
     </x:row>
-    <x:row r="14" ht="48" hidden="0" customHeight="1">
+    <x:row r="14" ht="108" hidden="0" customHeight="1">
       <x:c r="A14" s="66" t="str">
         <x:v>P1</x:v>
       </x:c>
@@ -2970,10 +2970,10 @@
         <x:v>Full TCI radio provider</x:v>
       </x:c>
       <x:c r="C14" s="67" t="str">
-        <x:v>Receive tune/filter plus passive split, TX-frequency and spot-click observation source complete</x:v>
+        <x:v>Receive tune/filter plus passive split, TX-frequency, APP_FOCUS, addressed/legacy spot-click CW_MACROS_EMPTY receipt and opaque CALLSIGN_SEND observations source complete</x:v>
       </x:c>
       <x:c r="D14" s="67" t="str">
-        <x:v>Extend the existing no-replay owner with separately reviewed split/TX-VFO controls, urgent release and optional audio/IQ slices; do not assign global TX frequency or spot-click events to configured evidence/inventory. Transmit/PTT keeps its own explicit authority.</x:v>
+        <x:v>Extend the existing no-replay owner with separately reviewed split/TX-VFO controls, urgent release and optional audio/IQ slices; passive notifications never become configured evidence/inventory or CW/RF authority. Transmit/PTT keeps its own explicit authority.</x:v>
       </x:c>
       <x:c r="E14" s="67" t="str">
         <x:v>Simulated-server races, package tests, then operator-controlled SunSDR acceptance</x:v>
@@ -3150,13 +3150,13 @@
         <x:v>Online-log follow-up UI</x:v>
       </x:c>
       <x:c r="C23" s="67" t="str">
-        <x:v>Core projection source complete</x:v>
+        <x:v>Read-only route/UI source and browser verified</x:v>
       </x:c>
       <x:c r="D23" s="67" t="str">
-        <x:v>Add a bounded worker/native surface only after the provider acceptance/match timestamp contract is explicit; never infer confirmation or sponsor credit from upload delivery.</x:v>
+        <x:v>Accept the exact package/native interaction; define provider acceptance/match timestamps and sponsor rules before extending the retained-evidence contract. Upload delivery never establishes confirmation or sponsor credit.</x:v>
       </x:c>
       <x:c r="E23" s="67" t="str">
-        <x:v>Focused route/UI tests, exact package and live-account evidence</x:v>
+        <x:v>Exact-package/native interaction and live-account evidence</x:v>
       </x:c>
       <x:c r="F23" s="67" t="str">
         <x:v>RUMlogNG/QLog online-log status workflows</x:v>
@@ -4640,7 +4640,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rca28128b13914bb3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4a02a4fb4df24c5f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4783,13 +4783,13 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="C10" s="67" t="str">
-        <x:v>Five compatibility fixes complete</x:v>
+        <x:v>Seven compatibility stages complete</x:v>
       </x:c>
       <x:c r="D10" s="67" t="str">
         <x:v>ADIF parser/writer and frontend transfer</x:v>
       </x:c>
       <x:c r="E10" s="67" t="str">
-        <x:v>Finish the remaining 3.1.8 enum/deprecation audit before header bump.</x:v>
+        <x:v>Finish remaining 3.1.8 audit after PSK63/PSK63F; retain ADIF_VER 3.1.7.</x:v>
       </x:c>
       <x:c r="F10" s="59"/>
     </x:row>
@@ -4837,13 +4837,13 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="C13" s="67" t="str">
-        <x:v>Core evidence projection complete; route/UI open</x:v>
+        <x:v>Read-only route/UI source and browser verified; package/provider open</x:v>
       </x:c>
       <x:c r="D13" s="67" t="str">
         <x:v>Sync/delivery/confirmation and award state</x:v>
       </x:c>
       <x:c r="E13" s="67" t="str">
-        <x:v>Expose the bounded projection after provider timestamp and sponsor-rule contracts; keep upload, confirmation and credit distinct.</x:v>
+        <x:v>Package-test 5486aff; retain unknown provider ages/credit until timestamp and sponsor-rule contracts exist.</x:v>
       </x:c>
       <x:c r="F13" s="59"/>
     </x:row>
@@ -4865,7 +4865,7 @@
       </x:c>
       <x:c r="F14" s="59"/>
     </x:row>
-    <x:row r="15" ht="15" hidden="0" customHeight="1">
+    <x:row r="15" ht="36" hidden="0" customHeight="1">
       <x:c r="A15" s="66" t="str">
         <x:v>R09</x:v>
       </x:c>
@@ -4873,13 +4873,13 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="C15" s="67" t="str">
-        <x:v>Useful extension</x:v>
+        <x:v>QRP DXCC preflight dependency source complete; executable award open</x:v>
       </x:c>
       <x:c r="D15" s="67" t="str">
-        <x:v>Award calculators and research registry</x:v>
+        <x:v>Award calculators, research registry and QRPDXCCPreflightV1</x:v>
       </x:c>
       <x:c r="E15" s="67" t="str">
-        <x:v>One executable dated sponsor pack and supported application/export.</x:v>
+        <x:v>7/7 Swift screens candidates only; resolve measurement/sponsor/scope/eligibility/declaration requirements before executable rules, application/export or credit.</x:v>
       </x:c>
       <x:c r="F15" s="59"/>
     </x:row>
@@ -6527,7 +6527,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9919fb6ed1614c66"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R33002aae89ca4fa4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6602,34 +6602,34 @@
       <x:c r="E6" s="59"/>
       <x:c r="F6" s="59"/>
     </x:row>
-    <x:row r="7" ht="24" hidden="0" customHeight="1">
+    <x:row r="7" ht="36" hidden="0" customHeight="1">
       <x:c r="A7" s="64" t="str">
         <x:v>OM0RX-xLog</x:v>
       </x:c>
       <x:c r="B7" s="65" t="str">
-        <x:v>Current implementation checkpoint 259b05d37d5d133ff9c3c9a7a659e851d81507e8</x:v>
+        <x:v>Current implementation checkpoint 7b2e0ea83490b98cd40f45a4881a949665b1a715</x:v>
       </x:c>
       <x:c r="C7" s="65" t="str">
         <x:v>2026-10-16</x:v>
       </x:c>
       <x:c r="D7" s="65" t="str">
-        <x:v>PROJECT_STATUS.md, PROJECT_BOARD.md, operator-feedback tracker and enhancement-recommendations reconciliation. Source/package/live/hardware states are kept separate.</x:v>
+        <x:v>PROJECT_STATUS.md, PROJECT_BOARD.md, operator-feedback tracker and enhancement-recommendations reconciliation. Source/test/browser results remain separate from package/native/live/hardware acceptance; installed alpha.31 is unchanged.</x:v>
       </x:c>
       <x:c r="E7" s="59"/>
       <x:c r="F7" s="59"/>
     </x:row>
-    <x:row r="8" ht="48" hidden="0" customHeight="1">
+    <x:row r="8" ht="60" hidden="0" customHeight="1">
       <x:c r="A8" s="66" t="str">
         <x:v>OM0RX-xLog</x:v>
       </x:c>
       <x:c r="B8" s="67" t="str">
-        <x:v>https://github.com/oliverbross/OM0RX-xLog/commit/259b05d37d5d133ff9c3c9a7a659e851d81507e8</x:v>
+        <x:v>https://github.com/oliverbross/OM0RX-xLog/commit/7b2e0ea83490b98cd40f45a4881a949665b1a715</x:v>
       </x:c>
       <x:c r="C8" s="67" t="str">
         <x:v>2026-10-16</x:v>
       </x:c>
       <x:c r="D8" s="67" t="str">
-        <x:v>Exact committed implementation baseline including passive TCI spot-click telemetry, QRZ/Club Log follow-up evidence, PSK31 deprecation compatibility, the OM0RX-xLog document title, earlier TCI receive tune/filter/split/global-TX stages, Operating Goals, Connection Doctor, saved filters, responsive windows, PJ/DXCC preview and Previous QSOs.</x:v>
+        <x:v>Exact committed implementation baseline includes conservative QRP DXCC preflight dependency (6d9b186), PSK63 (3002e96), PSK63F (a118dea), passive TCI APP_FOCUS (1e11f0f), legacy CLICKED_ON_SPOT (89cac01), receipt-only CW_MACROS_EMPTY (30ed9d0), passive CALLSIGN_SEND (7b2e0ea) and read-only online-log follow-up route/Logbook UI (5486aff), plus earlier tracked stages. Preflight does not implement an executable sponsor award or credit.</x:v>
       </x:c>
       <x:c r="E8" s="59"/>
       <x:c r="F8" s="59"/>
@@ -8256,7 +8256,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9a148ad66f1b49f4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc8524e8f6c554952"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Track passive TCI VFO lock stage
</commit_message>
<xml_diff>
--- a/outputs/feature-matrix-2026-10-16/OM0RX-xLog_Feature_Comparison_2026-10-16.xlsx
+++ b/outputs/feature-matrix-2026-10-16/OM0RX-xLog_Feature_Comparison_2026-10-16.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Matrix" sheetId="1" r:id="Re0b4912c92084d5a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Outstanding" sheetId="2" r:id="R0c8d239aa2034edd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enhancement Review" sheetId="3" r:id="R2f2679c3e7aa4ebc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="4" r:id="R61cd216046194268"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Matrix" sheetId="1" r:id="R1b6580a98ed14e24"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Outstanding" sheetId="2" r:id="Rf04e6379a75c4d15"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enhancement Review" sheetId="3" r:id="Rc80e4dc3fa1443f9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="4" r:id="R369262a2fded43c2"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1316,12 +1316,12 @@
       <x:c r="E38" s="59"/>
       <x:c r="F38" s="59"/>
     </x:row>
-    <x:row r="39" ht="132" hidden="0" customHeight="1">
+    <x:row r="39" ht="168" hidden="0" customHeight="1">
       <x:c r="A39" s="66" t="str">
         <x:v>TCI rig control — SunSDR/ExpertSDR and compatible servers</x:v>
       </x:c>
       <x:c r="B39" s="67" t="str">
-        <x:v>Source complete through receive tune/filter, configured-TRX split, global TX-frequency telemetry, APP_FOCUS, addressed RX_CLICKED_ON_SPOT, legacy CLICKED_ON_SPOT and receipt-only CW_MACROS_EMPTY and opaque CALLSIGN_SEND observations. Passive notifications retain independent producer receipts; legacy clicks infer no TRX/channel/VFO. CW_MACROS_EMPTY proves no queue-empty, TX/RX, CW or RF authority. APP_FOCUS Swift 45/45, legacy-click 50/50 (lifecycle rerun) CW receipt 55/55 and CALLSIGN_SEND 60/60 (34 protocol + 26 session) pass. CALLSIGN_SEND uses strict validation/reconnect clearing and confers no target/contact identity authority, command correlation, TX completion/success or RF inference. Explicit controls retain the existing no-replay/readback owner. Transmit/PTT, split/TX-VFO controls, outbound spots, audio/IQ and package/live-server/RF acceptance remain open.</x:v>
+        <x:v>Source complete through receive tune/filter, configured-TRX split, global TX-frequency telemetry, APP_FOCUS, addressed RX_CLICKED_ON_SPOT, legacy CLICKED_ON_SPOT and receipt-only CW_MACROS_EMPTY and opaque CALLSIGN_SEND and per-address VFO_LOCK observations. Passive notifications retain independent producer receipts; legacy clicks infer no TRX/channel/VFO. CW_MACROS_EMPTY proves no queue-empty, TX/RX, CW or RF authority. APP_FOCUS Swift 45/45, legacy-click 50/50 (lifecycle rerun) CW receipt 55/55 and CALLSIGN_SEND 60/60 (34 protocol + 26 session) pass. CALLSIGN_SEND uses strict validation/reconnect clearing and confers no target/contact identity authority, command correlation, TX completion/success or RF inference. VFO_LOCK 66/66 (38 protocol + 28 session) retains independent exact-address producer times, validates exactly three arguments within application/discovery bounds, prunes on discovery shrink and clears on reconnect. It grants no owner/expiry, tune confirmation, configured freshness or control authority. Explicit controls retain the existing no-replay/readback owner. Transmit/PTT, split/TX-VFO controls, outbound spots, audio/IQ and package/live-server/RF acceptance remain open.</x:v>
       </x:c>
       <x:c r="C39" s="67" t="str">
         <x:v>Not established in the reviewed primary RUMlogNG evidence.</x:v>
@@ -2738,7 +2738,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R02c02717c7284122"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rce75c4f8be344af7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2962,7 +2962,7 @@
         <x:v>Official/date-qualified CTY rules</x:v>
       </x:c>
     </x:row>
-    <x:row r="14" ht="108" hidden="0" customHeight="1">
+    <x:row r="14" ht="120" hidden="0" customHeight="1">
       <x:c r="A14" s="66" t="str">
         <x:v>P1</x:v>
       </x:c>
@@ -2970,7 +2970,7 @@
         <x:v>Full TCI radio provider</x:v>
       </x:c>
       <x:c r="C14" s="67" t="str">
-        <x:v>Receive tune/filter plus passive split, TX-frequency, APP_FOCUS, addressed/legacy spot-click CW_MACROS_EMPTY receipt and opaque CALLSIGN_SEND observations source complete</x:v>
+        <x:v>Receive tune/filter plus passive split, TX-frequency, APP_FOCUS, addressed/legacy spot-click CW_MACROS_EMPTY receipt and opaque CALLSIGN_SEND plus exact-address VFO_LOCK observations source complete</x:v>
       </x:c>
       <x:c r="D14" s="67" t="str">
         <x:v>Extend the existing no-replay owner with separately reviewed split/TX-VFO controls, urgent release and optional audio/IQ slices; passive notifications never become configured evidence/inventory or CW/RF authority. Transmit/PTT keeps its own explicit authority.</x:v>
@@ -4640,7 +4640,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4a02a4fb4df24c5f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R119f8e9327d54ea9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6527,7 +6527,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R33002aae89ca4fa4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra354221105f34519"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6607,7 +6607,7 @@
         <x:v>OM0RX-xLog</x:v>
       </x:c>
       <x:c r="B7" s="65" t="str">
-        <x:v>Current implementation checkpoint 7b2e0ea83490b98cd40f45a4881a949665b1a715</x:v>
+        <x:v>Current implementation checkpoint 6c1cad01b01c85772cfd8748bc3d9819dbd6ee32</x:v>
       </x:c>
       <x:c r="C7" s="65" t="str">
         <x:v>2026-10-16</x:v>
@@ -6618,18 +6618,18 @@
       <x:c r="E7" s="59"/>
       <x:c r="F7" s="59"/>
     </x:row>
-    <x:row r="8" ht="60" hidden="0" customHeight="1">
+    <x:row r="8" ht="72" hidden="0" customHeight="1">
       <x:c r="A8" s="66" t="str">
         <x:v>OM0RX-xLog</x:v>
       </x:c>
       <x:c r="B8" s="67" t="str">
-        <x:v>https://github.com/oliverbross/OM0RX-xLog/commit/7b2e0ea83490b98cd40f45a4881a949665b1a715</x:v>
+        <x:v>https://github.com/oliverbross/OM0RX-xLog/commit/6c1cad01b01c85772cfd8748bc3d9819dbd6ee32</x:v>
       </x:c>
       <x:c r="C8" s="67" t="str">
         <x:v>2026-10-16</x:v>
       </x:c>
       <x:c r="D8" s="67" t="str">
-        <x:v>Exact committed implementation baseline includes conservative QRP DXCC preflight dependency (6d9b186), PSK63 (3002e96), PSK63F (a118dea), passive TCI APP_FOCUS (1e11f0f), legacy CLICKED_ON_SPOT (89cac01), receipt-only CW_MACROS_EMPTY (30ed9d0), passive CALLSIGN_SEND (7b2e0ea) and read-only online-log follow-up route/Logbook UI (5486aff), plus earlier tracked stages. Preflight does not implement an executable sponsor award or credit.</x:v>
+        <x:v>Exact committed implementation baseline includes conservative QRP DXCC preflight dependency (6d9b186), PSK63 (3002e96), PSK63F (a118dea), passive TCI APP_FOCUS (1e11f0f), legacy CLICKED_ON_SPOT (89cac01), receipt-only CW_MACROS_EMPTY (30ed9d0), passive CALLSIGN_SEND (7b2e0ea), passive VFO_LOCK (6c1cad0) and read-only online-log follow-up route/Logbook UI (5486aff), plus earlier tracked stages. Preflight does not implement an executable sponsor award or credit.</x:v>
       </x:c>
       <x:c r="E8" s="59"/>
       <x:c r="F8" s="59"/>
@@ -8256,7 +8256,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc8524e8f6c554952"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf29a2fe14d5f4c21"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Track TCI receive sensor evidence
</commit_message>
<xml_diff>
--- a/outputs/feature-matrix-2026-10-16/OM0RX-xLog_Feature_Comparison_2026-10-16.xlsx
+++ b/outputs/feature-matrix-2026-10-16/OM0RX-xLog_Feature_Comparison_2026-10-16.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Matrix" sheetId="1" r:id="R1b6580a98ed14e24"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Outstanding" sheetId="2" r:id="Rf04e6379a75c4d15"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enhancement Review" sheetId="3" r:id="Rc80e4dc3fa1443f9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="4" r:id="R369262a2fded43c2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Matrix" sheetId="1" r:id="R5a99edd6b4e940a6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Outstanding" sheetId="2" r:id="R4b09ecb01c7b4c53"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enhancement Review" sheetId="3" r:id="Rc743aefcfbd54d16"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="4" r:id="R30030b2f7ae741b5"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1316,12 +1316,12 @@
       <x:c r="E38" s="59"/>
       <x:c r="F38" s="59"/>
     </x:row>
-    <x:row r="39" ht="168" hidden="0" customHeight="1">
+    <x:row r="39" ht="240" hidden="0" customHeight="1">
       <x:c r="A39" s="66" t="str">
         <x:v>TCI rig control — SunSDR/ExpertSDR and compatible servers</x:v>
       </x:c>
       <x:c r="B39" s="67" t="str">
-        <x:v>Source complete through receive tune/filter, configured-TRX split, global TX-frequency telemetry, APP_FOCUS, addressed RX_CLICKED_ON_SPOT, legacy CLICKED_ON_SPOT and receipt-only CW_MACROS_EMPTY and opaque CALLSIGN_SEND and per-address VFO_LOCK observations. Passive notifications retain independent producer receipts; legacy clicks infer no TRX/channel/VFO. CW_MACROS_EMPTY proves no queue-empty, TX/RX, CW or RF authority. APP_FOCUS Swift 45/45, legacy-click 50/50 (lifecycle rerun) CW receipt 55/55 and CALLSIGN_SEND 60/60 (34 protocol + 26 session) pass. CALLSIGN_SEND uses strict validation/reconnect clearing and confers no target/contact identity authority, command correlation, TX completion/success or RF inference. VFO_LOCK 66/66 (38 protocol + 28 session) retains independent exact-address producer times, validates exactly three arguments within application/discovery bounds, prunes on discovery shrink and clears on reconnect. It grants no owner/expiry, tune confirmation, configured freshness or control authority. Explicit controls retain the existing no-replay/readback owner. Transmit/PTT, split/TX-VFO controls, outbound spots, audio/IQ and package/live-server/RF acceptance remain open.</x:v>
+        <x:v>Source complete through receive tune/filter, configured-TRX split, global TX-frequency telemetry, APP_FOCUS, addressed RX_CLICKED_ON_SPOT, legacy CLICKED_ON_SPOT and receipt-only CW_MACROS_EMPTY and opaque CALLSIGN_SEND and per-address VFO_LOCK plus RX_CHANNEL_SENSORS token observations. Passive notifications retain independent producer receipts; legacy clicks infer no TRX/channel/VFO. CW_MACROS_EMPTY proves no queue-empty, TX/RX, CW or RF authority. APP_FOCUS Swift 45/45, legacy-click 50/50 (lifecycle rerun) CW receipt 55/55 and CALLSIGN_SEND 60/60 (34 protocol + 26 session) pass. CALLSIGN_SEND uses strict validation/reconnect clearing and confers no target/contact identity authority, command correlation, TX completion/success or RF inference. VFO_LOCK 66/66 (38 protocol + 28 session) retains independent exact-address producer times, validates exactly three arguments within application/discovery bounds, prunes on discovery shrink and clears on reconnect. It grants no owner/expiry, tune confirmation, configured freshness or control authority. RX_CHANNEL_SENSORS preserves exact bounded ASCII decimals per address without Double conversion or physical range/calibration/quality/readiness/freshness/control claims; discovery prunes and reconnect clears. Six new tests pass twice, protocol 42/42; broader session rerun remains 71/72 on unchanged testDroppingLastSessionReferenceClosesPendingConnection (closeCount 0 vs 1); initial existing tune-yield miss passed rerun. Build/diff clean; full session gate open. Explicit controls retain the existing no-replay/readback owner. Transmit/PTT, split/TX-VFO controls, outbound spots, audio/IQ and package/live-server/RF acceptance remain open.</x:v>
       </x:c>
       <x:c r="C39" s="67" t="str">
         <x:v>Not established in the reviewed primary RUMlogNG evidence.</x:v>
@@ -2738,7 +2738,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rce75c4f8be344af7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Red1e19b2bcbe4a88"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2962,7 +2962,7 @@
         <x:v>Official/date-qualified CTY rules</x:v>
       </x:c>
     </x:row>
-    <x:row r="14" ht="120" hidden="0" customHeight="1">
+    <x:row r="14" ht="132" hidden="0" customHeight="1">
       <x:c r="A14" s="66" t="str">
         <x:v>P1</x:v>
       </x:c>
@@ -2970,7 +2970,7 @@
         <x:v>Full TCI radio provider</x:v>
       </x:c>
       <x:c r="C14" s="67" t="str">
-        <x:v>Receive tune/filter plus passive split, TX-frequency, APP_FOCUS, addressed/legacy spot-click CW_MACROS_EMPTY receipt and opaque CALLSIGN_SEND plus exact-address VFO_LOCK observations source complete</x:v>
+        <x:v>Receive tune/filter plus passive split, TX-frequency, APP_FOCUS, addressed/legacy spot-click CW_MACROS_EMPTY receipt and opaque CALLSIGN_SEND plus VFO_LOCK and RX_CHANNEL_SENSORS tokens source complete; broader session 71/72</x:v>
       </x:c>
       <x:c r="D14" s="67" t="str">
         <x:v>Extend the existing no-replay owner with separately reviewed split/TX-VFO controls, urgent release and optional audio/IQ slices; passive notifications never become configured evidence/inventory or CW/RF authority. Transmit/PTT keeps its own explicit authority.</x:v>
@@ -4640,7 +4640,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R119f8e9327d54ea9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra505eb6f1d0e4cb0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6527,7 +6527,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra354221105f34519"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8f08924a06c24f1e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6607,7 +6607,7 @@
         <x:v>OM0RX-xLog</x:v>
       </x:c>
       <x:c r="B7" s="65" t="str">
-        <x:v>Current implementation checkpoint 6c1cad01b01c85772cfd8748bc3d9819dbd6ee32</x:v>
+        <x:v>Current implementation checkpoint ed8ed379005a170629988a136fb872124ab4ea33</x:v>
       </x:c>
       <x:c r="C7" s="65" t="str">
         <x:v>2026-10-16</x:v>
@@ -6623,13 +6623,13 @@
         <x:v>OM0RX-xLog</x:v>
       </x:c>
       <x:c r="B8" s="67" t="str">
-        <x:v>https://github.com/oliverbross/OM0RX-xLog/commit/6c1cad01b01c85772cfd8748bc3d9819dbd6ee32</x:v>
+        <x:v>https://github.com/oliverbross/OM0RX-xLog/commit/ed8ed379005a170629988a136fb872124ab4ea33</x:v>
       </x:c>
       <x:c r="C8" s="67" t="str">
         <x:v>2026-10-16</x:v>
       </x:c>
       <x:c r="D8" s="67" t="str">
-        <x:v>Exact committed implementation baseline includes conservative QRP DXCC preflight dependency (6d9b186), PSK63 (3002e96), PSK63F (a118dea), passive TCI APP_FOCUS (1e11f0f), legacy CLICKED_ON_SPOT (89cac01), receipt-only CW_MACROS_EMPTY (30ed9d0), passive CALLSIGN_SEND (7b2e0ea), passive VFO_LOCK (6c1cad0) and read-only online-log follow-up route/Logbook UI (5486aff), plus earlier tracked stages. Preflight does not implement an executable sponsor award or credit.</x:v>
+        <x:v>Exact committed implementation baseline includes conservative QRP DXCC preflight dependency (6d9b186), PSK63 (3002e96), PSK63F (a118dea), passive TCI APP_FOCUS (1e11f0f), legacy CLICKED_ON_SPOT (89cac01), receipt-only CW_MACROS_EMPTY (30ed9d0), passive CALLSIGN_SEND (7b2e0ea), passive VFO_LOCK (6c1cad0), exact-token RX_CHANNEL_SENSORS (ed8ed37; broader session gate remains 71/72) and read-only online-log follow-up route/Logbook UI (5486aff), plus earlier tracked stages. Preflight does not implement an executable sponsor award or credit.</x:v>
       </x:c>
       <x:c r="E8" s="59"/>
       <x:c r="F8" s="59"/>
@@ -8256,7 +8256,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf29a2fe14d5f4c21"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R749ea292cd2745c2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Track deprecated TCI sensor evidence
</commit_message>
<xml_diff>
--- a/outputs/feature-matrix-2026-10-16/OM0RX-xLog_Feature_Comparison_2026-10-16.xlsx
+++ b/outputs/feature-matrix-2026-10-16/OM0RX-xLog_Feature_Comparison_2026-10-16.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Matrix" sheetId="1" r:id="R5a99edd6b4e940a6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Outstanding" sheetId="2" r:id="R4b09ecb01c7b4c53"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enhancement Review" sheetId="3" r:id="Rc743aefcfbd54d16"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="4" r:id="R30030b2f7ae741b5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Matrix" sheetId="1" r:id="R93033a0df4804905"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Outstanding" sheetId="2" r:id="R50da18b7c0444e0c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enhancement Review" sheetId="3" r:id="R4edc326067c94b6b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="4" r:id="R01c6549883de45ca"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1316,12 +1316,12 @@
       <x:c r="E38" s="59"/>
       <x:c r="F38" s="59"/>
     </x:row>
-    <x:row r="39" ht="240" hidden="0" customHeight="1">
+    <x:row r="39" ht="312" hidden="0" customHeight="1">
       <x:c r="A39" s="66" t="str">
         <x:v>TCI rig control — SunSDR/ExpertSDR and compatible servers</x:v>
       </x:c>
       <x:c r="B39" s="67" t="str">
-        <x:v>Source complete through receive tune/filter, configured-TRX split, global TX-frequency telemetry, APP_FOCUS, addressed RX_CLICKED_ON_SPOT, legacy CLICKED_ON_SPOT and receipt-only CW_MACROS_EMPTY and opaque CALLSIGN_SEND and per-address VFO_LOCK plus RX_CHANNEL_SENSORS token observations. Passive notifications retain independent producer receipts; legacy clicks infer no TRX/channel/VFO. CW_MACROS_EMPTY proves no queue-empty, TX/RX, CW or RF authority. APP_FOCUS Swift 45/45, legacy-click 50/50 (lifecycle rerun) CW receipt 55/55 and CALLSIGN_SEND 60/60 (34 protocol + 26 session) pass. CALLSIGN_SEND uses strict validation/reconnect clearing and confers no target/contact identity authority, command correlation, TX completion/success or RF inference. VFO_LOCK 66/66 (38 protocol + 28 session) retains independent exact-address producer times, validates exactly three arguments within application/discovery bounds, prunes on discovery shrink and clears on reconnect. It grants no owner/expiry, tune confirmation, configured freshness or control authority. RX_CHANNEL_SENSORS preserves exact bounded ASCII decimals per address without Double conversion or physical range/calibration/quality/readiness/freshness/control claims; discovery prunes and reconnect clears. Six new tests pass twice, protocol 42/42; broader session rerun remains 71/72 on unchanged testDroppingLastSessionReferenceClosesPendingConnection (closeCount 0 vs 1); initial existing tune-yield miss passed rerun. Build/diff clean; full session gate open. Explicit controls retain the existing no-replay/readback owner. Transmit/PTT, split/TX-VFO controls, outbound spots, audio/IQ and package/live-server/RF acceptance remain open.</x:v>
+        <x:v>Source complete through receive tune/filter, configured-TRX split, global TX-frequency telemetry, APP_FOCUS, addressed RX_CLICKED_ON_SPOT, legacy CLICKED_ON_SPOT and receipt-only CW_MACROS_EMPTY and opaque CALLSIGN_SEND and per-address VFO_LOCK plus RX_CHANNEL_SENSORS and separate deprecated RX_SENSORS token observations. Passive notifications retain independent producer receipts; legacy clicks infer no TRX/channel/VFO. CW_MACROS_EMPTY proves no queue-empty, TX/RX, CW or RF authority. APP_FOCUS Swift 45/45, legacy-click 50/50 (lifecycle rerun) CW receipt 55/55 and CALLSIGN_SEND 60/60 (34 protocol + 26 session) pass. CALLSIGN_SEND uses strict validation/reconnect clearing and confers no target/contact identity authority, command correlation, TX completion/success or RF inference. VFO_LOCK 66/66 (38 protocol + 28 session) retains independent exact-address producer times, validates exactly three arguments within application/discovery bounds, prunes on discovery shrink and clears on reconnect. It grants no owner/expiry, tune confirmation, configured freshness or control authority. RX_CHANNEL_SENSORS preserves exact bounded ASCII decimals per address without Double conversion or physical range/calibration/quality/readiness/freshness/control claims; discovery prunes and reconnect clears. Six new tests pass twice, protocol 42/42; broader session rerun at ed8ed37 was 71/72 on unchanged testDroppingLastSessionReferenceClosesPendingConnection (closeCount 0 vs 1); initial existing tune-yield miss passed rerun. Build/diff clean. 2d7bb1f adds deprecated server-only RX_SENSORS as separate per-TRX raw bounded decimal tokens plus local producer receipt, never channel-attributed or merged with RX_CHANNEL_SENSORS. TRX discovery prunes, channel-count changes do not remap and reconnect clears. No physical range/calibration/readiness/freshness/control/RF inference. Later independent focused tests 78/78 pass; earlier timing miss is not claimed fixed. Explicit controls retain the existing no-replay/readback owner. Transmit/PTT, split/TX-VFO controls, outbound spots, audio/IQ and package/live-server/RF acceptance remain open.</x:v>
       </x:c>
       <x:c r="C39" s="67" t="str">
         <x:v>Not established in the reviewed primary RUMlogNG evidence.</x:v>
@@ -2738,7 +2738,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Red1e19b2bcbe4a88"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf808ae769514475a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2962,7 +2962,7 @@
         <x:v>Official/date-qualified CTY rules</x:v>
       </x:c>
     </x:row>
-    <x:row r="14" ht="132" hidden="0" customHeight="1">
+    <x:row r="14" ht="156" hidden="0" customHeight="1">
       <x:c r="A14" s="66" t="str">
         <x:v>P1</x:v>
       </x:c>
@@ -2970,7 +2970,7 @@
         <x:v>Full TCI radio provider</x:v>
       </x:c>
       <x:c r="C14" s="67" t="str">
-        <x:v>Receive tune/filter plus passive split, TX-frequency, APP_FOCUS, addressed/legacy spot-click CW_MACROS_EMPTY receipt and opaque CALLSIGN_SEND plus VFO_LOCK and RX_CHANNEL_SENSORS tokens source complete; broader session 71/72</x:v>
+        <x:v>Receive tune/filter plus passive split, TX-frequency, APP_FOCUS, addressed/legacy spot-click CW_MACROS_EMPTY receipt and opaque CALLSIGN_SEND plus VFO_LOCK, RX_CHANNEL_SENSORS and separate deprecated RX_SENSORS tokens source complete; latest focused tests 78/78</x:v>
       </x:c>
       <x:c r="D14" s="67" t="str">
         <x:v>Extend the existing no-replay owner with separately reviewed split/TX-VFO controls, urgent release and optional audio/IQ slices; passive notifications never become configured evidence/inventory or CW/RF authority. Transmit/PTT keeps its own explicit authority.</x:v>
@@ -4640,7 +4640,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra505eb6f1d0e4cb0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R861ec0cd4c5a471c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6527,7 +6527,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8f08924a06c24f1e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfe3962042cb6446c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6607,7 +6607,7 @@
         <x:v>OM0RX-xLog</x:v>
       </x:c>
       <x:c r="B7" s="65" t="str">
-        <x:v>Current implementation checkpoint ed8ed379005a170629988a136fb872124ab4ea33</x:v>
+        <x:v>Current implementation checkpoint 2d7bb1f627139c55cd32e5dd673dab4d271031d1</x:v>
       </x:c>
       <x:c r="C7" s="65" t="str">
         <x:v>2026-10-16</x:v>
@@ -6618,18 +6618,18 @@
       <x:c r="E7" s="59"/>
       <x:c r="F7" s="59"/>
     </x:row>
-    <x:row r="8" ht="72" hidden="0" customHeight="1">
+    <x:row r="8" ht="84" hidden="0" customHeight="1">
       <x:c r="A8" s="66" t="str">
         <x:v>OM0RX-xLog</x:v>
       </x:c>
       <x:c r="B8" s="67" t="str">
-        <x:v>https://github.com/oliverbross/OM0RX-xLog/commit/ed8ed379005a170629988a136fb872124ab4ea33</x:v>
+        <x:v>https://github.com/oliverbross/OM0RX-xLog/commit/2d7bb1f627139c55cd32e5dd673dab4d271031d1</x:v>
       </x:c>
       <x:c r="C8" s="67" t="str">
         <x:v>2026-10-16</x:v>
       </x:c>
       <x:c r="D8" s="67" t="str">
-        <x:v>Exact committed implementation baseline includes conservative QRP DXCC preflight dependency (6d9b186), PSK63 (3002e96), PSK63F (a118dea), passive TCI APP_FOCUS (1e11f0f), legacy CLICKED_ON_SPOT (89cac01), receipt-only CW_MACROS_EMPTY (30ed9d0), passive CALLSIGN_SEND (7b2e0ea), passive VFO_LOCK (6c1cad0), exact-token RX_CHANNEL_SENSORS (ed8ed37; broader session gate remains 71/72) and read-only online-log follow-up route/Logbook UI (5486aff), plus earlier tracked stages. Preflight does not implement an executable sponsor award or credit.</x:v>
+        <x:v>Exact committed implementation baseline includes conservative QRP DXCC preflight dependency (6d9b186), PSK63 (3002e96), PSK63F (a118dea), passive TCI APP_FOCUS (1e11f0f), legacy CLICKED_ON_SPOT (89cac01), receipt-only CW_MACROS_EMPTY (30ed9d0), passive CALLSIGN_SEND (7b2e0ea), passive VFO_LOCK (6c1cad0), exact-token RX_CHANNEL_SENSORS (ed8ed37; earlier rerun 71/72), separate deprecated per-TRX RX_SENSORS (2d7bb1f; later independent focused 78/78) and read-only online-log follow-up route/Logbook UI (5486aff), plus earlier tracked stages. Preflight does not implement an executable sponsor award or credit.</x:v>
       </x:c>
       <x:c r="E8" s="59"/>
       <x:c r="F8" s="59"/>
@@ -8256,7 +8256,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R749ea292cd2745c2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R281677291b2c43f7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Track ADIF TCI and data quality stages
</commit_message>
<xml_diff>
--- a/outputs/feature-matrix-2026-10-16/OM0RX-xLog_Feature_Comparison_2026-10-16.xlsx
+++ b/outputs/feature-matrix-2026-10-16/OM0RX-xLog_Feature_Comparison_2026-10-16.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Matrix" sheetId="1" r:id="R93033a0df4804905"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Outstanding" sheetId="2" r:id="R50da18b7c0444e0c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enhancement Review" sheetId="3" r:id="R4edc326067c94b6b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="4" r:id="R01c6549883de45ca"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Matrix" sheetId="1" r:id="R8d425f43706f4800"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Outstanding" sheetId="2" r:id="R4d9341c6dd62478a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enhancement Review" sheetId="3" r:id="Ra028556bac284a5d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="4" r:id="R5ef82882c9864c10"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -482,7 +482,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="FeatureComparisonTable" displayName="FeatureComparisonTable" ref="A6:D52" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="FeatureComparisonTable" displayName="FeatureComparisonTable" ref="A6:D53" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="4">
     <x:tableColumn id="1" name="Feature"/>
     <x:tableColumn id="2" name="OM0RX-xLog"/>
@@ -769,7 +769,7 @@
         <x:v>Implemented or source complete</x:v>
       </x:c>
       <x:c r="B4" s="18" t="n">
-        <x:v>33</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="C4" s="18" t="str">
         <x:v>Active, partial or outstanding</x:v>
@@ -852,699 +852,707 @@
       <x:c r="E9" s="59"/>
       <x:c r="F9" s="59"/>
     </x:row>
-    <x:row r="10" ht="84" hidden="0" customHeight="1">
+    <x:row r="10" ht="72" hidden="0" customHeight="1">
       <x:c r="A10" s="66" t="str">
-        <x:v>ADIF field preservation</x:v>
+        <x:v>QSO data quality findings</x:v>
       </x:c>
       <x:c r="B10" s="67" t="str">
-        <x:v>Source complete for seven reviewed compatibility stages — local records retain a JSON field bag; unknown/custom fields, Unicode, station/contact and RX/TX data survive supported ADI/ADX round trips. UTF-8 byte scanning, FT4/FT2/JTTY MFSK-submode export, C4FM/DSTAR DIGITALVOICE-submode handling and import-only PSK31/PSK63/PSK63F to PSK/submode normalization are fixed. Latest Swift 18/18 and frontend 1,170/1,170 pass (CLI-timeout-only retry); current-source TypeScript passes. Remaining 3.1.8 audit and package/real-log acceptance stay open; ADIF_VER stays 3.1.7.</x:v>
+        <x:v>Source complete for read-only core — QSODataQuality inspects one retained revision using existing validation, supplied dated CTY comparison at QSO date, retained power provenance and exact-context conflict alternatives (5d11996; 5/5 Swift). Stored/manual overrides stay authoritative. Dates retain source/observation/detection roles rather than field origin. Findings supply qualitative impacts only, no correction or award/confirmation/sync delta. Route/UI, corrections and package/copied-log/live acceptance remain open.</x:v>
       </x:c>
       <x:c r="C10" s="67" t="str">
-        <x:v>Documented — import/export plus four user-definable logging fields.</x:v>
+        <x:v>Documented — QSO editing and DXCC/QSL workflows; comparable field-provenance findings were not established.</x:v>
       </x:c>
       <x:c r="D10" s="67" t="str">
-        <x:v>Documented — ADIF-oriented logbook and online-service interchange; unknown-field preservation was not established in the reviewed README.</x:v>
+        <x:v>Documented — log management and service reconciliation; comparable field-provenance findings were not established.</x:v>
       </x:c>
       <x:c r="E10" s="59"/>
       <x:c r="F10" s="59"/>
     </x:row>
-    <x:row r="11" ht="24" hidden="0" customHeight="1">
+    <x:row r="11" ht="84" hidden="0" customHeight="1">
       <x:c r="A11" s="66" t="str">
-        <x:v>ADIF import — duplicate/update review</x:v>
+        <x:v>ADIF field preservation</x:v>
       </x:c>
       <x:c r="B11" s="67" t="str">
-        <x:v>Source complete — bounded ADI/ADX preview, invalid-record reporting, explicit insert/duplicate counts and revision-fenced field update choices.</x:v>
+        <x:v>Source complete for eight reviewed compatibility stages — local records retain a JSON field bag; unknown/custom fields, Unicode, station/contact and RX/TX data survive supported ADI/ADX round trips. UTF-8 byte scanning, FT4/FT2/JTTY MFSK-submode export, C4FM/DSTAR DIGITALVOICE-submode handling and import-only PSK31/PSK63/PSK63F/PSK125 to PSK/submode normalization are fixed. Latest Swift 18/18 and frontend 1,186/1,186 and TypeScript pass at PSK125 (6253f8f). Remaining 3.1.8 audit and package/real-log acceptance stay open; ADIF_VER stays 3.1.7.</x:v>
       </x:c>
       <x:c r="C11" s="67" t="str">
-        <x:v>Documented — ADIF import and exchange with other logging tools.</x:v>
+        <x:v>Documented — import/export plus four user-definable logging fields.</x:v>
       </x:c>
       <x:c r="D11" s="67" t="str">
-        <x:v>Documented — import and service reconciliation are present; exact duplicate/update review behavior was not established in the reviewed README.</x:v>
+        <x:v>Documented — ADIF-oriented logbook and online-service interchange; unknown-field preservation was not established in the reviewed README.</x:v>
       </x:c>
       <x:c r="E11" s="59"/>
       <x:c r="F11" s="59"/>
     </x:row>
     <x:row r="12" ht="24" hidden="0" customHeight="1">
       <x:c r="A12" s="66" t="str">
-        <x:v>ADIF export — all, filtered and selected</x:v>
+        <x:v>ADIF import — duplicate/update review</x:v>
       </x:c>
       <x:c r="B12" s="67" t="str">
-        <x:v>Source complete — freezes a consistent all/filtered/selected snapshot before paged ADI or ADX export.</x:v>
+        <x:v>Source complete — bounded ADI/ADX preview, invalid-record reporting, explicit insert/duplicate counts and revision-fenced field update choices.</x:v>
       </x:c>
       <x:c r="C12" s="67" t="str">
-        <x:v>Documented — quick/detailed queries and export routines.</x:v>
+        <x:v>Documented — ADIF import and exchange with other logging tools.</x:v>
       </x:c>
       <x:c r="D12" s="67" t="str">
-        <x:v>Documented — log and service integrations imply interchange; exact selected/filtered export behavior was not established in the reviewed README.</x:v>
+        <x:v>Documented — import and service reconciliation are present; exact duplicate/update review behavior was not established in the reviewed README.</x:v>
       </x:c>
       <x:c r="E12" s="59"/>
       <x:c r="F12" s="59"/>
     </x:row>
     <x:row r="13" ht="24" hidden="0" customHeight="1">
       <x:c r="A13" s="66" t="str">
-        <x:v>Logbook table — selectable columns</x:v>
+        <x:v>ADIF export — all, filtered and selected</x:v>
       </x:c>
       <x:c r="B13" s="67" t="str">
-        <x:v>Source complete — normal Logbook columns are available in dedicated, detached and map-split views with separate visibility preferences.</x:v>
+        <x:v>Source complete — freezes a consistent all/filtered/selected snapshot before paged ADI or ADX export.</x:v>
       </x:c>
       <x:c r="C13" s="67" t="str">
-        <x:v>Documented / locally observed — configurable Logbook columns and table sizing.</x:v>
+        <x:v>Documented — quick/detailed queries and export routines.</x:v>
       </x:c>
       <x:c r="D13" s="67" t="str">
-        <x:v>Documented — customizable GUI and saved table state patterns.</x:v>
+        <x:v>Documented — log and service integrations imply interchange; exact selected/filtered export behavior was not established in the reviewed README.</x:v>
       </x:c>
       <x:c r="E13" s="59"/>
       <x:c r="F13" s="59"/>
     </x:row>
     <x:row r="14" ht="24" hidden="0" customHeight="1">
       <x:c r="A14" s="66" t="str">
-        <x:v>Logbook table — adjustable column widths</x:v>
+        <x:v>Logbook table — selectable columns</x:v>
       </x:c>
       <x:c r="B14" s="67" t="str">
-        <x:v>Source complete — bounded pointer, keyboard and numeric width controls persist per presentation context; packaged follow-up acceptance remains open.</x:v>
+        <x:v>Source complete — normal Logbook columns are available in dedicated, detached and map-split views with separate visibility preferences.</x:v>
       </x:c>
       <x:c r="C14" s="67" t="str">
-        <x:v>Documented / locally observed — adjustable table columns.</x:v>
+        <x:v>Documented / locally observed — configurable Logbook columns and table sizing.</x:v>
       </x:c>
       <x:c r="D14" s="67" t="str">
-        <x:v>Documented — movable/visible columns are used in QLog tables; exact persistence varies by view.</x:v>
+        <x:v>Documented — customizable GUI and saved table state patterns.</x:v>
       </x:c>
       <x:c r="E14" s="59"/>
       <x:c r="F14" s="59"/>
     </x:row>
-    <x:row r="15" ht="48" hidden="0" customHeight="1">
+    <x:row r="15" ht="24" hidden="0" customHeight="1">
       <x:c r="A15" s="66" t="str">
-        <x:v>Previous QSOs — independent window</x:v>
+        <x:v>Logbook table — adjustable column widths</x:v>
       </x:c>
       <x:c r="B15" s="67" t="str">
-        <x:v>Source and synthetic visual stage complete — a native Window-menu surface follows the canonical Log QSO draft and existing local-history projection, closes on Canvas transition, and adds no contact owner. Focused frontend/Rust/build checks and 320/420/900-pixel visual checks pass; exact packaged native acceptance remains.</x:v>
+        <x:v>Source complete — bounded pointer, keyboard and numeric width controls persist per presentation context; packaged follow-up acceptance remains open.</x:v>
       </x:c>
       <x:c r="C15" s="67" t="str">
-        <x:v>Documented — QSO search and entity/QSO search windows.</x:v>
+        <x:v>Documented / locally observed — adjustable table columns.</x:v>
       </x:c>
       <x:c r="D15" s="67" t="str">
-        <x:v>Not established in reviewed evidence as a dedicated independent window.</x:v>
+        <x:v>Documented — movable/visible columns are used in QLog tables; exact persistence varies by view.</x:v>
       </x:c>
       <x:c r="E15" s="59"/>
       <x:c r="F15" s="59"/>
     </x:row>
-    <x:row r="16" ht="60" hidden="0" customHeight="1">
+    <x:row r="16" ht="48" hidden="0" customHeight="1">
       <x:c r="A16" s="66" t="str">
-        <x:v>Callsign and DXCC intelligence</x:v>
+        <x:v>Previous QSOs — independent window</x:v>
       </x:c>
       <x:c r="B16" s="67" t="str">
-        <x:v>Source complete — dedicated/detached panel with QRZ enrichment, date-aware CTY/DXCC classification, grids, zones, distance and worked/confirmed matrices. The incorrect all-PJ-to-305 shortcut is removed, stored DXCC overrides remain authoritative, and a bounded read-only Logbook preview explains inferred PJ changes without a correction route. Exact-package/copied-log acceptance remains open.</x:v>
+        <x:v>Source and synthetic visual stage complete — a native Window-menu surface follows the canonical Log QSO draft and existing local-history projection, closes on Canvas transition, and adds no contact owner. Focused frontend/Rust/build checks and 320/420/900-pixel visual checks pass; exact packaged native acceptance remains.</x:v>
       </x:c>
       <x:c r="C16" s="67" t="str">
-        <x:v>Documented — QRZ/HamQTH lookups, Club Log DXCC recognition and detailed DXCC status.</x:v>
+        <x:v>Documented — QSO search and entity/QSO search windows.</x:v>
       </x:c>
       <x:c r="D16" s="67" t="str">
-        <x:v>Documented — QRZ.com and HamQTH callbook integration plus club-member lookup.</x:v>
+        <x:v>Not established in reviewed evidence as a dedicated independent window.</x:v>
       </x:c>
       <x:c r="E16" s="59"/>
       <x:c r="F16" s="59"/>
     </x:row>
     <x:row r="17" ht="60" hidden="0" customHeight="1">
       <x:c r="A17" s="66" t="str">
-        <x:v>Operating goals and opportunity context</x:v>
+        <x:v>Callsign and DXCC intelligence</x:v>
       </x:c>
       <x:c r="B17" s="67" t="str">
-        <x:v>Passive source window complete — explicit callsign, entity/band/mode and IOTA/POTA/SOTA/WWFF targets are evaluated against station-scoped retained history and official opportunities. The native window keeps selection ephemeral and separates worked, confirmed, sponsor evidence and sponsor credit while showing source age/time basis. Cluster observations are explicitly excluded; package acceptance and opt-in reminders remain open.</x:v>
+        <x:v>Source complete — dedicated/detached panel with QRZ enrichment, date-aware CTY/DXCC classification, grids, zones, distance and worked/confirmed matrices. The incorrect all-PJ-to-305 shortcut is removed, stored DXCC overrides remain authoritative, and a bounded read-only Logbook preview explains inferred PJ changes without a correction route. Exact-package/copied-log acceptance remains open.</x:v>
       </x:c>
       <x:c r="C17" s="67" t="str">
-        <x:v>Documented — DX-alarm, band-map and award-status workflows; the reviewed evidence did not establish the same shared goal model.</x:v>
+        <x:v>Documented — QRZ/HamQTH lookups, Club Log DXCC recognition and detailed DXCC status.</x:v>
       </x:c>
       <x:c r="D17" s="67" t="str">
-        <x:v>Documented — alerts, custom filters and award tracking; the reviewed evidence did not establish the same shared goal model.</x:v>
+        <x:v>Documented — QRZ.com and HamQTH callbook integration plus club-member lookup.</x:v>
       </x:c>
       <x:c r="E17" s="59"/>
       <x:c r="F17" s="59"/>
     </x:row>
-    <x:row r="18" ht="72" hidden="0" customHeight="1">
+    <x:row r="18" ht="60" hidden="0" customHeight="1">
       <x:c r="A18" s="66" t="str">
-        <x:v>Connection Doctor and support preview</x:v>
+        <x:v>Operating goals and opportunity context</x:v>
       </x:c>
       <x:c r="B18" s="67" t="str">
-        <x:v>Passive native window plus click-only redacted export source complete — fixed provider/configuration/connection/freshness/capability stages consume only already-retained allowlisted state. The typed preview and exported JSON cannot represent secrets, endpoints, identifiers, raw errors, radio values, timestamps or log contents. The former late-CSS bundle gate is fixed; exact-package Save/Cancel/overwrite and retained-provider acceptance remain open.</x:v>
+        <x:v>Passive source window complete — explicit callsign, entity/band/mode and IOTA/POTA/SOTA/WWFF targets are evaluated against station-scoped retained history and official opportunities. The native window keeps selection ephemeral and separates worked, confirmed, sponsor evidence and sponsor credit while showing source age/time basis. Cluster observations are explicitly excluded; package acceptance and opt-in reminders remain open.</x:v>
       </x:c>
       <x:c r="C18" s="67" t="str">
-        <x:v>Not established as a comparable product surface in reviewed primary evidence.</x:v>
+        <x:v>Documented — DX-alarm, band-map and award-status workflows; the reviewed evidence did not establish the same shared goal model.</x:v>
       </x:c>
       <x:c r="D18" s="67" t="str">
-        <x:v>Not established as a comparable product surface in reviewed primary evidence.</x:v>
+        <x:v>Documented — alerts, custom filters and award tracking; the reviewed evidence did not establish the same shared goal model.</x:v>
       </x:c>
       <x:c r="E18" s="59"/>
       <x:c r="F18" s="59"/>
     </x:row>
-    <x:row r="19" ht="24" hidden="0" customHeight="1">
+    <x:row r="19" ht="72" hidden="0" customHeight="1">
       <x:c r="A19" s="66" t="str">
-        <x:v>Wavelog two-way reconciliation</x:v>
+        <x:v>Connection Doctor and support preview</x:v>
       </x:c>
       <x:c r="B19" s="67" t="str">
-        <x:v>Installed / live accepted — read-first reconciliation imported safe contacts and refreshed linked confirmations/enrichment without deleting or overwriting ambiguous records.</x:v>
+        <x:v>Passive native window plus click-only redacted export source complete — fixed provider/configuration/connection/freshness/capability stages consume only already-retained allowlisted state. The typed preview and exported JSON cannot represent secrets, endpoints, identifiers, raw errors, radio values, timestamps or log contents. The former late-CSS bundle gate is fixed; exact-package Save/Cancel/overwrite and retained-provider acceptance remain open.</x:v>
       </x:c>
       <x:c r="C19" s="67" t="str">
-        <x:v>Not documented as a native Wavelog workflow in reviewed primary evidence.</x:v>
+        <x:v>Not established as a comparable product surface in reviewed primary evidence.</x:v>
       </x:c>
       <x:c r="D19" s="67" t="str">
-        <x:v>Documented — Cloudlog/Wavelog integration.</x:v>
+        <x:v>Not established as a comparable product surface in reviewed primary evidence.</x:v>
       </x:c>
       <x:c r="E19" s="59"/>
       <x:c r="F19" s="59"/>
     </x:row>
     <x:row r="20" ht="24" hidden="0" customHeight="1">
       <x:c r="A20" s="66" t="str">
-        <x:v>Confirmation refresh from remote services</x:v>
+        <x:v>Wavelog two-way reconciliation</x:v>
       </x:c>
       <x:c r="B20" s="67" t="str">
-        <x:v>Installed / live accepted through Wavelog — LoTW, eQSL, QRZ and enrichment changes update matching local QSOs while ambiguous identities remain held for review.</x:v>
+        <x:v>Installed / live accepted — read-first reconciliation imported safe contacts and refreshed linked confirmations/enrichment without deleting or overwriting ambiguous records.</x:v>
       </x:c>
       <x:c r="C20" s="67" t="str">
-        <x:v>Documented — direct LoTW/eQSL workflows and Club Log real-time synchronization.</x:v>
+        <x:v>Not documented as a native Wavelog workflow in reviewed primary evidence.</x:v>
       </x:c>
       <x:c r="D20" s="67" t="str">
-        <x:v>Documented — LoTW, eQSL, QRZ.com, Club Log, HRDLog.net and Cloudlog/Wavelog integrations.</x:v>
+        <x:v>Documented — Cloudlog/Wavelog integration.</x:v>
       </x:c>
       <x:c r="E20" s="59"/>
       <x:c r="F20" s="59"/>
     </x:row>
     <x:row r="21" ht="24" hidden="0" customHeight="1">
       <x:c r="A21" s="66" t="str">
-        <x:v>QRZ.com callbook lookup</x:v>
+        <x:v>Confirmation refresh from remote services</x:v>
       </x:c>
       <x:c r="B21" s="67" t="str">
-        <x:v>Partial — Keychain-backed live lookup, operator-edit preservation and precise-grid targeting exist; cache/session/privacy controls remain.</x:v>
+        <x:v>Installed / live accepted through Wavelog — LoTW, eQSL, QRZ and enrichment changes update matching local QSOs while ambiguous identities remain held for review.</x:v>
       </x:c>
       <x:c r="C21" s="67" t="str">
-        <x:v>Documented — QRZ.com and other online directory queries.</x:v>
+        <x:v>Documented — direct LoTW/eQSL workflows and Club Log real-time synchronization.</x:v>
       </x:c>
       <x:c r="D21" s="67" t="str">
-        <x:v>Documented — QRZ.com callbook integration.</x:v>
+        <x:v>Documented — LoTW, eQSL, QRZ.com, Club Log, HRDLog.net and Cloudlog/Wavelog integrations.</x:v>
       </x:c>
       <x:c r="E21" s="59"/>
       <x:c r="F21" s="59"/>
     </x:row>
     <x:row r="22" ht="24" hidden="0" customHeight="1">
       <x:c r="A22" s="66" t="str">
-        <x:v>QRZ.com log upload</x:v>
+        <x:v>QRZ.com callbook lookup</x:v>
       </x:c>
       <x:c r="B22" s="67" t="str">
-        <x:v>Source complete — prospective default-off upload owner with vault credentials, exact claims, durable receipts and no ambiguous replay; live account acceptance open.</x:v>
+        <x:v>Partial — Keychain-backed live lookup, operator-edit preservation and precise-grid targeting exist; cache/session/privacy controls remain.</x:v>
       </x:c>
       <x:c r="C22" s="67" t="str">
-        <x:v>Documented via the separate real-time upload utility.</x:v>
+        <x:v>Documented — QRZ.com and other online directory queries.</x:v>
       </x:c>
       <x:c r="D22" s="67" t="str">
-        <x:v>Documented — QRZ.com online-log integration.</x:v>
+        <x:v>Documented — QRZ.com callbook integration.</x:v>
       </x:c>
       <x:c r="E22" s="59"/>
       <x:c r="F22" s="59"/>
     </x:row>
     <x:row r="23" ht="24" hidden="0" customHeight="1">
       <x:c r="A23" s="66" t="str">
-        <x:v>Club Log upload/sync</x:v>
+        <x:v>QRZ.com log upload</x:v>
       </x:c>
       <x:c r="B23" s="67" t="str">
-        <x:v>Source complete for prospective upload; installed Wavelog reconciliation also receives Club Log-related log state. Direct live account acceptance remains open.</x:v>
+        <x:v>Source complete — prospective default-off upload owner with vault credentials, exact claims, durable receipts and no ambiguous replay; live account acceptance open.</x:v>
       </x:c>
       <x:c r="C23" s="67" t="str">
-        <x:v>Documented — real-time Club Log synchronization.</x:v>
+        <x:v>Documented via the separate real-time upload utility.</x:v>
       </x:c>
       <x:c r="D23" s="67" t="str">
-        <x:v>Documented — Club Log integration.</x:v>
+        <x:v>Documented — QRZ.com online-log integration.</x:v>
       </x:c>
       <x:c r="E23" s="59"/>
       <x:c r="F23" s="59"/>
     </x:row>
-    <x:row r="24" ht="84" hidden="0" customHeight="1">
+    <x:row r="24" ht="24" hidden="0" customHeight="1">
       <x:c r="A24" s="66" t="str">
-        <x:v>Online-log follow-up evidence</x:v>
+        <x:v>Club Log upload/sync</x:v>
       </x:c>
       <x:c r="B24" s="67" t="str">
-        <x:v>Source and browser verified — generation-fenced local route and Logbook row panel expose canonical QRZ/Club Log delivery state, receipt revision and attempt age, separately from retained paper/LoTW/eQSL confirmations. Opening performs no fetch; explicit Refresh reads local evidence, and Close/context changes retire pending reads. Swift route 1/1, Rust permission 1/1, frontend 31/31, TypeScript/build/bundle gates and 640x480/1280x800 actual-Logbook browser checks pass. Provider acceptance/match age and sponsor credit remain unknown; exact-package/native and live-account acceptance remain open.</x:v>
+        <x:v>Source complete for prospective upload; installed Wavelog reconciliation also receives Club Log-related log state. Direct live account acceptance remains open.</x:v>
       </x:c>
       <x:c r="C24" s="67" t="str">
-        <x:v>Documented service status and confirmation workflows; exact evidence boundaries were not audited.</x:v>
+        <x:v>Documented — real-time Club Log synchronization.</x:v>
       </x:c>
       <x:c r="D24" s="67" t="str">
-        <x:v>Documented online-log integrations; exact evidence boundaries were not audited.</x:v>
+        <x:v>Documented — Club Log integration.</x:v>
       </x:c>
       <x:c r="E24" s="59"/>
       <x:c r="F24" s="59"/>
     </x:row>
-    <x:row r="25" ht="24" hidden="0" customHeight="1">
+    <x:row r="25" ht="84" hidden="0" customHeight="1">
       <x:c r="A25" s="66" t="str">
-        <x:v>HRDLog.net upload</x:v>
+        <x:v>Online-log follow-up evidence</x:v>
       </x:c>
       <x:c r="B25" s="67" t="str">
-        <x:v>Outstanding — deferred until the current official service contract is verified and implemented behind the same vault/receipt/no-replay boundary.</x:v>
+        <x:v>Source and browser verified — generation-fenced local route and Logbook row panel expose canonical QRZ/Club Log delivery state, receipt revision and attempt age, separately from retained paper/LoTW/eQSL confirmations. Opening performs no fetch; explicit Refresh reads local evidence, and Close/context changes retire pending reads. Swift route 1/1, Rust permission 1/1, frontend 31/31, TypeScript/build/bundle gates and 640x480/1280x800 actual-Logbook browser checks pass. Provider acceptance/match age and sponsor credit remain unknown; exact-package/native and live-account acceptance remain open.</x:v>
       </x:c>
       <x:c r="C25" s="67" t="str">
-        <x:v>Documented via the separate real-time upload utility.</x:v>
+        <x:v>Documented service status and confirmation workflows; exact evidence boundaries were not audited.</x:v>
       </x:c>
       <x:c r="D25" s="67" t="str">
-        <x:v>Documented — HRDLog.net integration.</x:v>
+        <x:v>Documented online-log integrations; exact evidence boundaries were not audited.</x:v>
       </x:c>
       <x:c r="E25" s="59"/>
       <x:c r="F25" s="59"/>
     </x:row>
     <x:row r="26" ht="24" hidden="0" customHeight="1">
       <x:c r="A26" s="66" t="str">
-        <x:v>Direct LoTW and eQSL workflows</x:v>
+        <x:v>HRDLog.net upload</x:v>
       </x:c>
       <x:c r="B26" s="67" t="str">
-        <x:v>Outstanding as independent providers — confirmation fields and Wavelog refresh are supported, but direct credential/upload/download owners remain separate programmes.</x:v>
+        <x:v>Outstanding — deferred until the current official service contract is verified and implemented behind the same vault/receipt/no-replay boundary.</x:v>
       </x:c>
       <x:c r="C26" s="67" t="str">
-        <x:v>Documented — direct upload/download, QSL statistics and paper-QSL workflows.</x:v>
+        <x:v>Documented via the separate real-time upload utility.</x:v>
       </x:c>
       <x:c r="D26" s="67" t="str">
-        <x:v>Documented — LoTW and eQSL integration; TQSL is optional for LoTW and eQSL can download QSL pictures.</x:v>
+        <x:v>Documented — HRDLog.net integration.</x:v>
       </x:c>
       <x:c r="E26" s="59"/>
       <x:c r="F26" s="59"/>
     </x:row>
     <x:row r="27" ht="24" hidden="0" customHeight="1">
       <x:c r="A27" s="66" t="str">
-        <x:v>WSJT-X Logged ADIF UDP intake</x:v>
+        <x:v>Direct LoTW and eQSL workflows</x:v>
       </x:c>
       <x:c r="B27" s="67" t="str">
-        <x:v>Source complete — explicit default-off receive-only listener for official Logged ADIF messages; loopback/multicast validation and duplicate-safe local save; live WSJT-X acceptance open.</x:v>
+        <x:v>Outstanding as independent providers — confirmation fields and Wavelog refresh are supported, but direct credential/upload/download owners remain separate programmes.</x:v>
       </x:c>
       <x:c r="C27" s="67" t="str">
-        <x:v>Documented / locally inventoried — configurable WSJT-X UDP logging and save choices.</x:v>
+        <x:v>Documented — direct upload/download, QSL statistics and paper-QSL workflows.</x:v>
       </x:c>
       <x:c r="D27" s="67" t="str">
-        <x:v>Documented — WSJT-X integration; source audit shows one configurable unicast/multicast receiver and QSO Logged/Logged ADIF parsing.</x:v>
+        <x:v>Documented — LoTW and eQSL integration; TQSL is optional for LoTW and eQSL can download QSL pictures.</x:v>
       </x:c>
       <x:c r="E27" s="59"/>
       <x:c r="F27" s="59"/>
     </x:row>
     <x:row r="28" ht="24" hidden="0" customHeight="1">
       <x:c r="A28" s="66" t="str">
-        <x:v>WSJT-X CQ activity and novelty</x:v>
+        <x:v>WSJT-X Logged ADIF UDP intake</x:v>
       </x:c>
       <x:c r="B28" s="67" t="str">
-        <x:v>Source complete — bounded receive-only FT8/FT4 CQ activity feeds named alerts with current local call/DXCC novelty; no reply, CAT, PTT or save authority.</x:v>
+        <x:v>Source complete — explicit default-off receive-only listener for official Logged ADIF messages; loopback/multicast validation and duplicate-safe local save; live WSJT-X acceptance open.</x:v>
       </x:c>
       <x:c r="C28" s="67" t="str">
-        <x:v>Documented / locally inventoried — WSJT-X activity-window and callsign-checking choices.</x:v>
+        <x:v>Documented / locally inventoried — configurable WSJT-X UDP logging and save choices.</x:v>
       </x:c>
       <x:c r="D28" s="67" t="str">
-        <x:v>Documented — WSJT-X activity can feed its alert evaluator.</x:v>
+        <x:v>Documented — WSJT-X integration; source audit shows one configurable unicast/multicast receiver and QSO Logged/Logged ADIF parsing.</x:v>
       </x:c>
       <x:c r="E28" s="59"/>
       <x:c r="F28" s="59"/>
     </x:row>
     <x:row r="29" ht="24" hidden="0" customHeight="1">
       <x:c r="A29" s="66" t="str">
-        <x:v>DX Cluster</x:v>
+        <x:v>WSJT-X CQ activity and novelty</x:v>
       </x:c>
       <x:c r="B29" s="67" t="str">
-        <x:v>Implemented — native shared cluster owner, profiles, filters, console paths and retained spot state; configuration and display remain separated.</x:v>
+        <x:v>Source complete — bounded receive-only FT8/FT4 CQ activity feeds named alerts with current local call/DXCC novelty; no reply, CAT, PTT or save authority.</x:v>
       </x:c>
       <x:c r="C29" s="67" t="str">
-        <x:v>Documented — internet/local-skimmer cluster, terminal and separated/alerted spots.</x:v>
+        <x:v>Documented / locally inventoried — WSJT-X activity-window and callsign-checking choices.</x:v>
       </x:c>
       <x:c r="D29" s="67" t="str">
-        <x:v>Documented — DX cluster integration.</x:v>
+        <x:v>Documented — WSJT-X activity can feed its alert evaluator.</x:v>
       </x:c>
       <x:c r="E29" s="59"/>
       <x:c r="F29" s="59"/>
     </x:row>
     <x:row r="30" ht="24" hidden="0" customHeight="1">
       <x:c r="A30" s="66" t="str">
-        <x:v>Spot History</x:v>
+        <x:v>DX Cluster</x:v>
       </x:c>
       <x:c r="B30" s="67" t="str">
-        <x:v>Source complete — separate retained local reports, search/filter/statistics and read-only review. Detached column controls exist; packaged/live retention acceptance remains open.</x:v>
+        <x:v>Implemented — native shared cluster owner, profiles, filters, console paths and retained spot state; configuration and display remain separated.</x:v>
       </x:c>
       <x:c r="C30" s="67" t="str">
-        <x:v>Documented — incoming cluster data and spot/search workflows; exact retained-history model differs.</x:v>
+        <x:v>Documented — internet/local-skimmer cluster, terminal and separated/alerted spots.</x:v>
       </x:c>
       <x:c r="D30" s="67" t="str">
-        <x:v>Documented alert/history tables; exact long-term raw report retention was not established in the reviewed README.</x:v>
+        <x:v>Documented — DX cluster integration.</x:v>
       </x:c>
       <x:c r="E30" s="59"/>
       <x:c r="F30" s="59"/>
     </x:row>
-    <x:row r="31" ht="48" hidden="0" customHeight="1">
+    <x:row r="31" ht="24" hidden="0" customHeight="1">
       <x:c r="A31" s="66" t="str">
-        <x:v>Named DX/WSJT-X alert rules</x:v>
+        <x:v>Spot History</x:v>
       </x:c>
       <x:c r="B31" s="67" t="str">
-        <x:v>Source complete — independently enabled structured rules, all matching names, bounded dedup/rate limiting and passive recent-alert dashboard. Each retained event explains its call/DXCC/band/mode/special evidence and first-to-last report history; compact windows use cards instead of horizontal scrolling.</x:v>
+        <x:v>Source complete — separate retained local reports, search/filter/statistics and read-only review. Detached column controls exist; packaged/live retention acceptance remains open.</x:v>
       </x:c>
       <x:c r="C31" s="67" t="str">
-        <x:v>Documented — DXCC/band/mode/IOTA novelty, confirmation source choices, wildcard station watches and optional spoken delivery.</x:v>
+        <x:v>Documented — incoming cluster data and spot/search workflows; exact retained-history model differs.</x:v>
       </x:c>
       <x:c r="D31" s="67" t="str">
-        <x:v>Documented — named cloneable rules combining source, callsign, entity, novelty, geography, comment, band, mode, memberships and activity references.</x:v>
+        <x:v>Documented alert/history tables; exact long-term raw report retention was not established in the reviewed README.</x:v>
       </x:c>
       <x:c r="E31" s="59"/>
       <x:c r="F31" s="59"/>
     </x:row>
-    <x:row r="32" ht="24" hidden="0" customHeight="1">
+    <x:row r="32" ht="48" hidden="0" customHeight="1">
       <x:c r="A32" s="66" t="str">
-        <x:v>Alert delivery without RF authority</x:v>
+        <x:v>Named DX/WSJT-X alert rules</x:v>
       </x:c>
       <x:c r="B32" s="67" t="str">
-        <x:v>Source complete — native default-off popup plus optional sound, no action button or station authority; installed live-cluster popup/sound acceptance open.</x:v>
+        <x:v>Source complete — independently enabled structured rules, all matching names, bounded dedup/rate limiting and passive recent-alert dashboard. Each retained event explains its call/DXCC/band/mode/special evidence and first-to-last report history; compact windows use cards instead of horizontal scrolling.</x:v>
       </x:c>
       <x:c r="C32" s="67" t="str">
-        <x:v>Documented — color-only or opt-in spoken alarm delivery.</x:v>
+        <x:v>Documented — DXCC/band/mode/IOTA novelty, confirmation source choices, wildcard station watches and optional spoken delivery.</x:v>
       </x:c>
       <x:c r="D32" s="67" t="str">
-        <x:v>Documented — optional bell and outbound UDP; QLog may also tune/reply from alert UI, which OM0RX-xLog intentionally does not copy.</x:v>
+        <x:v>Documented — named cloneable rules combining source, callsign, entity, novelty, geography, comment, band, mode, memberships and activity references.</x:v>
       </x:c>
       <x:c r="E32" s="59"/>
       <x:c r="F32" s="59"/>
     </x:row>
     <x:row r="33" ht="24" hidden="0" customHeight="1">
       <x:c r="A33" s="66" t="str">
-        <x:v>World map and grayline</x:v>
+        <x:v>Alert delivery without RF authority</x:v>
       </x:c>
       <x:c r="B33" s="67" t="str">
-        <x:v>Implemented — online hybrid/satellite/standard map, spot and DXCC layers, route/grayline/sun overlays and semantic labels; prolonged operator observation remains.</x:v>
+        <x:v>Source complete — native default-off popup plus optional sound, no action button or station authority; installed live-cluster popup/sound acceptance open.</x:v>
       </x:c>
       <x:c r="C33" s="67" t="str">
-        <x:v>Documented — maps/grayline and DXCC/spot workflows.</x:v>
+        <x:v>Documented — color-only or opt-in spoken alarm delivery.</x:v>
       </x:c>
       <x:c r="D33" s="67" t="str">
-        <x:v>Documented — online and offline map.</x:v>
+        <x:v>Documented — optional bell and outbound UDP; QLog may also tune/reply from alert UI, which OM0RX-xLog intentionally does not copy.</x:v>
       </x:c>
       <x:c r="E33" s="59"/>
       <x:c r="F33" s="59"/>
     </x:row>
     <x:row r="34" ht="24" hidden="0" customHeight="1">
       <x:c r="A34" s="66" t="str">
-        <x:v>Band maps</x:v>
+        <x:v>World map and grayline</x:v>
       </x:c>
       <x:c r="B34" s="67" t="str">
-        <x:v>Implemented — multiple independently keyed band maps, follow-radio behavior and detached windows; final mixed-size/multi-display packaged acceptance remains.</x:v>
+        <x:v>Implemented — online hybrid/satellite/standard map, spot and DXCC layers, route/grayline/sun overlays and semantic labels; prolonged operator observation remains.</x:v>
       </x:c>
       <x:c r="C34" s="67" t="str">
-        <x:v>Documented / locally observed — multiple independent band-map windows.</x:v>
+        <x:v>Documented — maps/grayline and DXCC/spot workflows.</x:v>
       </x:c>
       <x:c r="D34" s="67" t="str">
-        <x:v>Documented — bandmap.</x:v>
+        <x:v>Documented — online and offline map.</x:v>
       </x:c>
       <x:c r="E34" s="59"/>
       <x:c r="F34" s="59"/>
     </x:row>
-    <x:row r="35" ht="36" hidden="0" customHeight="1">
+    <x:row r="35" ht="24" hidden="0" customHeight="1">
       <x:c r="A35" s="66" t="str">
-        <x:v>Canvas and separate-window modes</x:v>
+        <x:v>Band maps</x:v>
       </x:c>
       <x:c r="B35" s="67" t="str">
-        <x:v>Source complete — persistent Canvas/Separate Windows choice, named native task windows and geometry recovery. Switching to Canvas closes child windows; simultaneous multi-display packaged acceptance remains.</x:v>
+        <x:v>Implemented — multiple independently keyed band maps, follow-radio behavior and detached windows; final mixed-size/multi-display packaged acceptance remains.</x:v>
       </x:c>
       <x:c r="C35" s="67" t="str">
-        <x:v>Documented / locally observed — many named native windows with saved placement conventions.</x:v>
+        <x:v>Documented / locally observed — multiple independent band-map windows.</x:v>
       </x:c>
       <x:c r="D35" s="67" t="str">
-        <x:v>Documented — customizable GUI and saved layout profiles; macOS is experimental.</x:v>
+        <x:v>Documented — bandmap.</x:v>
       </x:c>
       <x:c r="E35" s="59"/>
       <x:c r="F35" s="59"/>
     </x:row>
-    <x:row r="36" ht="60" hidden="0" customHeight="1">
+    <x:row r="36" ht="36" hidden="0" customHeight="1">
       <x:c r="A36" s="66" t="str">
-        <x:v>Responsive detached windows</x:v>
+        <x:v>Canvas and separate-window modes</x:v>
       </x:c>
       <x:c r="B36" s="67" t="str">
-        <x:v>Partial — common chrome removal and targeted fixes cover many roles. Detached Propagation rows align; Station Status and Rotor use the shared inset; Rotor starts at the top. Focused 31/31 UI, rendered geometry, Band Map 380×1100, Callsign Intelligence 680×500 and Rotor 676×500/400×600 browser checks pass without page overflow. The packaged all-window resolution/scale matrix remains outstanding.</x:v>
+        <x:v>Source complete — persistent Canvas/Separate Windows choice, named native task windows and geometry recovery. Switching to Canvas closes child windows; simultaneous multi-display packaged acceptance remains.</x:v>
       </x:c>
       <x:c r="C36" s="67" t="str">
-        <x:v>Mature native macOS window behavior is the reference; exact responsive tests were not obtained.</x:v>
+        <x:v>Documented / locally observed — many named native windows with saved placement conventions.</x:v>
       </x:c>
       <x:c r="D36" s="67" t="str">
-        <x:v>Recommended resolution is 1920×1080; cross-platform GUI is customizable, but compact-window behavior was not established.</x:v>
+        <x:v>Documented — customizable GUI and saved layout profiles; macOS is experimental.</x:v>
       </x:c>
       <x:c r="E36" s="59"/>
       <x:c r="F36" s="59"/>
     </x:row>
-    <x:row r="37" ht="24" hidden="0" customHeight="1">
+    <x:row r="37" ht="60" hidden="0" customHeight="1">
       <x:c r="A37" s="66" t="str">
-        <x:v>Custom canvas panel move/resize</x:v>
+        <x:v>Responsive detached windows</x:v>
       </x:c>
       <x:c r="B37" s="67" t="str">
-        <x:v>Source complete for traditional unlock/edit interaction — panel arrow enters edit mode, title drags position and edges/corners resize; broader mixed-size acceptance remains.</x:v>
+        <x:v>Partial — common chrome removal and targeted fixes cover many roles. Detached Propagation rows align; Station Status and Rotor use the shared inset; Rotor starts at the top. Focused 31/31 UI, rendered geometry, Band Map 380×1100, Callsign Intelligence 680×500 and Rotor 676×500/400×600 browser checks pass without page overflow. The packaged all-window resolution/scale matrix remains outstanding.</x:v>
       </x:c>
       <x:c r="C37" s="67" t="str">
-        <x:v>Not a directly comparable canvas workflow in reviewed evidence.</x:v>
+        <x:v>Mature native macOS window behavior is the reference; exact responsive tests were not obtained.</x:v>
       </x:c>
       <x:c r="D37" s="67" t="str">
-        <x:v>Documented saved layout profiles; exact freeform canvas resize interaction differs.</x:v>
+        <x:v>Recommended resolution is 1920×1080; cross-platform GUI is customizable, but compact-window behavior was not established.</x:v>
       </x:c>
       <x:c r="E37" s="59"/>
       <x:c r="F37" s="59"/>
     </x:row>
     <x:row r="38" ht="24" hidden="0" customHeight="1">
       <x:c r="A38" s="66" t="str">
-        <x:v>Radio control providers</x:v>
+        <x:v>Custom canvas panel move/resize</x:v>
       </x:c>
       <x:c r="B38" s="67" t="str">
-        <x:v>Implemented — Remote Agent, direct FLEX LAN and local Hamlib paths are capability-separated with explicit selection/connect and retained observed state.</x:v>
+        <x:v>Source complete for traditional unlock/edit interaction — panel arrow enters edit mode, title drags position and edges/corners resize; broader mixed-size acceptance remains.</x:v>
       </x:c>
       <x:c r="C38" s="67" t="str">
-        <x:v>Documented — Kenwood, Elecraft, Yaesu and Icom support, with deeper controls for selected models.</x:v>
+        <x:v>Not a directly comparable canvas workflow in reviewed evidence.</x:v>
       </x:c>
       <x:c r="D38" s="67" t="str">
-        <x:v>Documented — Hamlib, OmniRig, TCI and FLRig.</x:v>
+        <x:v>Documented saved layout profiles; exact freeform canvas resize interaction differs.</x:v>
       </x:c>
       <x:c r="E38" s="59"/>
       <x:c r="F38" s="59"/>
     </x:row>
-    <x:row r="39" ht="312" hidden="0" customHeight="1">
+    <x:row r="39" ht="24" hidden="0" customHeight="1">
       <x:c r="A39" s="66" t="str">
-        <x:v>TCI rig control — SunSDR/ExpertSDR and compatible servers</x:v>
+        <x:v>Radio control providers</x:v>
       </x:c>
       <x:c r="B39" s="67" t="str">
-        <x:v>Source complete through receive tune/filter, configured-TRX split, global TX-frequency telemetry, APP_FOCUS, addressed RX_CLICKED_ON_SPOT, legacy CLICKED_ON_SPOT and receipt-only CW_MACROS_EMPTY and opaque CALLSIGN_SEND and per-address VFO_LOCK plus RX_CHANNEL_SENSORS and separate deprecated RX_SENSORS token observations. Passive notifications retain independent producer receipts; legacy clicks infer no TRX/channel/VFO. CW_MACROS_EMPTY proves no queue-empty, TX/RX, CW or RF authority. APP_FOCUS Swift 45/45, legacy-click 50/50 (lifecycle rerun) CW receipt 55/55 and CALLSIGN_SEND 60/60 (34 protocol + 26 session) pass. CALLSIGN_SEND uses strict validation/reconnect clearing and confers no target/contact identity authority, command correlation, TX completion/success or RF inference. VFO_LOCK 66/66 (38 protocol + 28 session) retains independent exact-address producer times, validates exactly three arguments within application/discovery bounds, prunes on discovery shrink and clears on reconnect. It grants no owner/expiry, tune confirmation, configured freshness or control authority. RX_CHANNEL_SENSORS preserves exact bounded ASCII decimals per address without Double conversion or physical range/calibration/quality/readiness/freshness/control claims; discovery prunes and reconnect clears. Six new tests pass twice, protocol 42/42; broader session rerun at ed8ed37 was 71/72 on unchanged testDroppingLastSessionReferenceClosesPendingConnection (closeCount 0 vs 1); initial existing tune-yield miss passed rerun. Build/diff clean. 2d7bb1f adds deprecated server-only RX_SENSORS as separate per-TRX raw bounded decimal tokens plus local producer receipt, never channel-attributed or merged with RX_CHANNEL_SENSORS. TRX discovery prunes, channel-count changes do not remap and reconnect clears. No physical range/calibration/readiness/freshness/control/RF inference. Later independent focused tests 78/78 pass; earlier timing miss is not claimed fixed. Explicit controls retain the existing no-replay/readback owner. Transmit/PTT, split/TX-VFO controls, outbound spots, audio/IQ and package/live-server/RF acceptance remain open.</x:v>
+        <x:v>Implemented — Remote Agent, direct FLEX LAN and local Hamlib paths are capability-separated with explicit selection/connect and retained observed state.</x:v>
       </x:c>
       <x:c r="C39" s="67" t="str">
-        <x:v>Not established in the reviewed primary RUMlogNG evidence.</x:v>
+        <x:v>Documented — Kenwood, Elecraft, Yaesu and Icom support, with deeper controls for selected models.</x:v>
       </x:c>
       <x:c r="D39" s="67" t="str">
-        <x:v>Documented — QLog supports all TCI-compatible rigs through its native TCI provider.</x:v>
+        <x:v>Documented — Hamlib, OmniRig, TCI and FLRig.</x:v>
       </x:c>
       <x:c r="E39" s="59"/>
       <x:c r="F39" s="59"/>
     </x:row>
-    <x:row r="40" ht="24" hidden="0" customHeight="1">
+    <x:row r="40" ht="336" hidden="0" customHeight="1">
       <x:c r="A40" s="66" t="str">
-        <x:v>Safe simplex tuning and Tune/Cancel</x:v>
+        <x:v>TCI rig control — SunSDR/ExpertSDR and compatible servers</x:v>
       </x:c>
       <x:c r="B40" s="67" t="str">
-        <x:v>Source complete — durable exact-owner transactions, one existing-worker dispatch, no replay and authoritative readback where available; packaged/hardware acceptance open.</x:v>
+        <x:v>Source complete through receive tune/filter, configured-TRX split, global TX-frequency telemetry, APP_FOCUS, addressed RX_CLICKED_ON_SPOT, legacy CLICKED_ON_SPOT and receipt-only CW_MACROS_EMPTY and opaque CALLSIGN_SEND and per-address VFO_LOCK plus RX_CHANNEL_SENSORS and separate deprecated RX_SENSORS plus formal-five-field TX_SENSORS token observations. Passive notifications retain independent producer receipts; legacy clicks infer no TRX/channel/VFO. CW_MACROS_EMPTY proves no queue-empty, TX/RX, CW or RF authority. APP_FOCUS Swift 45/45, legacy-click 50/50 (lifecycle rerun) CW receipt 55/55 and CALLSIGN_SEND 60/60 (34 protocol + 26 session) pass. CALLSIGN_SEND uses strict validation/reconnect clearing and confers no target/contact identity authority, command correlation, TX completion/success or RF inference. VFO_LOCK 66/66 (38 protocol + 28 session) retains independent exact-address producer times, validates exactly three arguments within application/discovery bounds, prunes on discovery shrink and clears on reconnect. It grants no owner/expiry, tune confirmation, configured freshness or control authority. RX_CHANNEL_SENSORS preserves exact bounded ASCII decimals per address without Double conversion or physical range/calibration/quality/readiness/freshness/control claims; discovery prunes and reconnect clears. Six new tests pass twice, protocol 42/42; broader session rerun at ed8ed37 was 71/72 on unchanged testDroppingLastSessionReferenceClosesPendingConnection (closeCount 0 vs 1); initial existing tune-yield miss passed rerun. Build/diff clean. 2d7bb1f adds deprecated server-only RX_SENSORS as separate per-TRX raw bounded decimal tokens plus local producer receipt, never channel-attributed or merged with RX_CHANNEL_SENSORS. TRX discovery prunes, channel-count changes do not remap and reconnect clears. No physical range/calibration/readiness/freshness/control/RF inference. Later independent focused tests 78/78 pass; earlier timing miss is not claimed fixed. dbf6e36 adds passive formal-five-field TX_SENSORS raw per-TRX receipts (84/84); malformed printed example rejects and no TX/RF/physical power/SWR authority is inferred. Explicit controls retain the existing no-replay/readback owner. Transmit/PTT, split/TX-VFO controls, outbound spots, audio/IQ and package/live-server/RF acceptance remain open.</x:v>
       </x:c>
       <x:c r="C40" s="67" t="str">
-        <x:v>Documented — CAT can set transceiver parameters from the logbook and vice versa; safety contract was not audited.</x:v>
+        <x:v>Not established in the reviewed primary RUMlogNG evidence.</x:v>
       </x:c>
       <x:c r="D40" s="67" t="str">
-        <x:v>Documented — rig control and cluster/bandmap integration; safety contract was not audited.</x:v>
+        <x:v>Documented — QLog supports all TCI-compatible rigs through its native TCI provider.</x:v>
       </x:c>
       <x:c r="E40" s="59"/>
       <x:c r="F40" s="59"/>
     </x:row>
-    <x:row r="41" ht="48" hidden="0" customHeight="1">
+    <x:row r="41" ht="24" hidden="0" customHeight="1">
       <x:c r="A41" s="66" t="str">
-        <x:v>Amplifier Operate/Standby</x:v>
+        <x:v>Safe simplex tuning and Tune/Cancel</x:v>
       </x:c>
       <x:c r="B41" s="67" t="str">
-        <x:v>Source complete — one shared Agent-only durable owner provides separate Operate and urgent Standby lanes, exact identity/freshness fences, one-attempt journal-before-send dispatch and explicit unknown-receipt recovery. Packaged Agent, amplifier-readback, hardware and RF acceptance remain.</x:v>
+        <x:v>Source complete — durable exact-owner transactions, one existing-worker dispatch, no replay and authoritative readback where available; packaged/hardware acceptance open.</x:v>
       </x:c>
       <x:c r="C41" s="67" t="str">
-        <x:v>Model/device controls exist for supported station equipment; exact KPA-style workflow was not established.</x:v>
+        <x:v>Documented — CAT can set transceiver parameters from the logbook and vice versa; safety contract was not audited.</x:v>
       </x:c>
       <x:c r="D41" s="67" t="str">
-        <x:v>No comparable amplifier owner was established in reviewed evidence.</x:v>
+        <x:v>Documented — rig control and cluster/bandmap integration; safety contract was not audited.</x:v>
       </x:c>
       <x:c r="E41" s="59"/>
       <x:c r="F41" s="59"/>
     </x:row>
-    <x:row r="42" ht="24" hidden="0" customHeight="1">
+    <x:row r="42" ht="48" hidden="0" customHeight="1">
       <x:c r="A42" s="66" t="str">
-        <x:v>Rotor control</x:v>
+        <x:v>Amplifier Operate/Standby</x:v>
       </x:c>
       <x:c r="B42" s="67" t="str">
-        <x:v>Source complete — shared manual Goto, native urgent Stop and standalone Auto/Stop with exact owner/generation fences; packaged/hardware acceptance open.</x:v>
+        <x:v>Source complete — one shared Agent-only durable owner provides separate Operate and urgent Standby lanes, exact identity/freshness fences, one-attempt journal-before-send dispatch and explicit unknown-receipt recovery. Packaged Agent, amplifier-readback, hardware and RF acceptance remain.</x:v>
       </x:c>
       <x:c r="C42" s="67" t="str">
-        <x:v>Documented through a companion advanced Rotor application interacting with RUMlogNG and WSJT-X.</x:v>
+        <x:v>Model/device controls exist for supported station equipment; exact KPA-style workflow was not established.</x:v>
       </x:c>
       <x:c r="D42" s="67" t="str">
-        <x:v>Documented — Hamlib and PSTRotator control.</x:v>
+        <x:v>No comparable amplifier owner was established in reviewed evidence.</x:v>
       </x:c>
       <x:c r="E42" s="59"/>
       <x:c r="F42" s="59"/>
     </x:row>
     <x:row r="43" ht="24" hidden="0" customHeight="1">
       <x:c r="A43" s="66" t="str">
-        <x:v>CW keyer and console</x:v>
+        <x:v>Rotor control</x:v>
       </x:c>
       <x:c r="B43" s="67" t="str">
-        <x:v>Implemented foundation — shared saved macros/new-QSO context plus explicit selected-radio and independent WinKeyer ownership; remaining end-to-end hardware acceptance is open.</x:v>
+        <x:v>Source complete — shared manual Goto, native urgent Stop and standalone Auto/Stop with exact owner/generation fences; packaged/hardware acceptance open.</x:v>
       </x:c>
       <x:c r="C43" s="67" t="str">
-        <x:v>Documented — K1EL WinKeyer, CW keyer and RTTY application.</x:v>
+        <x:v>Documented through a companion advanced Rotor application interacting with RUMlogNG and WSJT-X.</x:v>
       </x:c>
       <x:c r="D43" s="67" t="str">
-        <x:v>Documented — CWDaemon, FLDigi, Morse over CAT, WinKey v1/v2 and CW Console.</x:v>
+        <x:v>Documented — Hamlib and PSTRotator control.</x:v>
       </x:c>
       <x:c r="E43" s="59"/>
       <x:c r="F43" s="59"/>
     </x:row>
     <x:row r="44" ht="24" hidden="0" customHeight="1">
       <x:c r="A44" s="66" t="str">
-        <x:v>Propagation display</x:v>
+        <x:v>CW keyer and console</x:v>
       </x:c>
       <x:c r="B44" s="67" t="str">
-        <x:v>Source complete with live provider proof — bounded HamQSL/N0NBH refresh and correct freshness semantics; final packaged outage/freshness observation remains.</x:v>
+        <x:v>Implemented foundation — shared saved macros/new-QSO context plus explicit selected-radio and independent WinKeyer ownership; remaining end-to-end hardware acceptance is open.</x:v>
       </x:c>
       <x:c r="C44" s="67" t="str">
-        <x:v>Not highlighted in reviewed primary feature listing.</x:v>
+        <x:v>Documented — K1EL WinKeyer, CW keyer and RTTY application.</x:v>
       </x:c>
       <x:c r="D44" s="67" t="str">
-        <x:v>Not highlighted in reviewed primary feature listing.</x:v>
+        <x:v>Documented — CWDaemon, FLDigi, Morse over CAT, WinKey v1/v2 and CW Console.</x:v>
       </x:c>
       <x:c r="E44" s="59"/>
       <x:c r="F44" s="59"/>
     </x:row>
-    <x:row r="45" ht="84" hidden="0" customHeight="1">
+    <x:row r="45" ht="24" hidden="0" customHeight="1">
       <x:c r="A45" s="66" t="str">
-        <x:v>Awards and statistics</x:v>
+        <x:v>Propagation display</x:v>
       </x:c>
       <x:c r="B45" s="67" t="str">
-        <x:v>Implemented foundation — nine native calculators plus a 192-programme research library. 6d9b186 adds pure QRPDXCCPreflightV1 snapshot screening (7/7 Swift) as an R09 dependency only: candidates/exclusions/unknowns and exact retained-power checks. Candidate stored DXCCs are not validated entities, progress, completion or sponsor credit. Measurement, sponsor validity, applicant scope, land/direct-contact eligibility and declaration remain unresolved; executable sponsor rules, application/export, route/UI and package/live acceptance stay open.</x:v>
+        <x:v>Source complete with live provider proof — bounded HamQSL/N0NBH refresh and correct freshness semantics; final packaged outage/freshness observation remains.</x:v>
       </x:c>
       <x:c r="C45" s="67" t="str">
-        <x:v>Documented — DXCC plus IOTA, CQ/ITU zones, grids, states, counties, DOKs and detailed QSL statistics.</x:v>
+        <x:v>Not highlighted in reviewed primary feature listing.</x:v>
       </x:c>
       <x:c r="D45" s="67" t="str">
-        <x:v>Documented — basic awards and station statistics.</x:v>
+        <x:v>Not highlighted in reviewed primary feature listing.</x:v>
       </x:c>
       <x:c r="E45" s="59"/>
       <x:c r="F45" s="59"/>
     </x:row>
-    <x:row r="46" ht="24" hidden="0" customHeight="1">
+    <x:row r="46" ht="84" hidden="0" customHeight="1">
       <x:c r="A46" s="66" t="str">
-        <x:v>Contest logging</x:v>
+        <x:v>Awards and statistics</x:v>
       </x:c>
       <x:c r="B46" s="67" t="str">
-        <x:v>Outstanding as a separate programme — ordinary logging remains primary; do not add empty parity UI.</x:v>
+        <x:v>Implemented foundation — nine native calculators plus a 192-programme research library. 6d9b186 adds pure QRPDXCCPreflightV1 snapshot screening (7/7 Swift) as an R09 dependency only: candidates/exclusions/unknowns and exact retained-power checks. Candidate stored DXCCs are not validated entities, progress, completion or sponsor credit. Measurement, sponsor validity, applicant scope, land/direct-contact eligibility and declaration remain unresolved; executable sponsor rules, application/export, route/UI and package/live acceptance stay open.</x:v>
       </x:c>
       <x:c r="C46" s="67" t="str">
-        <x:v>Documented — specialized contest/DXpedition logger with scoring and ESM.</x:v>
+        <x:v>Documented — DXCC plus IOTA, CQ/ITU zones, grids, states, counties, DOKs and detailed QSL statistics.</x:v>
       </x:c>
       <x:c r="D46" s="67" t="str">
-        <x:v>Documented — basic contest support; QLog states contests are not its current focus.</x:v>
+        <x:v>Documented — basic awards and station statistics.</x:v>
       </x:c>
       <x:c r="E46" s="59"/>
       <x:c r="F46" s="59"/>
     </x:row>
     <x:row r="47" ht="24" hidden="0" customHeight="1">
       <x:c r="A47" s="66" t="str">
-        <x:v>Paper QSL and label printing</x:v>
+        <x:v>Contest logging</x:v>
       </x:c>
       <x:c r="B47" s="67" t="str">
-        <x:v>Outstanding as a dedicated workflow; ADIF QSL fields are preserved and remote confirmations can refresh.</x:v>
+        <x:v>Outstanding as a separate programme — ordinary logging remains primary; do not add empty parity UI.</x:v>
       </x:c>
       <x:c r="C47" s="67" t="str">
-        <x:v>Documented — incoming paper QSL management and QSL label printing.</x:v>
+        <x:v>Documented — specialized contest/DXpedition logger with scoring and ESM.</x:v>
       </x:c>
       <x:c r="D47" s="67" t="str">
-        <x:v>No paper-label workflow established in the reviewed README.</x:v>
+        <x:v>Documented — basic contest support; QLog states contests are not its current focus.</x:v>
       </x:c>
       <x:c r="E47" s="59"/>
       <x:c r="F47" s="59"/>
     </x:row>
     <x:row r="48" ht="24" hidden="0" customHeight="1">
       <x:c r="A48" s="66" t="str">
-        <x:v>Station/location profiles</x:v>
+        <x:v>Paper QSL and label printing</x:v>
       </x:c>
       <x:c r="B48" s="67" t="str">
-        <x:v>Partial — saved station identity/equipment/workspace configuration exists with separate radio, rotor, antenna and activity ownership; profile UX can be improved without unsafe implicit apply.</x:v>
+        <x:v>Outstanding as a dedicated workflow; ADIF QSL fields are preserved and remote confirmations can refresh.</x:v>
       </x:c>
       <x:c r="C48" s="67" t="str">
-        <x:v>Documented / locally observed — operator identity, radios, QRGs, modes/satellites, cluster, QSL and service groups.</x:v>
+        <x:v>Documented — incoming paper QSL management and QSL label printing.</x:v>
       </x:c>
       <x:c r="D48" s="67" t="str">
-        <x:v>Documented — station location profile support.</x:v>
+        <x:v>No paper-label workflow established in the reviewed README.</x:v>
       </x:c>
       <x:c r="E48" s="59"/>
       <x:c r="F48" s="59"/>
     </x:row>
     <x:row r="49" ht="24" hidden="0" customHeight="1">
       <x:c r="A49" s="66" t="str">
-        <x:v>Secure credential storage</x:v>
+        <x:v>Station/location profiles</x:v>
       </x:c>
       <x:c r="B49" s="67" t="str">
-        <x:v>Implemented — Keychain/vault-backed provider credentials with ownership and revision fencing.</x:v>
+        <x:v>Partial — saved station identity/equipment/workspace configuration exists with separate radio, rotor, antenna and activity ownership; profile UX can be improved without unsafe implicit apply.</x:v>
       </x:c>
       <x:c r="C49" s="67" t="str">
-        <x:v>Uses macOS platform storage for supported services; exact architecture was not audited.</x:v>
+        <x:v>Documented / locally observed — operator identity, radios, QRGs, modes/satellites, cluster, QSL and service groups.</x:v>
       </x:c>
       <x:c r="D49" s="67" t="str">
-        <x:v>Documented — system keyring/credential store support on Linux, Windows and macOS.</x:v>
+        <x:v>Documented — station location profile support.</x:v>
       </x:c>
       <x:c r="E49" s="59"/>
       <x:c r="F49" s="59"/>
     </x:row>
     <x:row r="50" ht="24" hidden="0" customHeight="1">
       <x:c r="A50" s="66" t="str">
-        <x:v>Backups</x:v>
+        <x:v>Secure credential storage</x:v>
       </x:c>
       <x:c r="B50" s="67" t="str">
-        <x:v>Partial — local backup/restore safety exists; optional remote FTP/FTPS/SFTP work is active in a separate user-owned change set and is not counted complete here.</x:v>
+        <x:v>Implemented — Keychain/vault-backed provider credentials with ownership and revision fencing.</x:v>
       </x:c>
       <x:c r="C50" s="67" t="str">
-        <x:v>Not established in reviewed primary feature listing.</x:v>
+        <x:v>Uses macOS platform storage for supported services; exact architecture was not audited.</x:v>
       </x:c>
       <x:c r="D50" s="67" t="str">
-        <x:v>Not established in reviewed primary feature listing.</x:v>
+        <x:v>Documented — system keyring/credential store support on Linux, Windows and macOS.</x:v>
       </x:c>
       <x:c r="E50" s="59"/>
       <x:c r="F50" s="59"/>
     </x:row>
     <x:row r="51" ht="24" hidden="0" customHeight="1">
       <x:c r="A51" s="66" t="str">
-        <x:v>Cross-platform delivery</x:v>
+        <x:v>Backups</x:v>
       </x:c>
       <x:c r="B51" s="67" t="str">
-        <x:v>Partial — one shared UI/domain targets macOS, Windows and Linux; Mac is the current acceptance focus and Windows/Linux packaging is intentionally deferred.</x:v>
+        <x:v>Partial — local backup/restore safety exists; optional remote FTP/FTPS/SFTP work is active in a separate user-owned change set and is not counted complete here.</x:v>
       </x:c>
       <x:c r="C51" s="67" t="str">
-        <x:v>Mac only.</x:v>
+        <x:v>Not established in reviewed primary feature listing.</x:v>
       </x:c>
       <x:c r="D51" s="67" t="str">
-        <x:v>Linux and Windows supported; macOS is documented as experimental/developer-only.</x:v>
+        <x:v>Not established in reviewed primary feature listing.</x:v>
       </x:c>
       <x:c r="E51" s="59"/>
       <x:c r="F51" s="59"/>
     </x:row>
     <x:row r="52" ht="24" hidden="0" customHeight="1">
       <x:c r="A52" s="66" t="str">
-        <x:v>Privacy and telemetry</x:v>
+        <x:v>Cross-platform delivery</x:v>
       </x:c>
       <x:c r="B52" s="67" t="str">
-        <x:v>Implemented by design — local-first operation, explicit external-service enrollment and no hidden station/network actions in source acceptance tests.</x:v>
+        <x:v>Partial — one shared UI/domain targets macOS, Windows and Linux; Mac is the current acceptance focus and Windows/Linux packaging is intentionally deferred.</x:v>
       </x:c>
       <x:c r="C52" s="67" t="str">
-        <x:v>Current App Store disclosure says data is not collected.</x:v>
+        <x:v>Mac only.</x:v>
       </x:c>
       <x:c r="D52" s="67" t="str">
-        <x:v>Documented — no ads, user tracking or hidden telemetry.</x:v>
+        <x:v>Linux and Windows supported; macOS is documented as experimental/developer-only.</x:v>
       </x:c>
       <x:c r="E52" s="59"/>
       <x:c r="F52" s="59"/>
     </x:row>
-    <x:row r="53" ht="15" hidden="0" customHeight="1">
-      <x:c r="A53" s="59"/>
-      <x:c r="B53" s="59"/>
-      <x:c r="C53" s="59"/>
-      <x:c r="D53" s="59"/>
+    <x:row r="53" ht="24" hidden="0" customHeight="1">
+      <x:c r="A53" s="66" t="str">
+        <x:v>Privacy and telemetry</x:v>
+      </x:c>
+      <x:c r="B53" s="67" t="str">
+        <x:v>Implemented by design — local-first operation, explicit external-service enrollment and no hidden station/network actions in source acceptance tests.</x:v>
+      </x:c>
+      <x:c r="C53" s="67" t="str">
+        <x:v>Current App Store disclosure says data is not collected.</x:v>
+      </x:c>
+      <x:c r="D53" s="67" t="str">
+        <x:v>Documented — no ads, user tracking or hidden telemetry.</x:v>
+      </x:c>
       <x:c r="E53" s="59"/>
       <x:c r="F53" s="59"/>
     </x:row>
@@ -2728,7 +2736,7 @@
   <x:mergeCells>
     <x:mergeCell ref="A3:D3"/>
   </x:mergeCells>
-  <x:conditionalFormatting sqref="B7:B52">
+  <x:conditionalFormatting sqref="B7:B53">
     <x:cfRule type="beginsWith" dxfId="0" priority="1" operator="beginsWith" text="Installed"/>
     <x:cfRule type="beginsWith" dxfId="1" priority="2" operator="beginsWith" text="Implemented"/>
     <x:cfRule type="beginsWith" dxfId="2" priority="3" operator="beginsWith" text="Source complete"/>
@@ -2738,7 +2746,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf808ae769514475a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf2635691972b4cc9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2930,7 +2938,7 @@
         <x:v>ADIF 3.1.8 conformance</x:v>
       </x:c>
       <x:c r="C12" s="67" t="str">
-        <x:v>Seven compatibility stages complete</x:v>
+        <x:v>Eight compatibility stages complete</x:v>
       </x:c>
       <x:c r="D12" s="67" t="str">
         <x:v>Complete the remaining enum/deprecation and MODE/SUBMODE audit before changing ADIF_VER; run copied-log/package and service-specific interoperability acceptance.</x:v>
@@ -2962,7 +2970,7 @@
         <x:v>Official/date-qualified CTY rules</x:v>
       </x:c>
     </x:row>
-    <x:row r="14" ht="156" hidden="0" customHeight="1">
+    <x:row r="14" ht="180" hidden="0" customHeight="1">
       <x:c r="A14" s="66" t="str">
         <x:v>P1</x:v>
       </x:c>
@@ -2970,7 +2978,7 @@
         <x:v>Full TCI radio provider</x:v>
       </x:c>
       <x:c r="C14" s="67" t="str">
-        <x:v>Receive tune/filter plus passive split, TX-frequency, APP_FOCUS, addressed/legacy spot-click CW_MACROS_EMPTY receipt and opaque CALLSIGN_SEND plus VFO_LOCK, RX_CHANNEL_SENSORS and separate deprecated RX_SENSORS tokens source complete; latest focused tests 78/78</x:v>
+        <x:v>Receive tune/filter plus passive split, TX-frequency, APP_FOCUS, addressed/legacy spot-click CW_MACROS_EMPTY receipt and opaque CALLSIGN_SEND plus VFO_LOCK, RX_CHANNEL_SENSORS and separate deprecated RX_SENSORS plus formal-five-field TX_SENSORS tokens source complete; latest focused tests 84/84</x:v>
       </x:c>
       <x:c r="D14" s="67" t="str">
         <x:v>Extend the existing no-replay owner with separately reviewed split/TX-VFO controls, urgent release and optional audio/IQ slices; passive notifications never become configured evidence/inventory or CW/RF authority. Transmit/PTT keeps its own explicit authority.</x:v>
@@ -4640,7 +4648,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R861ec0cd4c5a471c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rba573a0ee44840ea"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4783,13 +4791,13 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="C10" s="67" t="str">
-        <x:v>Seven compatibility stages complete</x:v>
+        <x:v>Eight compatibility stages complete</x:v>
       </x:c>
       <x:c r="D10" s="67" t="str">
         <x:v>ADIF parser/writer and frontend transfer</x:v>
       </x:c>
       <x:c r="E10" s="67" t="str">
-        <x:v>Finish remaining 3.1.8 audit after PSK63/PSK63F; retain ADIF_VER 3.1.7.</x:v>
+        <x:v>Finish remaining 3.1.8 audit after PSK63/PSK63F/PSK125; retain ADIF_VER 3.1.7.</x:v>
       </x:c>
       <x:c r="F10" s="59"/>
     </x:row>
@@ -4883,7 +4891,7 @@
       </x:c>
       <x:c r="F15" s="59"/>
     </x:row>
-    <x:row r="16" ht="15" hidden="0" customHeight="1">
+    <x:row r="16" ht="24" hidden="0" customHeight="1">
       <x:c r="A16" s="66" t="str">
         <x:v>R10</x:v>
       </x:c>
@@ -4891,13 +4899,13 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="C16" s="67" t="str">
-        <x:v>Useful extension</x:v>
+        <x:v>One-contact read-only core source complete; route/UI and corrections open</x:v>
       </x:c>
       <x:c r="D16" s="67" t="str">
-        <x:v>Validation, conflict merge, CTY and provenance</x:v>
+        <x:v>QSODataQuality, validation/conflict owner, dated CTY and retained power provenance</x:v>
       </x:c>
       <x:c r="E16" s="67" t="str">
-        <x:v>Read-only field source/date and reversible change preview.</x:v>
+        <x:v>5/5 Swift; qualitative findings only, no correction or award/sync delta. Next: bounded route/UI and package/copied-log acceptance.</x:v>
       </x:c>
       <x:c r="F16" s="59"/>
     </x:row>
@@ -6527,7 +6535,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfe3962042cb6446c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9d710e35c30945e1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6607,7 +6615,7 @@
         <x:v>OM0RX-xLog</x:v>
       </x:c>
       <x:c r="B7" s="65" t="str">
-        <x:v>Current implementation checkpoint 2d7bb1f627139c55cd32e5dd673dab4d271031d1</x:v>
+        <x:v>Current implementation checkpoint 5d1199646986ae708f2ed5423448cf87eef2155e</x:v>
       </x:c>
       <x:c r="C7" s="65" t="str">
         <x:v>2026-10-16</x:v>
@@ -6618,18 +6626,18 @@
       <x:c r="E7" s="59"/>
       <x:c r="F7" s="59"/>
     </x:row>
-    <x:row r="8" ht="84" hidden="0" customHeight="1">
+    <x:row r="8" ht="108" hidden="0" customHeight="1">
       <x:c r="A8" s="66" t="str">
         <x:v>OM0RX-xLog</x:v>
       </x:c>
       <x:c r="B8" s="67" t="str">
-        <x:v>https://github.com/oliverbross/OM0RX-xLog/commit/2d7bb1f627139c55cd32e5dd673dab4d271031d1</x:v>
+        <x:v>https://github.com/oliverbross/OM0RX-xLog/commit/5d1199646986ae708f2ed5423448cf87eef2155e</x:v>
       </x:c>
       <x:c r="C8" s="67" t="str">
         <x:v>2026-10-16</x:v>
       </x:c>
       <x:c r="D8" s="67" t="str">
-        <x:v>Exact committed implementation baseline includes conservative QRP DXCC preflight dependency (6d9b186), PSK63 (3002e96), PSK63F (a118dea), passive TCI APP_FOCUS (1e11f0f), legacy CLICKED_ON_SPOT (89cac01), receipt-only CW_MACROS_EMPTY (30ed9d0), passive CALLSIGN_SEND (7b2e0ea), passive VFO_LOCK (6c1cad0), exact-token RX_CHANNEL_SENSORS (ed8ed37; earlier rerun 71/72), separate deprecated per-TRX RX_SENSORS (2d7bb1f; later independent focused 78/78) and read-only online-log follow-up route/Logbook UI (5486aff), plus earlier tracked stages. Preflight does not implement an executable sponsor award or credit.</x:v>
+        <x:v>Exact committed implementation baseline includes one-contact read-only QSODataQuality findings (5d11996; 5/5), formal-five-field passive TX_SENSORS (dbf6e36; 84/84), PSK125 import-only normalization (6253f8f; Swift18/18, frontend1186/1186, tsc) and conservative QRP DXCC preflight dependency (6d9b186), PSK63 (3002e96), PSK63F (a118dea), passive TCI APP_FOCUS (1e11f0f), legacy CLICKED_ON_SPOT (89cac01), receipt-only CW_MACROS_EMPTY (30ed9d0), passive CALLSIGN_SEND (7b2e0ea), passive VFO_LOCK (6c1cad0), exact-token RX_CHANNEL_SENSORS (ed8ed37; earlier rerun 71/72), separate deprecated per-TRX RX_SENSORS (2d7bb1f; later independent focused 78/78) and read-only online-log follow-up route/Logbook UI (5486aff), plus earlier tracked stages. Preflight does not implement an executable sponsor award or credit.</x:v>
       </x:c>
       <x:c r="E8" s="59"/>
       <x:c r="F8" s="59"/>
@@ -8256,7 +8264,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R281677291b2c43f7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R707f3978b7554e1f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Track TCI mute and data quality route
</commit_message>
<xml_diff>
--- a/outputs/feature-matrix-2026-10-16/OM0RX-xLog_Feature_Comparison_2026-10-16.xlsx
+++ b/outputs/feature-matrix-2026-10-16/OM0RX-xLog_Feature_Comparison_2026-10-16.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Matrix" sheetId="1" r:id="R8d425f43706f4800"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Outstanding" sheetId="2" r:id="R4d9341c6dd62478a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enhancement Review" sheetId="3" r:id="Ra028556bac284a5d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="4" r:id="R5ef82882c9864c10"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Matrix" sheetId="1" r:id="Ra9f124f4ab844996"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Outstanding" sheetId="2" r:id="R0493fcb851164442"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enhancement Review" sheetId="3" r:id="R878a49e6d8c24f60"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="4" r:id="R7342fa5276114c64"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -852,12 +852,12 @@
       <x:c r="E9" s="59"/>
       <x:c r="F9" s="59"/>
     </x:row>
-    <x:row r="10" ht="72" hidden="0" customHeight="1">
+    <x:row r="10" ht="132" hidden="0" customHeight="1">
       <x:c r="A10" s="66" t="str">
         <x:v>QSO data quality findings</x:v>
       </x:c>
       <x:c r="B10" s="67" t="str">
-        <x:v>Source complete for read-only core — QSODataQuality inspects one retained revision using existing validation, supplied dated CTY comparison at QSO date, retained power provenance and exact-context conflict alternatives (5d11996; 5/5 Swift). Stored/manual overrides stay authoritative. Dates retain source/observation/detection roles rather than field origin. Findings supply qualitative impacts only, no correction or award/confirmation/sync delta. Route/UI, corrections and package/copied-log/live acceptance remain open.</x:v>
+        <x:v>Source complete for read-only core and exact-contact route — QSODataQuality inspects one retained revision using existing validation, supplied dated CTY comparison at QSO date, retained power provenance and exact-context conflict alternatives (5d11996; 5/5 Swift). Stored/manual overrides stay authoritative. Dates retain source/observation/detection roles rather than field origin. Findings supply qualitative impacts only, no correction or award/confirmation/sync delta. UI, corrections and package/copied-log/live acceptance remain open. 862e444 adds logbook_data_quality scoped to exact contact/generation/revision, optional primary-key retained conflict, canonical snapshot/current CTY owner with version/date unknown and duplicate review not performed. Main/Logbook only; no corrections/writes/provider refresh/award/sync delta/UI. Swift route 2/2, combined 3/3, Rust auth 1/1, frontend 7/7 and tsc pass; initial route-test compile defects fixed before commit.</x:v>
       </x:c>
       <x:c r="C10" s="67" t="str">
         <x:v>Documented — QSO editing and DXCC/QSL workflows; comparable field-provenance findings were not established.</x:v>
@@ -1332,12 +1332,12 @@
       <x:c r="E39" s="59"/>
       <x:c r="F39" s="59"/>
     </x:row>
-    <x:row r="40" ht="336" hidden="0" customHeight="1">
+    <x:row r="40" ht="384" hidden="0" customHeight="1">
       <x:c r="A40" s="66" t="str">
         <x:v>TCI rig control — SunSDR/ExpertSDR and compatible servers</x:v>
       </x:c>
       <x:c r="B40" s="67" t="str">
-        <x:v>Source complete through receive tune/filter, configured-TRX split, global TX-frequency telemetry, APP_FOCUS, addressed RX_CLICKED_ON_SPOT, legacy CLICKED_ON_SPOT and receipt-only CW_MACROS_EMPTY and opaque CALLSIGN_SEND and per-address VFO_LOCK plus RX_CHANNEL_SENSORS and separate deprecated RX_SENSORS plus formal-five-field TX_SENSORS token observations. Passive notifications retain independent producer receipts; legacy clicks infer no TRX/channel/VFO. CW_MACROS_EMPTY proves no queue-empty, TX/RX, CW or RF authority. APP_FOCUS Swift 45/45, legacy-click 50/50 (lifecycle rerun) CW receipt 55/55 and CALLSIGN_SEND 60/60 (34 protocol + 26 session) pass. CALLSIGN_SEND uses strict validation/reconnect clearing and confers no target/contact identity authority, command correlation, TX completion/success or RF inference. VFO_LOCK 66/66 (38 protocol + 28 session) retains independent exact-address producer times, validates exactly three arguments within application/discovery bounds, prunes on discovery shrink and clears on reconnect. It grants no owner/expiry, tune confirmation, configured freshness or control authority. RX_CHANNEL_SENSORS preserves exact bounded ASCII decimals per address without Double conversion or physical range/calibration/quality/readiness/freshness/control claims; discovery prunes and reconnect clears. Six new tests pass twice, protocol 42/42; broader session rerun at ed8ed37 was 71/72 on unchanged testDroppingLastSessionReferenceClosesPendingConnection (closeCount 0 vs 1); initial existing tune-yield miss passed rerun. Build/diff clean. 2d7bb1f adds deprecated server-only RX_SENSORS as separate per-TRX raw bounded decimal tokens plus local producer receipt, never channel-attributed or merged with RX_CHANNEL_SENSORS. TRX discovery prunes, channel-count changes do not remap and reconnect clears. No physical range/calibration/readiness/freshness/control/RF inference. Later independent focused tests 78/78 pass; earlier timing miss is not claimed fixed. dbf6e36 adds passive formal-five-field TX_SENSORS raw per-TRX receipts (84/84); malformed printed example rejects and no TX/RF/physical power/SWR authority is inferred. Explicit controls retain the existing no-replay/readback owner. Transmit/PTT, split/TX-VFO controls, outbound spots, audio/IQ and package/live-server/RF acceptance remain open.</x:v>
+        <x:v>Source complete through receive tune/filter, configured-TRX split, global TX-frequency telemetry, APP_FOCUS, addressed RX_CLICKED_ON_SPOT, legacy CLICKED_ON_SPOT and receipt-only CW_MACROS_EMPTY and opaque CALLSIGN_SEND and per-address VFO_LOCK plus RX_CHANNEL_SENSORS and separate deprecated RX_SENSORS plus formal-five-field TX_SENSORS token observations. Passive notifications retain independent producer receipts; legacy clicks infer no TRX/channel/VFO. CW_MACROS_EMPTY proves no queue-empty, TX/RX, CW or RF authority. APP_FOCUS Swift 45/45, legacy-click 50/50 (lifecycle rerun) CW receipt 55/55 and CALLSIGN_SEND 60/60 (34 protocol + 26 session) pass. CALLSIGN_SEND uses strict validation/reconnect clearing and confers no target/contact identity authority, command correlation, TX completion/success or RF inference. VFO_LOCK 66/66 (38 protocol + 28 session) retains independent exact-address producer times, validates exactly three arguments within application/discovery bounds, prunes on discovery shrink and clears on reconnect. It grants no owner/expiry, tune confirmation, configured freshness or control authority. RX_CHANNEL_SENSORS preserves exact bounded ASCII decimals per address without Double conversion or physical range/calibration/quality/readiness/freshness/control claims; discovery prunes and reconnect clears. Six new tests pass twice, protocol 42/42; broader session rerun at ed8ed37 was 71/72 on unchanged testDroppingLastSessionReferenceClosesPendingConnection (closeCount 0 vs 1); initial existing tune-yield miss passed rerun. Build/diff clean. 2d7bb1f adds deprecated server-only RX_SENSORS as separate per-TRX raw bounded decimal tokens plus local producer receipt, never channel-attributed or merged with RX_CHANNEL_SENSORS. TRX discovery prunes, channel-count changes do not remap and reconnect clears. No physical range/calibration/readiness/freshness/control/RF inference. Later independent focused tests 78/78 pass; earlier timing miss is not claimed fixed. dbf6e36 adds passive formal-five-field TX_SENSORS raw per-TRX receipts (84/84); malformed printed example rejects and no TX/RF/physical power/SWR authority is inferred. Explicit controls retain the existing no-replay/readback owner. Transmit/PTT, split/TX-VFO controls, outbound spots, audio/IQ and package/live-server/RF acceptance remain open. 711d4c4 retains global MUTE from pinned TCI pp 21–22 with own receipt, strict bool and reconnect clear; no encoder/query/setter/control/configured readiness/tune/TX/RF effect. New 5/5 and protocol 53/53 pass; broad 88/89 retains unchanged lifecycle closeCount 0 vs 1. Root combined-tree new 5/5 passes after R10 test compile fixes, not a lifecycle fix.</x:v>
       </x:c>
       <x:c r="C40" s="67" t="str">
         <x:v>Not established in the reviewed primary RUMlogNG evidence.</x:v>
@@ -2746,7 +2746,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf2635691972b4cc9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R70c32bf8e7674490"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2970,7 +2970,7 @@
         <x:v>Official/date-qualified CTY rules</x:v>
       </x:c>
     </x:row>
-    <x:row r="14" ht="180" hidden="0" customHeight="1">
+    <x:row r="14" ht="216" hidden="0" customHeight="1">
       <x:c r="A14" s="66" t="str">
         <x:v>P1</x:v>
       </x:c>
@@ -2978,7 +2978,7 @@
         <x:v>Full TCI radio provider</x:v>
       </x:c>
       <x:c r="C14" s="67" t="str">
-        <x:v>Receive tune/filter plus passive split, TX-frequency, APP_FOCUS, addressed/legacy spot-click CW_MACROS_EMPTY receipt and opaque CALLSIGN_SEND plus VFO_LOCK, RX_CHANNEL_SENSORS and separate deprecated RX_SENSORS plus formal-five-field TX_SENSORS tokens source complete; latest focused tests 84/84</x:v>
+        <x:v>Receive tune/filter plus passive split, TX-frequency, APP_FOCUS, addressed/legacy spot-click CW_MACROS_EMPTY receipt and opaque CALLSIGN_SEND plus VFO_LOCK, RX_CHANNEL_SENSORS and separate deprecated RX_SENSORS plus formal-five-field TX_SENSORS tokens source complete; latest focused tests 84/84; passive global MUTE source complete (broad gate88/89, new 5/5 root rerun)</x:v>
       </x:c>
       <x:c r="D14" s="67" t="str">
         <x:v>Extend the existing no-replay owner with separately reviewed split/TX-VFO controls, urgent release and optional audio/IQ slices; passive notifications never become configured evidence/inventory or CW/RF authority. Transmit/PTT keeps its own explicit authority.</x:v>
@@ -4648,7 +4648,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rba573a0ee44840ea"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6e124765c82a4949"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4891,7 +4891,7 @@
       </x:c>
       <x:c r="F15" s="59"/>
     </x:row>
-    <x:row r="16" ht="24" hidden="0" customHeight="1">
+    <x:row r="16" ht="36" hidden="0" customHeight="1">
       <x:c r="A16" s="66" t="str">
         <x:v>R10</x:v>
       </x:c>
@@ -4899,13 +4899,13 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="C16" s="67" t="str">
-        <x:v>One-contact read-only core source complete; route/UI and corrections open</x:v>
+        <x:v>Read-only core and exact-contact route source complete; UI/corrections open</x:v>
       </x:c>
       <x:c r="D16" s="67" t="str">
-        <x:v>QSODataQuality, validation/conflict owner, dated CTY and retained power provenance</x:v>
+        <x:v>QSODataQuality, canonical snapshot/current CTY owner and primary-key retained conflict</x:v>
       </x:c>
       <x:c r="E16" s="67" t="str">
-        <x:v>5/5 Swift; qualitative findings only, no correction or award/sync delta. Next: bounded route/UI and package/copied-log acceptance.</x:v>
+        <x:v>862e444: exact generation/revision, duplicate review not performed, CTY metadata unknown; route 2/2+combined 3/3, auth 1/1, frontend 7/7, tsc. Next UI/package; no correction/delta.</x:v>
       </x:c>
       <x:c r="F16" s="59"/>
     </x:row>
@@ -6535,7 +6535,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9d710e35c30945e1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R404814df650c4db6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6615,7 +6615,7 @@
         <x:v>OM0RX-xLog</x:v>
       </x:c>
       <x:c r="B7" s="65" t="str">
-        <x:v>Current implementation checkpoint 5d1199646986ae708f2ed5423448cf87eef2155e</x:v>
+        <x:v>Current implementation checkpoint 862e44456f1e88fb244e520d4107aa0fa5f3a566</x:v>
       </x:c>
       <x:c r="C7" s="65" t="str">
         <x:v>2026-10-16</x:v>
@@ -6626,18 +6626,18 @@
       <x:c r="E7" s="59"/>
       <x:c r="F7" s="59"/>
     </x:row>
-    <x:row r="8" ht="108" hidden="0" customHeight="1">
+    <x:row r="8" ht="48" hidden="0" customHeight="1">
       <x:c r="A8" s="66" t="str">
         <x:v>OM0RX-xLog</x:v>
       </x:c>
       <x:c r="B8" s="67" t="str">
-        <x:v>https://github.com/oliverbross/OM0RX-xLog/commit/5d1199646986ae708f2ed5423448cf87eef2155e</x:v>
+        <x:v>https://github.com/oliverbross/OM0RX-xLog/commit/862e44456f1e88fb244e520d4107aa0fa5f3a566</x:v>
       </x:c>
       <x:c r="C8" s="67" t="str">
         <x:v>2026-10-16</x:v>
       </x:c>
       <x:c r="D8" s="67" t="str">
-        <x:v>Exact committed implementation baseline includes one-contact read-only QSODataQuality findings (5d11996; 5/5), formal-five-field passive TX_SENSORS (dbf6e36; 84/84), PSK125 import-only normalization (6253f8f; Swift18/18, frontend1186/1186, tsc) and conservative QRP DXCC preflight dependency (6d9b186), PSK63 (3002e96), PSK63F (a118dea), passive TCI APP_FOCUS (1e11f0f), legacy CLICKED_ON_SPOT (89cac01), receipt-only CW_MACROS_EMPTY (30ed9d0), passive CALLSIGN_SEND (7b2e0ea), passive VFO_LOCK (6c1cad0), exact-token RX_CHANNEL_SENSORS (ed8ed37; earlier rerun 71/72), separate deprecated per-TRX RX_SENSORS (2d7bb1f; later independent focused 78/78) and read-only online-log follow-up route/Logbook UI (5486aff), plus earlier tracked stages. Preflight does not implement an executable sponsor award or credit.</x:v>
+        <x:v>Latest stages: passive global MUTE (711d4c4; new 5/5, protocol 53/53, broad 88/89 lifecycle timing miss, root combined new 5/5 pass) and read-only exact-contact data-quality route (862e444; Swift2/2+combined 3/3, auth 1/1, frontend 7/7, tsc; test compile fixes before commit). Earlier PSK125, TX_SENSORS and core findings remain included. UI/package/live gates remain open.</x:v>
       </x:c>
       <x:c r="E8" s="59"/>
       <x:c r="F8" s="59"/>
@@ -8264,7 +8264,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R707f3978b7554e1f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbc04f30c6fe24d68"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Track receiver mute ADIF and data quality UI
</commit_message>
<xml_diff>
--- a/outputs/feature-matrix-2026-10-16/OM0RX-xLog_Feature_Comparison_2026-10-16.xlsx
+++ b/outputs/feature-matrix-2026-10-16/OM0RX-xLog_Feature_Comparison_2026-10-16.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Matrix" sheetId="1" r:id="Ra9f124f4ab844996"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Outstanding" sheetId="2" r:id="R0493fcb851164442"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enhancement Review" sheetId="3" r:id="R878a49e6d8c24f60"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="4" r:id="R7342fa5276114c64"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Matrix" sheetId="1" r:id="R8d91510a7e61470a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Outstanding" sheetId="2" r:id="Rc0fbbbba2b6241dc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enhancement Review" sheetId="3" r:id="R6b7f0382fc644eaa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="4" r:id="Rda5108bcf57d4682"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -852,12 +852,12 @@
       <x:c r="E9" s="59"/>
       <x:c r="F9" s="59"/>
     </x:row>
-    <x:row r="10" ht="132" hidden="0" customHeight="1">
+    <x:row r="10" ht="180" hidden="0" customHeight="1">
       <x:c r="A10" s="66" t="str">
         <x:v>QSO data quality findings</x:v>
       </x:c>
       <x:c r="B10" s="67" t="str">
-        <x:v>Source complete for read-only core and exact-contact route — QSODataQuality inspects one retained revision using existing validation, supplied dated CTY comparison at QSO date, retained power provenance and exact-context conflict alternatives (5d11996; 5/5 Swift). Stored/manual overrides stay authoritative. Dates retain source/observation/detection roles rather than field origin. Findings supply qualitative impacts only, no correction or award/confirmation/sync delta. UI, corrections and package/copied-log/live acceptance remain open. 862e444 adds logbook_data_quality scoped to exact contact/generation/revision, optional primary-key retained conflict, canonical snapshot/current CTY owner with version/date unknown and duplicate review not performed. Main/Logbook only; no corrections/writes/provider refresh/award/sync delta/UI. Swift route 2/2, combined 3/3, Rust auth 1/1, frontend 7/7 and tsc pass; initial route-test compile defects fixed before commit.</x:v>
+        <x:v>Source complete for read-only core, exact-contact route and Details UI — QSODataQuality inspects one retained revision using existing validation, supplied dated CTY comparison at QSO date, retained power provenance and exact-context conflict alternatives (5d11996; 5/5 Swift). Stored/manual overrides stay authoritative. Dates retain source/observation/detection roles rather than field origin. Findings supply qualitative impacts only, no correction or award/confirmation/sync delta. Native/package/copied-log/live acceptance, full coverage and corrections remain open. 862e444 adds logbook_data_quality scoped to exact contact/generation/revision, optional primary-key retained conflict, canonical snapshot/current CTY owner with version/date unknown and duplicate review not performed. Main/Logbook only; no corrections/writes/provider refresh/award/sync delta. Swift route 2/2, combined 3/3, Rust auth 1/1, frontend 7/7 and tsc pass; initial route-test compile defects fixed before commit. c4b1602 adds exact-contact read-only Logbook Details findings with explicit Read findings and context retirement. Root 35/35 plus isolated detached 6/6 pass; agent build/tsc/browser geometry pass. No correction/provider refresh/native/package/live acceptance is claimed; installed alpha.31 is unchanged.</x:v>
       </x:c>
       <x:c r="C10" s="67" t="str">
         <x:v>Documented — QSO editing and DXCC/QSL workflows; comparable field-provenance findings were not established.</x:v>
@@ -873,7 +873,7 @@
         <x:v>ADIF field preservation</x:v>
       </x:c>
       <x:c r="B11" s="67" t="str">
-        <x:v>Source complete for eight reviewed compatibility stages — local records retain a JSON field bag; unknown/custom fields, Unicode, station/contact and RX/TX data survive supported ADI/ADX round trips. UTF-8 byte scanning, FT4/FT2/JTTY MFSK-submode export, C4FM/DSTAR DIGITALVOICE-submode handling and import-only PSK31/PSK63/PSK63F/PSK125 to PSK/submode normalization are fixed. Latest Swift 18/18 and frontend 1,186/1,186 and TypeScript pass at PSK125 (6253f8f). Remaining 3.1.8 audit and package/real-log acceptance stay open; ADIF_VER stays 3.1.7.</x:v>
+        <x:v>Source complete for nine reviewed compatibility stages — local records retain a JSON field bag; unknown/custom fields, Unicode, station/contact and RX/TX data survive supported ADI/ADX round trips. UTF-8 byte scanning, FT4/FT2/JTTY MFSK-submode export, C4FM/DSTAR DIGITALVOICE-submode handling and import-only PSK31/PSK63/PSK63F/PSK125/PSKAM10 to PSK/submode normalization are fixed. Latest Swift 18/18 and frontend 1,202/1,202 and TypeScript pass at PSKAM10 (770dda2). Remaining 3.1.8 audit and package/real-log acceptance stay open; ADIF_VER stays 3.1.7.</x:v>
       </x:c>
       <x:c r="C11" s="67" t="str">
         <x:v>Documented — import/export plus four user-definable logging fields.</x:v>
@@ -1332,12 +1332,12 @@
       <x:c r="E39" s="59"/>
       <x:c r="F39" s="59"/>
     </x:row>
-    <x:row r="40" ht="384" hidden="0" customHeight="1">
+    <x:row r="40" ht="420" hidden="0" customHeight="1">
       <x:c r="A40" s="66" t="str">
         <x:v>TCI rig control — SunSDR/ExpertSDR and compatible servers</x:v>
       </x:c>
       <x:c r="B40" s="67" t="str">
-        <x:v>Source complete through receive tune/filter, configured-TRX split, global TX-frequency telemetry, APP_FOCUS, addressed RX_CLICKED_ON_SPOT, legacy CLICKED_ON_SPOT and receipt-only CW_MACROS_EMPTY and opaque CALLSIGN_SEND and per-address VFO_LOCK plus RX_CHANNEL_SENSORS and separate deprecated RX_SENSORS plus formal-five-field TX_SENSORS token observations. Passive notifications retain independent producer receipts; legacy clicks infer no TRX/channel/VFO. CW_MACROS_EMPTY proves no queue-empty, TX/RX, CW or RF authority. APP_FOCUS Swift 45/45, legacy-click 50/50 (lifecycle rerun) CW receipt 55/55 and CALLSIGN_SEND 60/60 (34 protocol + 26 session) pass. CALLSIGN_SEND uses strict validation/reconnect clearing and confers no target/contact identity authority, command correlation, TX completion/success or RF inference. VFO_LOCK 66/66 (38 protocol + 28 session) retains independent exact-address producer times, validates exactly three arguments within application/discovery bounds, prunes on discovery shrink and clears on reconnect. It grants no owner/expiry, tune confirmation, configured freshness or control authority. RX_CHANNEL_SENSORS preserves exact bounded ASCII decimals per address without Double conversion or physical range/calibration/quality/readiness/freshness/control claims; discovery prunes and reconnect clears. Six new tests pass twice, protocol 42/42; broader session rerun at ed8ed37 was 71/72 on unchanged testDroppingLastSessionReferenceClosesPendingConnection (closeCount 0 vs 1); initial existing tune-yield miss passed rerun. Build/diff clean. 2d7bb1f adds deprecated server-only RX_SENSORS as separate per-TRX raw bounded decimal tokens plus local producer receipt, never channel-attributed or merged with RX_CHANNEL_SENSORS. TRX discovery prunes, channel-count changes do not remap and reconnect clears. No physical range/calibration/readiness/freshness/control/RF inference. Later independent focused tests 78/78 pass; earlier timing miss is not claimed fixed. dbf6e36 adds passive formal-five-field TX_SENSORS raw per-TRX receipts (84/84); malformed printed example rejects and no TX/RF/physical power/SWR authority is inferred. Explicit controls retain the existing no-replay/readback owner. Transmit/PTT, split/TX-VFO controls, outbound spots, audio/IQ and package/live-server/RF acceptance remain open. 711d4c4 retains global MUTE from pinned TCI pp 21–22 with own receipt, strict bool and reconnect clear; no encoder/query/setter/control/configured readiness/tune/TX/RF effect. New 5/5 and protocol 53/53 pass; broad 88/89 retains unchanged lifecycle closeCount 0 vs 1. Root combined-tree new 5/5 passes after R10 test compile fixes, not a lifecycle fix.</x:v>
+        <x:v>Source complete through receive tune/filter, configured-TRX split, global TX-frequency telemetry, APP_FOCUS, addressed RX_CLICKED_ON_SPOT, legacy CLICKED_ON_SPOT and receipt-only CW_MACROS_EMPTY and opaque CALLSIGN_SEND and per-address VFO_LOCK plus RX_CHANNEL_SENSORS and separate deprecated RX_SENSORS plus formal-five-field TX_SENSORS token observations. Passive notifications retain independent producer receipts; legacy clicks infer no TRX/channel/VFO. CW_MACROS_EMPTY proves no queue-empty, TX/RX, CW or RF authority. APP_FOCUS Swift 45/45, legacy-click 50/50 (lifecycle rerun) CW receipt 55/55 and CALLSIGN_SEND 60/60 (34 protocol + 26 session) pass. CALLSIGN_SEND uses strict validation/reconnect clearing and confers no target/contact identity authority, command correlation, TX completion/success or RF inference. VFO_LOCK 66/66 (38 protocol + 28 session) retains independent exact-address producer times, validates exactly three arguments within application/discovery bounds, prunes on discovery shrink and clears on reconnect. It grants no owner/expiry, tune confirmation, configured freshness or control authority. RX_CHANNEL_SENSORS preserves exact bounded ASCII decimals per address without Double conversion or physical range/calibration/quality/readiness/freshness/control claims; discovery prunes and reconnect clears. Six new tests pass twice, protocol 42/42; broader session rerun at ed8ed37 was 71/72 on unchanged testDroppingLastSessionReferenceClosesPendingConnection (closeCount 0 vs 1); initial existing tune-yield miss passed rerun. Build/diff clean. 2d7bb1f adds deprecated server-only RX_SENSORS as separate per-TRX raw bounded decimal tokens plus local producer receipt, never channel-attributed or merged with RX_CHANNEL_SENSORS. TRX discovery prunes, channel-count changes do not remap and reconnect clears. No physical range/calibration/readiness/freshness/control/RF inference. Later independent focused tests 78/78 pass; earlier timing miss is not claimed fixed. dbf6e36 adds passive formal-five-field TX_SENSORS raw per-TRX receipts (84/84); malformed printed example rejects and no TX/RF/physical power/SWR authority is inferred. Explicit controls retain the existing no-replay/readback owner. Transmit/PTT, split/TX-VFO controls, outbound spots, audio/IQ and package/live-server/RF acceptance remain open. 711d4c4 retains global MUTE from pinned TCI pp 21–22 with own receipt, strict bool and reconnect clear; no encoder/query/setter/control/configured readiness/tune/TX/RF effect. New 5/5 and protocol 53/53 pass; broad 88/89 retains unchanged lifecycle closeCount 0 vs 1. Root combined-tree new 5/5 passes after R10 test compile fixes, not a lifecycle fix. 46c862b separately observes RX_MUTE for exact receiver/strict bool, with independent receipts, pruning/reconnect clearing and no configured freshness/readiness/tune/TX/control/RF authority. Agent 95/95 and root new 6/6 pass. Earlier lifecycle flake and package/live gates stay disclosed.</x:v>
       </x:c>
       <x:c r="C40" s="67" t="str">
         <x:v>Not established in the reviewed primary RUMlogNG evidence.</x:v>
@@ -2746,7 +2746,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R70c32bf8e7674490"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra5c7238788ac491d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2938,7 +2938,7 @@
         <x:v>ADIF 3.1.8 conformance</x:v>
       </x:c>
       <x:c r="C12" s="67" t="str">
-        <x:v>Eight compatibility stages complete</x:v>
+        <x:v>Nine compatibility stages complete</x:v>
       </x:c>
       <x:c r="D12" s="67" t="str">
         <x:v>Complete the remaining enum/deprecation and MODE/SUBMODE audit before changing ADIF_VER; run copied-log/package and service-specific interoperability acceptance.</x:v>
@@ -2970,7 +2970,7 @@
         <x:v>Official/date-qualified CTY rules</x:v>
       </x:c>
     </x:row>
-    <x:row r="14" ht="216" hidden="0" customHeight="1">
+    <x:row r="14" ht="252" hidden="0" customHeight="1">
       <x:c r="A14" s="66" t="str">
         <x:v>P1</x:v>
       </x:c>
@@ -2978,7 +2978,7 @@
         <x:v>Full TCI radio provider</x:v>
       </x:c>
       <x:c r="C14" s="67" t="str">
-        <x:v>Receive tune/filter plus passive split, TX-frequency, APP_FOCUS, addressed/legacy spot-click CW_MACROS_EMPTY receipt and opaque CALLSIGN_SEND plus VFO_LOCK, RX_CHANNEL_SENSORS and separate deprecated RX_SENSORS plus formal-five-field TX_SENSORS tokens source complete; latest focused tests 84/84; passive global MUTE source complete (broad gate88/89, new 5/5 root rerun)</x:v>
+        <x:v>Receive tune/filter plus passive split, TX-frequency, APP_FOCUS, addressed/legacy spot-click CW_MACROS_EMPTY receipt and opaque CALLSIGN_SEND plus VFO_LOCK, RX_CHANNEL_SENSORS and separate deprecated RX_SENSORS plus formal-five-field TX_SENSORS tokens source complete; latest focused tests 84/84; passive global MUTE source complete (broad gate88/89, new 5/5 root rerun); exact-receiver RX_MUTE source complete (agent 95/95, root new 6/6)</x:v>
       </x:c>
       <x:c r="D14" s="67" t="str">
         <x:v>Extend the existing no-replay owner with separately reviewed split/TX-VFO controls, urgent release and optional audio/IQ slices; passive notifications never become configured evidence/inventory or CW/RF authority. Transmit/PTT keeps its own explicit authority.</x:v>
@@ -4648,7 +4648,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6e124765c82a4949"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7c42d95057c54358"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4783,7 +4783,7 @@
       </x:c>
       <x:c r="F9" s="59"/>
     </x:row>
-    <x:row r="10" ht="15" hidden="0" customHeight="1">
+    <x:row r="10" ht="24" hidden="0" customHeight="1">
       <x:c r="A10" s="66" t="str">
         <x:v>R04</x:v>
       </x:c>
@@ -4791,13 +4791,13 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="C10" s="67" t="str">
-        <x:v>Eight compatibility stages complete</x:v>
+        <x:v>Nine compatibility stages complete</x:v>
       </x:c>
       <x:c r="D10" s="67" t="str">
         <x:v>ADIF parser/writer and frontend transfer</x:v>
       </x:c>
       <x:c r="E10" s="67" t="str">
-        <x:v>Finish remaining 3.1.8 audit after PSK63/PSK63F/PSK125; retain ADIF_VER 3.1.7.</x:v>
+        <x:v>Finish remaining 3.1.8 audit after PSK63/PSK63F/PSK125/PSKAM10; retain ADIF_VER 3.1.7.</x:v>
       </x:c>
       <x:c r="F10" s="59"/>
     </x:row>
@@ -4899,13 +4899,13 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="C16" s="67" t="str">
-        <x:v>Read-only core and exact-contact route source complete; UI/corrections open</x:v>
+        <x:v>Read-only core/route/Details UI source complete; acceptance/corrections open</x:v>
       </x:c>
       <x:c r="D16" s="67" t="str">
-        <x:v>QSODataQuality, canonical snapshot/current CTY owner and primary-key retained conflict</x:v>
+        <x:v>QSODataQuality, exact-contact canonical route and Logbook Details</x:v>
       </x:c>
       <x:c r="E16" s="67" t="str">
-        <x:v>862e444: exact generation/revision, duplicate review not performed, CTY metadata unknown; route 2/2+combined 3/3, auth 1/1, frontend 7/7, tsc. Next UI/package; no correction/delta.</x:v>
+        <x:v>c4b1602: root 35/35 + detached 6/6; agent build/tsc/browser geometry pass. Next native/package/copied-log/live/full coverage; no correction, provider refresh or award/sync delta.</x:v>
       </x:c>
       <x:c r="F16" s="59"/>
     </x:row>
@@ -6535,7 +6535,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R404814df650c4db6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf09f673318bd494b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6615,7 +6615,7 @@
         <x:v>OM0RX-xLog</x:v>
       </x:c>
       <x:c r="B7" s="65" t="str">
-        <x:v>Current implementation checkpoint 862e44456f1e88fb244e520d4107aa0fa5f3a566</x:v>
+        <x:v>Current implementation checkpoint c4b160281b6fbf1a65adcb8f782ec41503a0f969</x:v>
       </x:c>
       <x:c r="C7" s="65" t="str">
         <x:v>2026-10-16</x:v>
@@ -6626,18 +6626,18 @@
       <x:c r="E7" s="59"/>
       <x:c r="F7" s="59"/>
     </x:row>
-    <x:row r="8" ht="48" hidden="0" customHeight="1">
+    <x:row r="8" ht="60" hidden="0" customHeight="1">
       <x:c r="A8" s="66" t="str">
         <x:v>OM0RX-xLog</x:v>
       </x:c>
       <x:c r="B8" s="67" t="str">
-        <x:v>https://github.com/oliverbross/OM0RX-xLog/commit/862e44456f1e88fb244e520d4107aa0fa5f3a566</x:v>
+        <x:v>https://github.com/oliverbross/OM0RX-xLog/commit/c4b160281b6fbf1a65adcb8f782ec41503a0f969</x:v>
       </x:c>
       <x:c r="C8" s="67" t="str">
         <x:v>2026-10-16</x:v>
       </x:c>
       <x:c r="D8" s="67" t="str">
-        <x:v>Latest stages: passive global MUTE (711d4c4; new 5/5, protocol 53/53, broad 88/89 lifecycle timing miss, root combined new 5/5 pass) and read-only exact-contact data-quality route (862e444; Swift2/2+combined 3/3, auth 1/1, frontend 7/7, tsc; test compile fixes before commit). Earlier PSK125, TX_SENSORS and core findings remain included. UI/package/live gates remain open.</x:v>
+        <x:v>Latest separate stages: passive exact-receiver RX_MUTE (46c862b; agent 95/95, root new 6/6), PSKAM10 ADIF normalization (770dda2; Swift 18/18, frontend 1202/1202, tsc; ADIF_VER 3.1.7), and exact-contact Logbook Details findings UI (c4b1602; root 35/35 + detached 6/6, agent build/tsc/browser geometry). Installed alpha.31 unchanged; earlier lifecycle flake remains disclosed. Native/package/live, full audits and correction/provider-refresh gates remain open.</x:v>
       </x:c>
       <x:c r="E8" s="59"/>
       <x:c r="F8" s="59"/>
@@ -8264,7 +8264,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbc04f30c6fe24d68"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcb291d93bc854667"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Track TCI volume and bounded duplicate review
</commit_message>
<xml_diff>
--- a/outputs/feature-matrix-2026-10-16/OM0RX-xLog_Feature_Comparison_2026-10-16.xlsx
+++ b/outputs/feature-matrix-2026-10-16/OM0RX-xLog_Feature_Comparison_2026-10-16.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Matrix" sheetId="1" r:id="R8d91510a7e61470a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Outstanding" sheetId="2" r:id="Rc0fbbbba2b6241dc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enhancement Review" sheetId="3" r:id="R6b7f0382fc644eaa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="4" r:id="Rda5108bcf57d4682"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Matrix" sheetId="1" r:id="Rae092293bdbf4238"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Outstanding" sheetId="2" r:id="R39af7a88d3ac4c93"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enhancement Review" sheetId="3" r:id="Ra46975ec5ec24c4a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="4" r:id="R290ab8883ae14a2e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -852,12 +852,12 @@
       <x:c r="E9" s="59"/>
       <x:c r="F9" s="59"/>
     </x:row>
-    <x:row r="10" ht="180" hidden="0" customHeight="1">
+    <x:row r="10" ht="108" hidden="0" customHeight="1">
       <x:c r="A10" s="66" t="str">
         <x:v>QSO data quality findings</x:v>
       </x:c>
       <x:c r="B10" s="67" t="str">
-        <x:v>Source complete for read-only core, exact-contact route and Details UI — QSODataQuality inspects one retained revision using existing validation, supplied dated CTY comparison at QSO date, retained power provenance and exact-context conflict alternatives (5d11996; 5/5 Swift). Stored/manual overrides stay authoritative. Dates retain source/observation/detection roles rather than field origin. Findings supply qualitative impacts only, no correction or award/confirmation/sync delta. Native/package/copied-log/live acceptance, full coverage and corrections remain open. 862e444 adds logbook_data_quality scoped to exact contact/generation/revision, optional primary-key retained conflict, canonical snapshot/current CTY owner with version/date unknown and duplicate review not performed. Main/Logbook only; no corrections/writes/provider refresh/award/sync delta. Swift route 2/2, combined 3/3, Rust auth 1/1, frontend 7/7 and tsc pass; initial route-test compile defects fixed before commit. c4b1602 adds exact-contact read-only Logbook Details findings with explicit Read findings and context retirement. Root 35/35 plus isolated detached 6/6 pass; agent build/tsc/browser geometry pass. No correction/provider refresh/native/package/live acceptance is claimed; installed alpha.31 is unchanged.</x:v>
+        <x:v>Source complete for read-only findings, exact-contact route, Details UI and bounded duplicate review. c6ada81 reuses native exact call/band/primary-mode case-insensitive +/-600-second matching, self/deleted excluded, cap 5 plus lookahead with complete/truncated/unknown states. No semantic/frequency/submode/portable-callsign inference or mutation. Existing validation, dated CTY comparisons and retained power provenance remain review evidence; CTY version/date unknown and stored/manual values authoritative. Agent core 8/8, route/regression 6/6, frontend 19/19, tsc/build/window gates; root route 3/3, duplicate 3/3, frontend 19/19 pass. Native/package/live/full-coverage/correction/provider gates stay open; no award/sync delta. Installed alpha.31 unchanged.</x:v>
       </x:c>
       <x:c r="C10" s="67" t="str">
         <x:v>Documented — QSO editing and DXCC/QSL workflows; comparable field-provenance findings were not established.</x:v>
@@ -1332,12 +1332,12 @@
       <x:c r="E39" s="59"/>
       <x:c r="F39" s="59"/>
     </x:row>
-    <x:row r="40" ht="420" hidden="0" customHeight="1">
+    <x:row r="40" ht="456" hidden="0" customHeight="1">
       <x:c r="A40" s="66" t="str">
         <x:v>TCI rig control — SunSDR/ExpertSDR and compatible servers</x:v>
       </x:c>
       <x:c r="B40" s="67" t="str">
-        <x:v>Source complete through receive tune/filter, configured-TRX split, global TX-frequency telemetry, APP_FOCUS, addressed RX_CLICKED_ON_SPOT, legacy CLICKED_ON_SPOT and receipt-only CW_MACROS_EMPTY and opaque CALLSIGN_SEND and per-address VFO_LOCK plus RX_CHANNEL_SENSORS and separate deprecated RX_SENSORS plus formal-five-field TX_SENSORS token observations. Passive notifications retain independent producer receipts; legacy clicks infer no TRX/channel/VFO. CW_MACROS_EMPTY proves no queue-empty, TX/RX, CW or RF authority. APP_FOCUS Swift 45/45, legacy-click 50/50 (lifecycle rerun) CW receipt 55/55 and CALLSIGN_SEND 60/60 (34 protocol + 26 session) pass. CALLSIGN_SEND uses strict validation/reconnect clearing and confers no target/contact identity authority, command correlation, TX completion/success or RF inference. VFO_LOCK 66/66 (38 protocol + 28 session) retains independent exact-address producer times, validates exactly three arguments within application/discovery bounds, prunes on discovery shrink and clears on reconnect. It grants no owner/expiry, tune confirmation, configured freshness or control authority. RX_CHANNEL_SENSORS preserves exact bounded ASCII decimals per address without Double conversion or physical range/calibration/quality/readiness/freshness/control claims; discovery prunes and reconnect clears. Six new tests pass twice, protocol 42/42; broader session rerun at ed8ed37 was 71/72 on unchanged testDroppingLastSessionReferenceClosesPendingConnection (closeCount 0 vs 1); initial existing tune-yield miss passed rerun. Build/diff clean. 2d7bb1f adds deprecated server-only RX_SENSORS as separate per-TRX raw bounded decimal tokens plus local producer receipt, never channel-attributed or merged with RX_CHANNEL_SENSORS. TRX discovery prunes, channel-count changes do not remap and reconnect clears. No physical range/calibration/readiness/freshness/control/RF inference. Later independent focused tests 78/78 pass; earlier timing miss is not claimed fixed. dbf6e36 adds passive formal-five-field TX_SENSORS raw per-TRX receipts (84/84); malformed printed example rejects and no TX/RF/physical power/SWR authority is inferred. Explicit controls retain the existing no-replay/readback owner. Transmit/PTT, split/TX-VFO controls, outbound spots, audio/IQ and package/live-server/RF acceptance remain open. 711d4c4 retains global MUTE from pinned TCI pp 21–22 with own receipt, strict bool and reconnect clear; no encoder/query/setter/control/configured readiness/tune/TX/RF effect. New 5/5 and protocol 53/53 pass; broad 88/89 retains unchanged lifecycle closeCount 0 vs 1. Root combined-tree new 5/5 passes after R10 test compile fixes, not a lifecycle fix. 46c862b separately observes RX_MUTE for exact receiver/strict bool, with independent receipts, pruning/reconnect clearing and no configured freshness/readiness/tune/TX/control/RF authority. Agent 95/95 and root new 6/6 pass. Earlier lifecycle flake and package/live gates stay disclosed.</x:v>
+        <x:v>Source complete through receive tune/filter, configured-TRX split, global TX-frequency telemetry, APP_FOCUS, addressed RX_CLICKED_ON_SPOT, legacy CLICKED_ON_SPOT and receipt-only CW_MACROS_EMPTY and opaque CALLSIGN_SEND and per-address VFO_LOCK plus RX_CHANNEL_SENSORS and separate deprecated RX_SENSORS plus formal-five-field TX_SENSORS token observations. Passive notifications retain independent producer receipts; legacy clicks infer no TRX/channel/VFO. CW_MACROS_EMPTY proves no queue-empty, TX/RX, CW or RF authority. APP_FOCUS Swift 45/45, legacy-click 50/50 (lifecycle rerun) CW receipt 55/55 and CALLSIGN_SEND 60/60 (34 protocol + 26 session) pass. CALLSIGN_SEND uses strict validation/reconnect clearing and confers no target/contact identity authority, command correlation, TX completion/success or RF inference. VFO_LOCK 66/66 (38 protocol + 28 session) retains independent exact-address producer times, validates exactly three arguments within application/discovery bounds, prunes on discovery shrink and clears on reconnect. It grants no owner/expiry, tune confirmation, configured freshness or control authority. RX_CHANNEL_SENSORS preserves exact bounded ASCII decimals per address without Double conversion or physical range/calibration/quality/readiness/freshness/control claims; discovery prunes and reconnect clears. Six new tests pass twice, protocol 42/42; broader session rerun at ed8ed37 was 71/72 on unchanged testDroppingLastSessionReferenceClosesPendingConnection (closeCount 0 vs 1); initial existing tune-yield miss passed rerun. Build/diff clean. 2d7bb1f adds deprecated server-only RX_SENSORS as separate per-TRX raw bounded decimal tokens plus local producer receipt, never channel-attributed or merged with RX_CHANNEL_SENSORS. TRX discovery prunes, channel-count changes do not remap and reconnect clears. No physical range/calibration/readiness/freshness/control/RF inference. Later independent focused tests 78/78 pass; earlier timing miss is not claimed fixed. dbf6e36 adds passive formal-five-field TX_SENSORS raw per-TRX receipts (84/84); malformed printed example rejects and no TX/RF/physical power/SWR authority is inferred. Explicit controls retain the existing no-replay/readback owner. Transmit/PTT, split/TX-VFO controls, outbound spots, audio/IQ and package/live-server/RF acceptance remain open. 711d4c4 retains global MUTE from pinned TCI pp 21–22 with own receipt, strict bool and reconnect clear; no encoder/query/setter/control/configured readiness/tune/TX/RF effect. New 5/5 and protocol 53/53 pass; broad 88/89 retains unchanged lifecycle closeCount 0 vs 1. Root combined-tree new 5/5 passes after R10 test compile fixes, not a lifecycle fix. 46c862b separately observes RX_MUTE for exact receiver/strict bool, with independent receipts, pruning/reconnect clearing and no configured freshness/readiness/tune/TX/control/RF authority. Agent 95/95 and root new 6/6 pass. Earlier lifecycle flake and package/live gates stay disclosed. ec83f28 passively observes global VOLUME as exact raw decimal [-60,0] dB plus receipt, without mute/audibility/streaming/readiness/control/RF inference. Agent compiled bundle 101/101 and root full-current-tree new 6/6 pass; earlier lifecycle flake remains disclosed.</x:v>
       </x:c>
       <x:c r="C40" s="67" t="str">
         <x:v>Not established in the reviewed primary RUMlogNG evidence.</x:v>
@@ -2746,7 +2746,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra5c7238788ac491d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd346a346163d4c86"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2970,7 +2970,7 @@
         <x:v>Official/date-qualified CTY rules</x:v>
       </x:c>
     </x:row>
-    <x:row r="14" ht="252" hidden="0" customHeight="1">
+    <x:row r="14" ht="288" hidden="0" customHeight="1">
       <x:c r="A14" s="66" t="str">
         <x:v>P1</x:v>
       </x:c>
@@ -2978,7 +2978,7 @@
         <x:v>Full TCI radio provider</x:v>
       </x:c>
       <x:c r="C14" s="67" t="str">
-        <x:v>Receive tune/filter plus passive split, TX-frequency, APP_FOCUS, addressed/legacy spot-click CW_MACROS_EMPTY receipt and opaque CALLSIGN_SEND plus VFO_LOCK, RX_CHANNEL_SENSORS and separate deprecated RX_SENSORS plus formal-five-field TX_SENSORS tokens source complete; latest focused tests 84/84; passive global MUTE source complete (broad gate88/89, new 5/5 root rerun); exact-receiver RX_MUTE source complete (agent 95/95, root new 6/6)</x:v>
+        <x:v>Receive tune/filter plus passive split, TX-frequency, APP_FOCUS, addressed/legacy spot-click CW_MACROS_EMPTY receipt and opaque CALLSIGN_SEND plus VFO_LOCK, RX_CHANNEL_SENSORS and separate deprecated RX_SENSORS plus formal-five-field TX_SENSORS tokens source complete; latest focused tests 84/84; passive global MUTE source complete (broad gate88/89, new 5/5 root rerun); exact-receiver RX_MUTE source complete (agent 95/95, root new 6/6); passive global VOLUME source complete (agent compiled 101/101, root new 6/6)</x:v>
       </x:c>
       <x:c r="D14" s="67" t="str">
         <x:v>Extend the existing no-replay owner with separately reviewed split/TX-VFO controls, urgent release and optional audio/IQ slices; passive notifications never become configured evidence/inventory or CW/RF authority. Transmit/PTT keeps its own explicit authority.</x:v>
@@ -4648,7 +4648,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7c42d95057c54358"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7b2e5737facf4cef"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4891,7 +4891,7 @@
       </x:c>
       <x:c r="F15" s="59"/>
     </x:row>
-    <x:row r="16" ht="36" hidden="0" customHeight="1">
+    <x:row r="16" ht="48" hidden="0" customHeight="1">
       <x:c r="A16" s="66" t="str">
         <x:v>R10</x:v>
       </x:c>
@@ -4899,13 +4899,13 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="C16" s="67" t="str">
-        <x:v>Read-only core/route/Details UI source complete; acceptance/corrections open</x:v>
+        <x:v>Read-only findings/UI and bounded duplicate review source complete; acceptance/corrections open</x:v>
       </x:c>
       <x:c r="D16" s="67" t="str">
-        <x:v>QSODataQuality, exact-contact canonical route and Logbook Details</x:v>
+        <x:v>Exact-contact canonical route, native duplicate rule and Logbook Details</x:v>
       </x:c>
       <x:c r="E16" s="67" t="str">
-        <x:v>c4b1602: root 35/35 + detached 6/6; agent build/tsc/browser geometry pass. Next native/package/copied-log/live/full coverage; no correction, provider refresh or award/sync delta.</x:v>
+        <x:v>c6ada81: exact call/band/primary-mode, +/-600s, cap 5 + lookahead, complete/truncated/unknown; agent core 8/8, route 6/6, frontend 19/19, tsc/build/windows; root route 3/3+duplicate 3/3+frontend 19/19. Next native/package/live/full coverage; no mutations/delta.</x:v>
       </x:c>
       <x:c r="F16" s="59"/>
     </x:row>
@@ -6535,7 +6535,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf09f673318bd494b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ref45cc0695f242a7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6615,7 +6615,7 @@
         <x:v>OM0RX-xLog</x:v>
       </x:c>
       <x:c r="B7" s="65" t="str">
-        <x:v>Current implementation checkpoint c4b160281b6fbf1a65adcb8f782ec41503a0f969</x:v>
+        <x:v>Current implementation checkpoint c6ada81ae2b90dba15f8d531cabe8524596f9527</x:v>
       </x:c>
       <x:c r="C7" s="65" t="str">
         <x:v>2026-10-16</x:v>
@@ -6631,13 +6631,13 @@
         <x:v>OM0RX-xLog</x:v>
       </x:c>
       <x:c r="B8" s="67" t="str">
-        <x:v>https://github.com/oliverbross/OM0RX-xLog/commit/c4b160281b6fbf1a65adcb8f782ec41503a0f969</x:v>
+        <x:v>https://github.com/oliverbross/OM0RX-xLog/commit/c6ada81ae2b90dba15f8d531cabe8524596f9527</x:v>
       </x:c>
       <x:c r="C8" s="67" t="str">
         <x:v>2026-10-16</x:v>
       </x:c>
       <x:c r="D8" s="67" t="str">
-        <x:v>Latest separate stages: passive exact-receiver RX_MUTE (46c862b; agent 95/95, root new 6/6), PSKAM10 ADIF normalization (770dda2; Swift 18/18, frontend 1202/1202, tsc; ADIF_VER 3.1.7), and exact-contact Logbook Details findings UI (c4b1602; root 35/35 + detached 6/6, agent build/tsc/browser geometry). Installed alpha.31 unchanged; earlier lifecycle flake remains disclosed. Native/package/live, full audits and correction/provider-refresh gates remain open.</x:v>
+        <x:v>Latest separate stages: passive raw global VOLUME (ec83f28; exact [-60,0] dB token/receipt, agent compiled 101/101, root current-tree new 6/6) and bounded native-rule duplicate review (c6ada81; agent core 8/8, route 6/6, frontend 19/19, root route 3/3+duplicate 3/3+frontend 19/19, tsc/build/window gates). Installed alpha.31 and ADIF_VER 3.1.7 unchanged; lifecycle flake remains disclosed. Native/package/live/correction/provider gates remain open.</x:v>
       </x:c>
       <x:c r="E8" s="59"/>
       <x:c r="F8" s="59"/>
@@ -8264,7 +8264,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcb291d93bc854667"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R496c538a4de94f81"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Update implementation evidence through monitor enable
</commit_message>
<xml_diff>
--- a/outputs/feature-matrix-2026-10-16/OM0RX-xLog_Feature_Comparison_2026-10-16.xlsx
+++ b/outputs/feature-matrix-2026-10-16/OM0RX-xLog_Feature_Comparison_2026-10-16.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Matrix" sheetId="1" r:id="Rae092293bdbf4238"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Outstanding" sheetId="2" r:id="R39af7a88d3ac4c93"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enhancement Review" sheetId="3" r:id="Ra46975ec5ec24c4a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="4" r:id="R290ab8883ae14a2e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Matrix" sheetId="1" r:id="Rd0ef692efbda426a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Outstanding" sheetId="2" r:id="R8b9505d66e4c42a8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enhancement Review" sheetId="3" r:id="Rb383682e42ac4f5a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="4" r:id="R6c02b3a01f04414e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -370,7 +370,325 @@
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
-  <x:dxfs count="10">
+  <x:dxfs count="40">
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FF087A68"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFE7F6F1"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FF087A68"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFE7F6F1"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FF163A5F"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFEAF4FB"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF8A5A00"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFFF4D6"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FF8A5A00"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFFF4D6"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FFA61B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFCE8E6"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FFA61B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFCE8E6"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF8A5A00"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFFF4D6"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FFA61B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFCE8E6"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF8A5A00"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFFF4D6"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FF087A68"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFE7F6F1"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FF087A68"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFE7F6F1"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FF163A5F"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFEAF4FB"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF8A5A00"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFFF4D6"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FF8A5A00"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFFF4D6"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FFA61B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFCE8E6"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FFA61B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFCE8E6"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF8A5A00"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFFF4D6"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FFA61B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFCE8E6"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF8A5A00"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFFF4D6"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FF087A68"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFE7F6F1"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FF087A68"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFE7F6F1"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FF163A5F"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFEAF4FB"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF8A5A00"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFFF4D6"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FF8A5A00"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFFF4D6"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FFA61B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFCE8E6"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FFA61B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFCE8E6"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF8A5A00"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFFF4D6"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FFA61B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFCE8E6"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF8A5A00"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFFF4D6"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
     <x:dxf>
       <x:font>
         <x:color rgb="FF087A68"/>
@@ -852,12 +1170,12 @@
       <x:c r="E9" s="59"/>
       <x:c r="F9" s="59"/>
     </x:row>
-    <x:row r="10" ht="108" hidden="0" customHeight="1">
+    <x:row r="10" ht="264" hidden="0" customHeight="1">
       <x:c r="A10" s="66" t="str">
         <x:v>QSO data quality findings</x:v>
       </x:c>
       <x:c r="B10" s="67" t="str">
-        <x:v>Source complete for read-only findings, exact-contact route, Details UI and bounded duplicate review. c6ada81 reuses native exact call/band/primary-mode case-insensitive +/-600-second matching, self/deleted excluded, cap 5 plus lookahead with complete/truncated/unknown states. No semantic/frequency/submode/portable-callsign inference or mutation. Existing validation, dated CTY comparisons and retained power provenance remain review evidence; CTY version/date unknown and stored/manual values authoritative. Agent core 8/8, route/regression 6/6, frontend 19/19, tsc/build/window gates; root route 3/3, duplicate 3/3, frontend 19/19 pass. Native/package/live/full-coverage/correction/provider gates stay open; no award/sync delta. Installed alpha.31 unchanged.</x:v>
+        <x:v>Source complete for read-only findings, exact-contact route, Details UI and bounded duplicate review. c6ada81 reuses native exact call/band/primary-mode case-insensitive +/-600-second matching, self/deleted excluded, cap 5 plus lookahead with complete/truncated/unknown states. No semantic/frequency/submode/portable-callsign inference or mutation. Existing validation, dated CTY comparisons and retained power provenance remain review evidence; CTY version/date unknown and stored/manual values authoritative. Agent core 8/8, route/regression 6/6, frontend 19/19, tsc/build/window gates; root route 3/3, duplicate 3/3, frontend 19/19 pass. Native/package/live/full-coverage/correction/provider gates stay open; no award/sync delta. Installed alpha.31 unchanged. 33e5eb4 adds a pure bounded contact-update validation/raw field-diff prerequisite reused by canonical apply without changing receipts/revision/save semantics. Explicit invalid/stale/protected-identity failures; literal arbitrary fields preserve absent/empty distinction; cap 128 changes and 24,576 bytes/input with truncated/unavailable states. New 6/6 plus route/contact 15/15 and root focused 6/6 pass, including DB/WAL/SHM/journal purity. Not a saved-value simulation or correction-preview route/UI; correction UI/apply/undo remain open. 8ccffe7 adds read-only CTY DXCC-only correction preview, exact-contact/generation/revision/current-comparison-evidence fenced, using the canonical finding and pure review owner (root 2/2 plus data-quality regression). Unknown source/version/date facts stay unknown; stored/manual values are unchanged. No apply/undo/UI, operation ID, receipt, journal, provider correction or live acceptance. 327648c adds compact read-only CTY DXCC preview inside existing Logbook Details only, validating exact scope/evidence (Swift 2/2, UI/bridge 22/22, tsc). No apply/undo, operation ID, receipt, journal or provider correction; package/native/copied-log/live acceptance stays open.</x:v>
       </x:c>
       <x:c r="C10" s="67" t="str">
         <x:v>Documented — QSO editing and DXCC/QSL workflows; comparable field-provenance findings were not established.</x:v>
@@ -868,12 +1186,12 @@
       <x:c r="E10" s="59"/>
       <x:c r="F10" s="59"/>
     </x:row>
-    <x:row r="11" ht="84" hidden="0" customHeight="1">
+    <x:row r="11" ht="132" hidden="0" customHeight="1">
       <x:c r="A11" s="66" t="str">
         <x:v>ADIF field preservation</x:v>
       </x:c>
       <x:c r="B11" s="67" t="str">
-        <x:v>Source complete for nine reviewed compatibility stages — local records retain a JSON field bag; unknown/custom fields, Unicode, station/contact and RX/TX data survive supported ADI/ADX round trips. UTF-8 byte scanning, FT4/FT2/JTTY MFSK-submode export, C4FM/DSTAR DIGITALVOICE-submode handling and import-only PSK31/PSK63/PSK63F/PSK125/PSKAM10 to PSK/submode normalization are fixed. Latest Swift 18/18 and frontend 1,202/1,202 and TypeScript pass at PSKAM10 (770dda2). Remaining 3.1.8 audit and package/real-log acceptance stay open; ADIF_VER stays 3.1.7.</x:v>
+        <x:v>Source complete for thirteen reviewed compatibility stages — local records retain a JSON field bag; unknown/custom fields, Unicode, station/contact and RX/TX data survive supported ADI/ADX round trips. UTF-8 byte scanning, FT4/FT2/JTTY MFSK-submode export, C4FM/DSTAR DIGITALVOICE-submode handling and import-only PSK31/PSK63/PSK63F/PSK125/PSKAM10/PSKAM31/PSKAM50/PSKFEC31 to PSK/submode normalization are fixed. PSKAM31 90f7a3e: Swift 18/18, frontend 1,218/1,218 and tsc. PSKAM50 e34a094: Swift 18/18, frontend 1,234/1,234 and tsc. PSKFEC31 8c43ef5: Swift 18/18, frontend 1,250/1,250 and tsc. PSKHELL 9e8b97b: official import-only to HELL; Swift 18/18, frontend 1,266/1,266, tsc; root reviewed/diff checked. Lexical import normalization exports canonical PSK/submode and preserves explicit submode authority. Remaining 3.1.8 audit and package/real-log acceptance stay open; ADIF_VER stays 3.1.7.</x:v>
       </x:c>
       <x:c r="C11" s="67" t="str">
         <x:v>Documented — import/export plus four user-definable logging fields.</x:v>
@@ -1332,12 +1650,12 @@
       <x:c r="E39" s="59"/>
       <x:c r="F39" s="59"/>
     </x:row>
-    <x:row r="40" ht="456" hidden="0" customHeight="1">
+    <x:row r="40" ht="276" hidden="0" customHeight="1">
       <x:c r="A40" s="66" t="str">
         <x:v>TCI rig control — SunSDR/ExpertSDR and compatible servers</x:v>
       </x:c>
       <x:c r="B40" s="67" t="str">
-        <x:v>Source complete through receive tune/filter, configured-TRX split, global TX-frequency telemetry, APP_FOCUS, addressed RX_CLICKED_ON_SPOT, legacy CLICKED_ON_SPOT and receipt-only CW_MACROS_EMPTY and opaque CALLSIGN_SEND and per-address VFO_LOCK plus RX_CHANNEL_SENSORS and separate deprecated RX_SENSORS plus formal-five-field TX_SENSORS token observations. Passive notifications retain independent producer receipts; legacy clicks infer no TRX/channel/VFO. CW_MACROS_EMPTY proves no queue-empty, TX/RX, CW or RF authority. APP_FOCUS Swift 45/45, legacy-click 50/50 (lifecycle rerun) CW receipt 55/55 and CALLSIGN_SEND 60/60 (34 protocol + 26 session) pass. CALLSIGN_SEND uses strict validation/reconnect clearing and confers no target/contact identity authority, command correlation, TX completion/success or RF inference. VFO_LOCK 66/66 (38 protocol + 28 session) retains independent exact-address producer times, validates exactly three arguments within application/discovery bounds, prunes on discovery shrink and clears on reconnect. It grants no owner/expiry, tune confirmation, configured freshness or control authority. RX_CHANNEL_SENSORS preserves exact bounded ASCII decimals per address without Double conversion or physical range/calibration/quality/readiness/freshness/control claims; discovery prunes and reconnect clears. Six new tests pass twice, protocol 42/42; broader session rerun at ed8ed37 was 71/72 on unchanged testDroppingLastSessionReferenceClosesPendingConnection (closeCount 0 vs 1); initial existing tune-yield miss passed rerun. Build/diff clean. 2d7bb1f adds deprecated server-only RX_SENSORS as separate per-TRX raw bounded decimal tokens plus local producer receipt, never channel-attributed or merged with RX_CHANNEL_SENSORS. TRX discovery prunes, channel-count changes do not remap and reconnect clears. No physical range/calibration/readiness/freshness/control/RF inference. Later independent focused tests 78/78 pass; earlier timing miss is not claimed fixed. dbf6e36 adds passive formal-five-field TX_SENSORS raw per-TRX receipts (84/84); malformed printed example rejects and no TX/RF/physical power/SWR authority is inferred. Explicit controls retain the existing no-replay/readback owner. Transmit/PTT, split/TX-VFO controls, outbound spots, audio/IQ and package/live-server/RF acceptance remain open. 711d4c4 retains global MUTE from pinned TCI pp 21–22 with own receipt, strict bool and reconnect clear; no encoder/query/setter/control/configured readiness/tune/TX/RF effect. New 5/5 and protocol 53/53 pass; broad 88/89 retains unchanged lifecycle closeCount 0 vs 1. Root combined-tree new 5/5 passes after R10 test compile fixes, not a lifecycle fix. 46c862b separately observes RX_MUTE for exact receiver/strict bool, with independent receipts, pruning/reconnect clearing and no configured freshness/readiness/tune/TX/control/RF authority. Agent 95/95 and root new 6/6 pass. Earlier lifecycle flake and package/live gates stay disclosed. ec83f28 passively observes global VOLUME as exact raw decimal [-60,0] dB plus receipt, without mute/audibility/streaming/readiness/control/RF inference. Agent compiled bundle 101/101 and root full-current-tree new 6/6 pass; earlier lifecycle flake remains disclosed.</x:v>
+        <x:v>Source complete for receive tune/filter, passive configured-TRX split/TX-frequency, APP_FOCUS, addressed/legacy spot clicks, receipt-only CW_MACROS_EMPTY/CALLSIGN_SEND, per-address VFO_LOCK, RX_CHANNEL_SENSORS, separate deprecated RX_SENSORS, formal-five-field TX_SENSORS, global MUTE/VOLUME and receiver RX_MUTE observations. Independent raw tokens/producer receipts do not establish physical power/calibration, queue-empty, contact identity, command correlation, configured freshness/readiness, control, TX completion or RF authority. 4a34eb4 adds passive RX_VOLUME exact raw [-60,0] dB per receiver/channel (agent 107/107; root focused 6/6). 63ef8b2 separately adds RX_BALANCE exact raw [-40,40] dB per receiver/channel (agent 113/113; root focused 6/6). Both have independent receipts, discovery-shrink pruning and reconnect clearing; no global mute/volume relationships, measured stereo output, audibility or streaming inference. Existing no-replay/readback owner is unchanged. Recurring testDroppingLastSessionReferenceClosesPendingConnection closeCount 0 vs 1 failure remains open; passing focused checks are not a lifecycle fix. Transmit/PTT, split/TX-VFO controls, outbound spots, audio/IQ and package/native/live station/provider/network/RF acceptance remain open. Earlier source/test history is retained in project tracking docs. Installed alpha.31 unchanged. d2b2d24 adds independent passive global MON_VOLUME exact raw [-60,0] dB with its own receipt/reconnect reset (agent 118/118; root focused 5/5). No relationship to other audio/mute and no monitoring/TX/readiness/RF inference; package/native/live acceptance stays open. c54cc0f adds passive global MON_ENABLE exact boolean token plus parsed setting, independent receipt/reset (agent 123/123; root focused 5/5). Independent of MON_VOLUME; no monitoring/audibility/streaming/TX/readiness/control/RF inference.</x:v>
       </x:c>
       <x:c r="C40" s="67" t="str">
         <x:v>Not established in the reviewed primary RUMlogNG evidence.</x:v>
@@ -2737,16 +3055,16 @@
     <x:mergeCell ref="A3:D3"/>
   </x:mergeCells>
   <x:conditionalFormatting sqref="B7:B53">
-    <x:cfRule type="beginsWith" dxfId="0" priority="1" operator="beginsWith" text="Installed"/>
-    <x:cfRule type="beginsWith" dxfId="1" priority="2" operator="beginsWith" text="Implemented"/>
-    <x:cfRule type="beginsWith" dxfId="2" priority="3" operator="beginsWith" text="Source complete"/>
-    <x:cfRule type="beginsWith" dxfId="3" priority="4" operator="beginsWith" text="Active"/>
-    <x:cfRule type="beginsWith" dxfId="4" priority="5" operator="beginsWith" text="Partial"/>
-    <x:cfRule type="beginsWith" dxfId="5" priority="6" operator="beginsWith" text="Outstanding"/>
+    <x:cfRule type="beginsWith" dxfId="30" priority="1" operator="beginsWith" text="Installed"/>
+    <x:cfRule type="beginsWith" dxfId="31" priority="2" operator="beginsWith" text="Implemented"/>
+    <x:cfRule type="beginsWith" dxfId="32" priority="3" operator="beginsWith" text="Source complete"/>
+    <x:cfRule type="beginsWith" dxfId="33" priority="4" operator="beginsWith" text="Active"/>
+    <x:cfRule type="beginsWith" dxfId="34" priority="5" operator="beginsWith" text="Partial"/>
+    <x:cfRule type="beginsWith" dxfId="35" priority="6" operator="beginsWith" text="Outstanding"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd346a346163d4c86"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R46235a6c54b54416"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2930,7 +3248,7 @@
         <x:v>RUMlogNG edit/search/export workflow</x:v>
       </x:c>
     </x:row>
-    <x:row r="12" ht="36" hidden="0" customHeight="1">
+    <x:row r="12" ht="84" hidden="0" customHeight="1">
       <x:c r="A12" s="66" t="str">
         <x:v>P0</x:v>
       </x:c>
@@ -2938,10 +3256,10 @@
         <x:v>ADIF 3.1.8 conformance</x:v>
       </x:c>
       <x:c r="C12" s="67" t="str">
-        <x:v>Nine compatibility stages complete</x:v>
+        <x:v>Thirteen compatibility stages complete</x:v>
       </x:c>
       <x:c r="D12" s="67" t="str">
-        <x:v>Complete the remaining enum/deprecation and MODE/SUBMODE audit before changing ADIF_VER; run copied-log/package and service-specific interoperability acceptance.</x:v>
+        <x:v>Complete the remaining enum/deprecation and MODE/SUBMODE audit before changing ADIF_VER; run copied-log/package and service-specific interoperability acceptance. PSKAM31 90f7a3e: Swift 18/18, frontend 1,218/1,218, tsc; PSKAM50 e34a094: Swift 18/18, frontend 1,234/1,234, tsc. Source evidence only. PSKFEC31 8c43ef5: Swift 18/18, frontend 1,250/1,250, tsc; ADIF_VER stays 3.1.7. PSKHELL 9e8b97b: official import-only to HELL, Swift 18/18, frontend 1,266/1,266, tsc; root reviewed/diff checked.</x:v>
       </x:c>
       <x:c r="E12" s="67" t="str">
         <x:v>Pinned official fixtures, copied-log round trip and exact package</x:v>
@@ -2970,7 +3288,7 @@
         <x:v>Official/date-qualified CTY rules</x:v>
       </x:c>
     </x:row>
-    <x:row r="14" ht="288" hidden="0" customHeight="1">
+    <x:row r="14" ht="312" hidden="0" customHeight="1">
       <x:c r="A14" s="66" t="str">
         <x:v>P1</x:v>
       </x:c>
@@ -2978,7 +3296,7 @@
         <x:v>Full TCI radio provider</x:v>
       </x:c>
       <x:c r="C14" s="67" t="str">
-        <x:v>Receive tune/filter plus passive split, TX-frequency, APP_FOCUS, addressed/legacy spot-click CW_MACROS_EMPTY receipt and opaque CALLSIGN_SEND plus VFO_LOCK, RX_CHANNEL_SENSORS and separate deprecated RX_SENSORS plus formal-five-field TX_SENSORS tokens source complete; latest focused tests 84/84; passive global MUTE source complete (broad gate88/89, new 5/5 root rerun); exact-receiver RX_MUTE source complete (agent 95/95, root new 6/6); passive global VOLUME source complete (agent compiled 101/101, root new 6/6)</x:v>
+        <x:v>Receive tune/filter and bounded passive telemetry source complete; full history in project docs. RX_VOLUME 4a34eb4: raw [-60,0] dB/address, agent 107/107 + root 6/6. RX_BALANCE 63ef8b2: raw [-40,40] dB/address, agent 113/113 + root 6/6. MON_VOLUME d2b2d24: independent global raw [-60,0] dB/receipt/reset, agent 118/118 + root 5/5. MON_ENABLE c54cc0f: separate global exact bool/parsed setting/receipt/reset, agent 123/123 + root 5/5. No audio/mute relationships or monitoring/audibility/streaming/TX/readiness/control/RF inference. closeCount 0 vs 1 lifecycle failure and package/native/live station/provider/network/RF gates remain open.</x:v>
       </x:c>
       <x:c r="D14" s="67" t="str">
         <x:v>Extend the existing no-replay owner with separately reviewed split/TX-VFO controls, urgent release and optional audio/IQ slices; passive notifications never become configured evidence/inventory or CW/RF authority. Transmit/PTT keeps its own explicit authority.</x:v>
@@ -4639,16 +4957,16 @@
     <x:mergeCell ref="A3:F3"/>
   </x:mergeCells>
   <x:conditionalFormatting sqref="A7:A27">
-    <x:cfRule type="cellIs" dxfId="6" priority="1" operator="equal">
+    <x:cfRule type="cellIs" dxfId="36" priority="1" operator="equal">
       <x:formula>"P0"</x:formula>
     </x:cfRule>
-    <x:cfRule type="cellIs" dxfId="7" priority="2" operator="equal">
+    <x:cfRule type="cellIs" dxfId="37" priority="2" operator="equal">
       <x:formula>"P1"</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7b2e5737facf4cef"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reeae2fe0e50345b4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4783,7 +5101,7 @@
       </x:c>
       <x:c r="F9" s="59"/>
     </x:row>
-    <x:row r="10" ht="24" hidden="0" customHeight="1">
+    <x:row r="10" ht="60" hidden="0" customHeight="1">
       <x:c r="A10" s="66" t="str">
         <x:v>R04</x:v>
       </x:c>
@@ -4791,13 +5109,13 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="C10" s="67" t="str">
-        <x:v>Nine compatibility stages complete</x:v>
+        <x:v>Thirteen compatibility stages complete</x:v>
       </x:c>
       <x:c r="D10" s="67" t="str">
         <x:v>ADIF parser/writer and frontend transfer</x:v>
       </x:c>
       <x:c r="E10" s="67" t="str">
-        <x:v>Finish remaining 3.1.8 audit after PSK63/PSK63F/PSK125/PSKAM10; retain ADIF_VER 3.1.7.</x:v>
+        <x:v>PSKAM31 90f7a3e: Swift 18/18, frontend 1,218/1,218, tsc. PSKAM50 e34a094: Swift 18/18, frontend 1,234/1,234, tsc. Finish remaining 3.1.8 audit/copied-log/package acceptance; retain ADIF_VER 3.1.7. PSKFEC31 8c43ef5: Swift 18/18, frontend 1,250/1,250, tsc; import-only to PSK. PSKHELL 9e8b97b: import-only to HELL, Swift 18/18, frontend 1,266/1,266, tsc; root reviewed/diff checked.</x:v>
       </x:c>
       <x:c r="F10" s="59"/>
     </x:row>
@@ -4891,7 +5209,7 @@
       </x:c>
       <x:c r="F15" s="59"/>
     </x:row>
-    <x:row r="16" ht="48" hidden="0" customHeight="1">
+    <x:row r="16" ht="144" hidden="0" customHeight="1">
       <x:c r="A16" s="66" t="str">
         <x:v>R10</x:v>
       </x:c>
@@ -4899,13 +5217,13 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="C16" s="67" t="str">
-        <x:v>Read-only findings/UI and bounded duplicate review source complete; acceptance/corrections open</x:v>
+        <x:v>Read-only findings/duplicate review, pure helper and CTY DXCC-only preview UI source complete; apply/undo open</x:v>
       </x:c>
       <x:c r="D16" s="67" t="str">
-        <x:v>Exact-contact canonical route, native duplicate rule and Logbook Details</x:v>
+        <x:v>Exact-contact canonical route, native duplicate rule, Details and canonical contact-update owner</x:v>
       </x:c>
       <x:c r="E16" s="67" t="str">
-        <x:v>c6ada81: exact call/band/primary-mode, +/-600s, cap 5 + lookahead, complete/truncated/unknown; agent core 8/8, route 6/6, frontend 19/19, tsc/build/windows; root route 3/3+duplicate 3/3+frontend 19/19. Next native/package/live/full coverage; no mutations/delta.</x:v>
+        <x:v>33e5eb4: zero-write bounded validation/raw diff reused by canonical apply unchanged; new 6/6 + route/contact 15/15, root focused 6/6, DB/WAL/SHM/journal purity. The helper is not saved-value simulation. Correction apply/undo and package/native/live/full coverage remain open. 8ccffe7 adds read-only CTY DXCC-only correction preview, exact-contact/generation/revision/current-comparison-evidence fenced, using the canonical finding and pure review owner (root 2/2 plus data-quality regression). Unknown source/version/date facts stay unknown; stored/manual values are unchanged. No apply/undo/UI, operation ID, receipt, journal, provider correction or live acceptance. 327648c adds compact read-only CTY DXCC preview inside existing Logbook Details only, validating exact scope/evidence (Swift 2/2, UI/bridge 22/22, tsc). No apply/undo, operation ID, receipt, journal or provider correction; package/native/copied-log/live acceptance stays open.</x:v>
       </x:c>
       <x:c r="F16" s="59"/>
     </x:row>
@@ -6526,16 +6844,16 @@
     <x:mergeCell ref="A3:E3"/>
   </x:mergeCells>
   <x:conditionalFormatting sqref="B7:B30">
-    <x:cfRule type="cellIs" dxfId="8" priority="1" operator="equal">
+    <x:cfRule type="cellIs" dxfId="38" priority="1" operator="equal">
       <x:formula>"P0"</x:formula>
     </x:cfRule>
-    <x:cfRule type="cellIs" dxfId="9" priority="2" operator="equal">
+    <x:cfRule type="cellIs" dxfId="39" priority="2" operator="equal">
       <x:formula>"P1"</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ref45cc0695f242a7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R41601e2d31994311"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6615,7 +6933,7 @@
         <x:v>OM0RX-xLog</x:v>
       </x:c>
       <x:c r="B7" s="65" t="str">
-        <x:v>Current implementation checkpoint c6ada81ae2b90dba15f8d531cabe8524596f9527</x:v>
+        <x:v>Current implementation checkpoint c54cc0f6ff68bc6108fb85fceec30402f4fd6615</x:v>
       </x:c>
       <x:c r="C7" s="65" t="str">
         <x:v>2026-10-16</x:v>
@@ -6626,18 +6944,18 @@
       <x:c r="E7" s="59"/>
       <x:c r="F7" s="59"/>
     </x:row>
-    <x:row r="8" ht="60" hidden="0" customHeight="1">
+    <x:row r="8" ht="168" hidden="0" customHeight="1">
       <x:c r="A8" s="66" t="str">
         <x:v>OM0RX-xLog</x:v>
       </x:c>
       <x:c r="B8" s="67" t="str">
-        <x:v>https://github.com/oliverbross/OM0RX-xLog/commit/c6ada81ae2b90dba15f8d531cabe8524596f9527</x:v>
+        <x:v>https://github.com/oliverbross/OM0RX-xLog/commit/c54cc0f6ff68bc6108fb85fceec30402f4fd6615</x:v>
       </x:c>
       <x:c r="C8" s="67" t="str">
         <x:v>2026-10-16</x:v>
       </x:c>
       <x:c r="D8" s="67" t="str">
-        <x:v>Latest separate stages: passive raw global VOLUME (ec83f28; exact [-60,0] dB token/receipt, agent compiled 101/101, root current-tree new 6/6) and bounded native-rule duplicate review (c6ada81; agent core 8/8, route 6/6, frontend 19/19, root route 3/3+duplicate 3/3+frontend 19/19, tsc/build/window gates). Installed alpha.31 and ADIF_VER 3.1.7 unchanged; lifecycle flake remains disclosed. Native/package/live/correction/provider gates remain open.</x:v>
+        <x:v>Accepted source increments after tracking 3acfc4d: RX_VOLUME 4a34eb4 (107/107 + root 6/6); PSKAM31 90f7a3e (Swift 18/18, frontend 1,218/1,218, tsc); PSKAM50 e34a094 (Swift 18/18, frontend 1,234/1,234, tsc); pure contact-update validation/diff 33e5eb4 (new 6/6 + regressions 15/15, root 6/6); RX_BALANCE 63ef8b2 (113/113 + root 6/6). Focused/source-level evidence only. Installed alpha.31 and ADIF_VER 3.1.7 unchanged; recurring closeCount lifecycle failure, correction UI/apply/undo, package/native/live station/provider/network/RF acceptance remain open. Later increments: PSKFEC31 8c43ef5 (Swift 18/18, frontend 1,250/1,250, tsc); MON_VOLUME d2b2d24 (118/118 + root 5/5); exact-evidence-fenced CTY DXCC-only correction preview 8ccffe7 (root 2/2 plus data-quality regression), without apply/undo/UI/operation ID/receipt/journal/provider correction or live acceptance. New source increments: Details-only CTY DXCC preview UI 327648c (Swift 2/2, UI/bridge 22/22, tsc; no apply/undo); PSKHELL 9e8b97b import-only to HELL (Swift 18/18, frontend 1,266/1,266, tsc; root reviewed/diff checked); passive MON_ENABLE c54cc0f (123/123 + root 5/5), independent setting/receipt/reset with no monitoring/audibility/streaming/TX/readiness/control/RF inference. ADIF_VER remains 3.1.7; installed alpha.31 unchanged.</x:v>
       </x:c>
       <x:c r="E8" s="59"/>
       <x:c r="F8" s="59"/>
@@ -8264,7 +8582,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R496c538a4de94f81"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5494f4c6af1c4ccc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Update implementation evidence through AGC mode
</commit_message>
<xml_diff>
--- a/outputs/feature-matrix-2026-10-16/OM0RX-xLog_Feature_Comparison_2026-10-16.xlsx
+++ b/outputs/feature-matrix-2026-10-16/OM0RX-xLog_Feature_Comparison_2026-10-16.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Matrix" sheetId="1" r:id="Rd0ef692efbda426a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Outstanding" sheetId="2" r:id="R8b9505d66e4c42a8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enhancement Review" sheetId="3" r:id="Rb383682e42ac4f5a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="4" r:id="R6c02b3a01f04414e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Matrix" sheetId="1" r:id="R1f707880367140ec"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Outstanding" sheetId="2" r:id="R84853679dc0f4c08"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enhancement Review" sheetId="3" r:id="R93b4f8c4afda4f89"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="4" r:id="Ra6c2289a0db44ed6"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -370,7 +370,113 @@
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
-  <x:dxfs count="40">
+  <x:dxfs count="50">
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FF087A68"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFE7F6F1"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FF087A68"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFE7F6F1"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FF163A5F"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFEAF4FB"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF8A5A00"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFFF4D6"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:color rgb="FF8A5A00"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFFF4D6"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FFA61B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFCE8E6"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FFA61B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFCE8E6"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF8A5A00"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFFF4D6"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FFA61B1B"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFCE8E6"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF8A5A00"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFFF4D6"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
     <x:dxf>
       <x:font>
         <x:color rgb="FF087A68"/>
@@ -1186,12 +1292,12 @@
       <x:c r="E10" s="59"/>
       <x:c r="F10" s="59"/>
     </x:row>
-    <x:row r="11" ht="132" hidden="0" customHeight="1">
+    <x:row r="11" ht="156" hidden="0" customHeight="1">
       <x:c r="A11" s="66" t="str">
         <x:v>ADIF field preservation</x:v>
       </x:c>
       <x:c r="B11" s="67" t="str">
-        <x:v>Source complete for thirteen reviewed compatibility stages — local records retain a JSON field bag; unknown/custom fields, Unicode, station/contact and RX/TX data survive supported ADI/ADX round trips. UTF-8 byte scanning, FT4/FT2/JTTY MFSK-submode export, C4FM/DSTAR DIGITALVOICE-submode handling and import-only PSK31/PSK63/PSK63F/PSK125/PSKAM10/PSKAM31/PSKAM50/PSKFEC31 to PSK/submode normalization are fixed. PSKAM31 90f7a3e: Swift 18/18, frontend 1,218/1,218 and tsc. PSKAM50 e34a094: Swift 18/18, frontend 1,234/1,234 and tsc. PSKFEC31 8c43ef5: Swift 18/18, frontend 1,250/1,250 and tsc. PSKHELL 9e8b97b: official import-only to HELL; Swift 18/18, frontend 1,266/1,266, tsc; root reviewed/diff checked. Lexical import normalization exports canonical PSK/submode and preserves explicit submode authority. Remaining 3.1.8 audit and package/real-log acceptance stay open; ADIF_VER stays 3.1.7.</x:v>
+        <x:v>Source complete for fourteen reviewed compatibility stages — local records retain a JSON field bag; unknown/custom fields, Unicode, station/contact and RX/TX data survive supported ADI/ADX round trips. UTF-8 byte scanning, FT4/FT2/JTTY MFSK-submode export, C4FM/DSTAR DIGITALVOICE-submode handling and import-only PSK31/PSK63/PSK63F/PSK125/PSKAM10/PSKAM31/PSKAM50/PSKFEC31 to PSK/submode normalization are fixed. PSKAM31 90f7a3e: Swift 18/18, frontend 1,218/1,218 and tsc. PSKAM50 e34a094: Swift 18/18, frontend 1,234/1,234 and tsc. PSKFEC31 8c43ef5: Swift 18/18, frontend 1,250/1,250 and tsc. PSKHELL 9e8b97b: official import-only to HELL; Swift 18/18, frontend 1,266/1,266, tsc; root reviewed/diff checked. QPSK31 8934ab6: official import-only to PSK/submode; agent Swift 18/18, frontend 1,282/1,282, tsc; root frontend 1,282/1,282, tsc/diff. Lexical import normalization exports canonical PSK/submode and preserves explicit submode authority. Remaining 3.1.8 audit and package/real-log acceptance stay open; ADIF_VER stays 3.1.7.</x:v>
       </x:c>
       <x:c r="C11" s="67" t="str">
         <x:v>Documented — import/export plus four user-definable logging fields.</x:v>
@@ -1330,12 +1436,12 @@
       <x:c r="E19" s="59"/>
       <x:c r="F19" s="59"/>
     </x:row>
-    <x:row r="20" ht="24" hidden="0" customHeight="1">
+    <x:row r="20" ht="72" hidden="0" customHeight="1">
       <x:c r="A20" s="66" t="str">
         <x:v>Wavelog two-way reconciliation</x:v>
       </x:c>
       <x:c r="B20" s="67" t="str">
-        <x:v>Installed / live accepted — read-first reconciliation imported safe contacts and refreshed linked confirmations/enrichment without deleting or overwriting ambiguous records.</x:v>
+        <x:v>Installed / live accepted — read-first reconciliation imported safe contacts and refreshed linked confirmations/enrichment without deleting or overwriting ambiguous records. 7adb008 adds an end-to-end synthetic Wavelog sync regression (focused 1/1): clean linked contacts receive fresh eQSL/LoTW/QRZ/message confirmation fields; local-only station/custom fields survive; no outbox/conflict; second sync idempotent. Fixture-only source evidence, not new live-provider/package acceptance.</x:v>
       </x:c>
       <x:c r="C20" s="67" t="str">
         <x:v>Not documented as a native Wavelog workflow in reviewed primary evidence.</x:v>
@@ -1346,12 +1452,12 @@
       <x:c r="E20" s="59"/>
       <x:c r="F20" s="59"/>
     </x:row>
-    <x:row r="21" ht="24" hidden="0" customHeight="1">
+    <x:row r="21" ht="72" hidden="0" customHeight="1">
       <x:c r="A21" s="66" t="str">
         <x:v>Confirmation refresh from remote services</x:v>
       </x:c>
       <x:c r="B21" s="67" t="str">
-        <x:v>Installed / live accepted through Wavelog — LoTW, eQSL, QRZ and enrichment changes update matching local QSOs while ambiguous identities remain held for review.</x:v>
+        <x:v>Installed / live accepted through Wavelog — LoTW, eQSL, QRZ and enrichment changes update matching local QSOs while ambiguous identities remain held for review. 7adb008 adds an end-to-end synthetic Wavelog sync regression (focused 1/1): clean linked contacts receive fresh eQSL/LoTW/QRZ/message confirmation fields; local-only station/custom fields survive; no outbox/conflict; second sync idempotent. Fixture-only source evidence, not new live-provider/package acceptance.</x:v>
       </x:c>
       <x:c r="C21" s="67" t="str">
         <x:v>Documented — direct LoTW/eQSL workflows and Club Log real-time synchronization.</x:v>
@@ -1650,12 +1756,12 @@
       <x:c r="E39" s="59"/>
       <x:c r="F39" s="59"/>
     </x:row>
-    <x:row r="40" ht="276" hidden="0" customHeight="1">
+    <x:row r="40" ht="300" hidden="0" customHeight="1">
       <x:c r="A40" s="66" t="str">
         <x:v>TCI rig control — SunSDR/ExpertSDR and compatible servers</x:v>
       </x:c>
       <x:c r="B40" s="67" t="str">
-        <x:v>Source complete for receive tune/filter, passive configured-TRX split/TX-frequency, APP_FOCUS, addressed/legacy spot clicks, receipt-only CW_MACROS_EMPTY/CALLSIGN_SEND, per-address VFO_LOCK, RX_CHANNEL_SENSORS, separate deprecated RX_SENSORS, formal-five-field TX_SENSORS, global MUTE/VOLUME and receiver RX_MUTE observations. Independent raw tokens/producer receipts do not establish physical power/calibration, queue-empty, contact identity, command correlation, configured freshness/readiness, control, TX completion or RF authority. 4a34eb4 adds passive RX_VOLUME exact raw [-60,0] dB per receiver/channel (agent 107/107; root focused 6/6). 63ef8b2 separately adds RX_BALANCE exact raw [-40,40] dB per receiver/channel (agent 113/113; root focused 6/6). Both have independent receipts, discovery-shrink pruning and reconnect clearing; no global mute/volume relationships, measured stereo output, audibility or streaming inference. Existing no-replay/readback owner is unchanged. Recurring testDroppingLastSessionReferenceClosesPendingConnection closeCount 0 vs 1 failure remains open; passing focused checks are not a lifecycle fix. Transmit/PTT, split/TX-VFO controls, outbound spots, audio/IQ and package/native/live station/provider/network/RF acceptance remain open. Earlier source/test history is retained in project tracking docs. Installed alpha.31 unchanged. d2b2d24 adds independent passive global MON_VOLUME exact raw [-60,0] dB with its own receipt/reconnect reset (agent 118/118; root focused 5/5). No relationship to other audio/mute and no monitoring/TX/readiness/RF inference; package/native/live acceptance stays open. c54cc0f adds passive global MON_ENABLE exact boolean token plus parsed setting, independent receipt/reset (agent 123/123; root focused 5/5). Independent of MON_VOLUME; no monitoring/audibility/streaming/TX/readiness/control/RF inference.</x:v>
+        <x:v>Source complete for receive tune/filter, passive configured-TRX split/TX-frequency, APP_FOCUS, addressed/legacy spot clicks, receipt-only CW_MACROS_EMPTY/CALLSIGN_SEND, per-address VFO_LOCK, RX_CHANNEL_SENSORS, separate deprecated RX_SENSORS, formal-five-field TX_SENSORS, global MUTE/VOLUME and receiver RX_MUTE observations. Independent raw tokens/producer receipts do not establish physical power/calibration, queue-empty, contact identity, command correlation, configured freshness/readiness, control, TX completion or RF authority. 4a34eb4 adds passive RX_VOLUME exact raw [-60,0] dB per receiver/channel (agent 107/107; root focused 6/6). 63ef8b2 separately adds RX_BALANCE exact raw [-40,40] dB per receiver/channel (agent 113/113; root focused 6/6). Both have independent receipts, discovery-shrink pruning and reconnect clearing; no global mute/volume relationships, measured stereo output, audibility or streaming inference. Existing no-replay/readback owner is unchanged. Recurring testDroppingLastSessionReferenceClosesPendingConnection closeCount 0 vs 1 failure remains open; passing focused checks are not a lifecycle fix. Transmit/PTT, split/TX-VFO controls, outbound spots, audio/IQ and package/native/live station/provider/network/RF acceptance remain open. Earlier source/test history is retained in project tracking docs. Installed alpha.31 unchanged. d2b2d24 adds independent passive global MON_VOLUME exact raw [-60,0] dB with its own receipt/reconnect reset (agent 118/118; root focused 5/5). No relationship to other audio/mute and no monitoring/TX/readiness/RF inference; package/native/live acceptance stays open. c54cc0f adds passive global MON_ENABLE exact boolean token plus parsed setting, independent receipt/reset (agent 123/123; root focused 5/5). Independent of MON_VOLUME; no monitoring/audibility/streaming/TX/readiness/control/RF inference. b1691a5 adds passive receiver AGC_MODE normal/fast/off exact token plus typed mode, independent receipt, TRX pruning/reconnect reset (agent 129/129; root focused 6/6). No gain/modulation/receiver-enable/audio/readiness/control/RF inference.</x:v>
       </x:c>
       <x:c r="C40" s="67" t="str">
         <x:v>Not established in the reviewed primary RUMlogNG evidence.</x:v>
@@ -3055,16 +3161,16 @@
     <x:mergeCell ref="A3:D3"/>
   </x:mergeCells>
   <x:conditionalFormatting sqref="B7:B53">
-    <x:cfRule type="beginsWith" dxfId="30" priority="1" operator="beginsWith" text="Installed"/>
-    <x:cfRule type="beginsWith" dxfId="31" priority="2" operator="beginsWith" text="Implemented"/>
-    <x:cfRule type="beginsWith" dxfId="32" priority="3" operator="beginsWith" text="Source complete"/>
-    <x:cfRule type="beginsWith" dxfId="33" priority="4" operator="beginsWith" text="Active"/>
-    <x:cfRule type="beginsWith" dxfId="34" priority="5" operator="beginsWith" text="Partial"/>
-    <x:cfRule type="beginsWith" dxfId="35" priority="6" operator="beginsWith" text="Outstanding"/>
+    <x:cfRule type="beginsWith" dxfId="40" priority="1" operator="beginsWith" text="Installed"/>
+    <x:cfRule type="beginsWith" dxfId="41" priority="2" operator="beginsWith" text="Implemented"/>
+    <x:cfRule type="beginsWith" dxfId="42" priority="3" operator="beginsWith" text="Source complete"/>
+    <x:cfRule type="beginsWith" dxfId="43" priority="4" operator="beginsWith" text="Active"/>
+    <x:cfRule type="beginsWith" dxfId="44" priority="5" operator="beginsWith" text="Partial"/>
+    <x:cfRule type="beginsWith" dxfId="45" priority="6" operator="beginsWith" text="Outstanding"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R46235a6c54b54416"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rff5f82e80c5d4779"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3248,7 +3354,7 @@
         <x:v>RUMlogNG edit/search/export workflow</x:v>
       </x:c>
     </x:row>
-    <x:row r="12" ht="84" hidden="0" customHeight="1">
+    <x:row r="12" ht="108" hidden="0" customHeight="1">
       <x:c r="A12" s="66" t="str">
         <x:v>P0</x:v>
       </x:c>
@@ -3256,10 +3362,10 @@
         <x:v>ADIF 3.1.8 conformance</x:v>
       </x:c>
       <x:c r="C12" s="67" t="str">
-        <x:v>Thirteen compatibility stages complete</x:v>
+        <x:v>Fourteen compatibility stages complete</x:v>
       </x:c>
       <x:c r="D12" s="67" t="str">
-        <x:v>Complete the remaining enum/deprecation and MODE/SUBMODE audit before changing ADIF_VER; run copied-log/package and service-specific interoperability acceptance. PSKAM31 90f7a3e: Swift 18/18, frontend 1,218/1,218, tsc; PSKAM50 e34a094: Swift 18/18, frontend 1,234/1,234, tsc. Source evidence only. PSKFEC31 8c43ef5: Swift 18/18, frontend 1,250/1,250, tsc; ADIF_VER stays 3.1.7. PSKHELL 9e8b97b: official import-only to HELL, Swift 18/18, frontend 1,266/1,266, tsc; root reviewed/diff checked.</x:v>
+        <x:v>Complete the remaining enum/deprecation and MODE/SUBMODE audit before changing ADIF_VER; run copied-log/package and service-specific interoperability acceptance. PSKAM31 90f7a3e: Swift 18/18, frontend 1,218/1,218, tsc; PSKAM50 e34a094: Swift 18/18, frontend 1,234/1,234, tsc. Source evidence only. PSKFEC31 8c43ef5: Swift 18/18, frontend 1,250/1,250, tsc; ADIF_VER stays 3.1.7. PSKHELL 9e8b97b: official import-only to HELL, Swift 18/18, frontend 1,266/1,266, tsc; root reviewed/diff checked. QPSK31 8934ab6: official import-only to PSK, agent Swift 18/18, frontend 1,282/1,282, tsc; root frontend 1,282/1,282, tsc/diff. ADIF_VER 3.1.7 unchanged.</x:v>
       </x:c>
       <x:c r="E12" s="67" t="str">
         <x:v>Pinned official fixtures, copied-log round trip and exact package</x:v>
@@ -3296,7 +3402,7 @@
         <x:v>Full TCI radio provider</x:v>
       </x:c>
       <x:c r="C14" s="67" t="str">
-        <x:v>Receive tune/filter and bounded passive telemetry source complete; full history in project docs. RX_VOLUME 4a34eb4: raw [-60,0] dB/address, agent 107/107 + root 6/6. RX_BALANCE 63ef8b2: raw [-40,40] dB/address, agent 113/113 + root 6/6. MON_VOLUME d2b2d24: independent global raw [-60,0] dB/receipt/reset, agent 118/118 + root 5/5. MON_ENABLE c54cc0f: separate global exact bool/parsed setting/receipt/reset, agent 123/123 + root 5/5. No audio/mute relationships or monitoring/audibility/streaming/TX/readiness/control/RF inference. closeCount 0 vs 1 lifecycle failure and package/native/live station/provider/network/RF gates remain open.</x:v>
+        <x:v>Receive tune/filter and bounded passive telemetry source complete; full history/counts in project docs and Feature Matrix. Independent RX_VOLUME/RX_BALANCE, global MON_VOLUME (d2b2d24: 118/118 + root 5/5) and MON_ENABLE (c54cc0f: 123/123 + root 5/5) receipts/reset confer no audio/monitoring authority. AGC_MODE b1691a5: receiver normal/fast/off exact token/typed mode, independent receipt, TRX pruning/reset; agent 129/129 + root 6/6. No gain/modulation/receiver-enable/audio/readiness/control/RF inference. closeCount 0 vs 1 lifecycle failure and package/native/live station/provider/network/RF gates remain open.</x:v>
       </x:c>
       <x:c r="D14" s="67" t="str">
         <x:v>Extend the existing no-replay owner with separately reviewed split/TX-VFO controls, urgent release and optional audio/IQ slices; passive notifications never become configured evidence/inventory or CW/RF authority. Transmit/PTT keeps its own explicit authority.</x:v>
@@ -4957,16 +5063,16 @@
     <x:mergeCell ref="A3:F3"/>
   </x:mergeCells>
   <x:conditionalFormatting sqref="A7:A27">
-    <x:cfRule type="cellIs" dxfId="36" priority="1" operator="equal">
+    <x:cfRule type="cellIs" dxfId="46" priority="1" operator="equal">
       <x:formula>"P0"</x:formula>
     </x:cfRule>
-    <x:cfRule type="cellIs" dxfId="37" priority="2" operator="equal">
+    <x:cfRule type="cellIs" dxfId="47" priority="2" operator="equal">
       <x:formula>"P1"</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reeae2fe0e50345b4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R54539ca392bc42bf"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5101,7 +5207,7 @@
       </x:c>
       <x:c r="F9" s="59"/>
     </x:row>
-    <x:row r="10" ht="60" hidden="0" customHeight="1">
+    <x:row r="10" ht="84" hidden="0" customHeight="1">
       <x:c r="A10" s="66" t="str">
         <x:v>R04</x:v>
       </x:c>
@@ -5109,13 +5215,13 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="C10" s="67" t="str">
-        <x:v>Thirteen compatibility stages complete</x:v>
+        <x:v>Fourteen compatibility stages complete</x:v>
       </x:c>
       <x:c r="D10" s="67" t="str">
         <x:v>ADIF parser/writer and frontend transfer</x:v>
       </x:c>
       <x:c r="E10" s="67" t="str">
-        <x:v>PSKAM31 90f7a3e: Swift 18/18, frontend 1,218/1,218, tsc. PSKAM50 e34a094: Swift 18/18, frontend 1,234/1,234, tsc. Finish remaining 3.1.8 audit/copied-log/package acceptance; retain ADIF_VER 3.1.7. PSKFEC31 8c43ef5: Swift 18/18, frontend 1,250/1,250, tsc; import-only to PSK. PSKHELL 9e8b97b: import-only to HELL, Swift 18/18, frontend 1,266/1,266, tsc; root reviewed/diff checked.</x:v>
+        <x:v>PSKAM31 90f7a3e: Swift 18/18, frontend 1,218/1,218, tsc. PSKAM50 e34a094: Swift 18/18, frontend 1,234/1,234, tsc. Finish remaining 3.1.8 audit/copied-log/package acceptance; retain ADIF_VER 3.1.7. PSKFEC31 8c43ef5: Swift 18/18, frontend 1,250/1,250, tsc; import-only to PSK. PSKHELL 9e8b97b: import-only to HELL, Swift 18/18, frontend 1,266/1,266, tsc; root reviewed/diff checked. QPSK31 8934ab6: import-only to PSK; agent Swift 18/18, frontend 1,282/1,282, tsc; root frontend 1,282/1,282, tsc/diff. ADIF_VER 3.1.7.</x:v>
       </x:c>
       <x:c r="F10" s="59"/>
     </x:row>
@@ -5155,7 +5261,7 @@
       </x:c>
       <x:c r="F12" s="59"/>
     </x:row>
-    <x:row r="13" ht="24" hidden="0" customHeight="1">
+    <x:row r="13" ht="72" hidden="0" customHeight="1">
       <x:c r="A13" s="66" t="str">
         <x:v>R07</x:v>
       </x:c>
@@ -5169,7 +5275,7 @@
         <x:v>Sync/delivery/confirmation and award state</x:v>
       </x:c>
       <x:c r="E13" s="67" t="str">
-        <x:v>Package-test 5486aff; retain unknown provider ages/credit until timestamp and sponsor-rule contracts exist.</x:v>
+        <x:v>Package-test 5486aff; retain unknown provider ages/credit until timestamp and sponsor-rule contracts exist. 7adb008 adds an end-to-end synthetic Wavelog sync regression (focused 1/1): clean linked contacts receive fresh eQSL/LoTW/QRZ/message confirmation fields; local-only station/custom fields survive; no outbox/conflict; second sync idempotent. Fixture-only source evidence, not new live-provider/package acceptance.</x:v>
       </x:c>
       <x:c r="F13" s="59"/>
     </x:row>
@@ -6844,16 +6950,16 @@
     <x:mergeCell ref="A3:E3"/>
   </x:mergeCells>
   <x:conditionalFormatting sqref="B7:B30">
-    <x:cfRule type="cellIs" dxfId="38" priority="1" operator="equal">
+    <x:cfRule type="cellIs" dxfId="48" priority="1" operator="equal">
       <x:formula>"P0"</x:formula>
     </x:cfRule>
-    <x:cfRule type="cellIs" dxfId="39" priority="2" operator="equal">
+    <x:cfRule type="cellIs" dxfId="49" priority="2" operator="equal">
       <x:formula>"P1"</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R41601e2d31994311"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R16285621e4c84f4a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6933,7 +7039,7 @@
         <x:v>OM0RX-xLog</x:v>
       </x:c>
       <x:c r="B7" s="65" t="str">
-        <x:v>Current implementation checkpoint c54cc0f6ff68bc6108fb85fceec30402f4fd6615</x:v>
+        <x:v>Current implementation checkpoint b1691a5712ef9e8bbcd29038f12ade0954334735</x:v>
       </x:c>
       <x:c r="C7" s="65" t="str">
         <x:v>2026-10-16</x:v>
@@ -6944,18 +7050,18 @@
       <x:c r="E7" s="59"/>
       <x:c r="F7" s="59"/>
     </x:row>
-    <x:row r="8" ht="168" hidden="0" customHeight="1">
+    <x:row r="8" ht="228" hidden="0" customHeight="1">
       <x:c r="A8" s="66" t="str">
         <x:v>OM0RX-xLog</x:v>
       </x:c>
       <x:c r="B8" s="67" t="str">
-        <x:v>https://github.com/oliverbross/OM0RX-xLog/commit/c54cc0f6ff68bc6108fb85fceec30402f4fd6615</x:v>
+        <x:v>https://github.com/oliverbross/OM0RX-xLog/commit/b1691a5712ef9e8bbcd29038f12ade0954334735</x:v>
       </x:c>
       <x:c r="C8" s="67" t="str">
         <x:v>2026-10-16</x:v>
       </x:c>
       <x:c r="D8" s="67" t="str">
-        <x:v>Accepted source increments after tracking 3acfc4d: RX_VOLUME 4a34eb4 (107/107 + root 6/6); PSKAM31 90f7a3e (Swift 18/18, frontend 1,218/1,218, tsc); PSKAM50 e34a094 (Swift 18/18, frontend 1,234/1,234, tsc); pure contact-update validation/diff 33e5eb4 (new 6/6 + regressions 15/15, root 6/6); RX_BALANCE 63ef8b2 (113/113 + root 6/6). Focused/source-level evidence only. Installed alpha.31 and ADIF_VER 3.1.7 unchanged; recurring closeCount lifecycle failure, correction UI/apply/undo, package/native/live station/provider/network/RF acceptance remain open. Later increments: PSKFEC31 8c43ef5 (Swift 18/18, frontend 1,250/1,250, tsc); MON_VOLUME d2b2d24 (118/118 + root 5/5); exact-evidence-fenced CTY DXCC-only correction preview 8ccffe7 (root 2/2 plus data-quality regression), without apply/undo/UI/operation ID/receipt/journal/provider correction or live acceptance. New source increments: Details-only CTY DXCC preview UI 327648c (Swift 2/2, UI/bridge 22/22, tsc; no apply/undo); PSKHELL 9e8b97b import-only to HELL (Swift 18/18, frontend 1,266/1,266, tsc; root reviewed/diff checked); passive MON_ENABLE c54cc0f (123/123 + root 5/5), independent setting/receipt/reset with no monitoring/audibility/streaming/TX/readiness/control/RF inference. ADIF_VER remains 3.1.7; installed alpha.31 unchanged.</x:v>
+        <x:v>Accepted source increments after tracking 3acfc4d: RX_VOLUME 4a34eb4 (107/107 + root 6/6); PSKAM31 90f7a3e (Swift 18/18, frontend 1,218/1,218, tsc); PSKAM50 e34a094 (Swift 18/18, frontend 1,234/1,234, tsc); pure contact-update validation/diff 33e5eb4 (new 6/6 + regressions 15/15, root 6/6); RX_BALANCE 63ef8b2 (113/113 + root 6/6). Focused/source-level evidence only. Installed alpha.31 and ADIF_VER 3.1.7 unchanged; recurring closeCount lifecycle failure, correction UI/apply/undo, package/native/live station/provider/network/RF acceptance remain open. Later increments: PSKFEC31 8c43ef5 (Swift 18/18, frontend 1,250/1,250, tsc); MON_VOLUME d2b2d24 (118/118 + root 5/5); exact-evidence-fenced CTY DXCC-only correction preview 8ccffe7 (root 2/2 plus data-quality regression), without apply/undo/UI/operation ID/receipt/journal/provider correction or live acceptance. New source increments: Details-only CTY DXCC preview UI 327648c (Swift 2/2, UI/bridge 22/22, tsc; no apply/undo); PSKHELL 9e8b97b import-only to HELL (Swift 18/18, frontend 1,266/1,266, tsc; root reviewed/diff checked); passive MON_ENABLE c54cc0f (123/123 + root 5/5), independent setting/receipt/reset with no monitoring/audibility/streaming/TX/readiness/control/RF inference. ADIF_VER remains 3.1.7; installed alpha.31 unchanged. Since c54cc0f: synthetic Wavelog confirmation-refresh regression 7adb008 (1/1; preserved local-only fields, no outbox/conflict, idempotent second sync; no live provider); QPSK31 8934ab6 import-only to PSK (agent Swift 18/18, frontend 1,282/1,282, tsc; root frontend 1,282/1,282, tsc/diff); passive receiver AGC_MODE b1691a5 (129/129 + root 6/6; exact token/typed mode, independent receipt/TRX pruning/reset; no gain/modulation/receiver-enable/audio/readiness/control/RF inference). All existing acceptance limits remain open.</x:v>
       </x:c>
       <x:c r="E8" s="59"/>
       <x:c r="F8" s="59"/>
@@ -8582,7 +8688,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5494f4c6af1c4ccc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdfb797c89d93414b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add OpsLog as supplementary feature reference
</commit_message>
<xml_diff>
--- a/outputs/feature-matrix-2026-10-16/OM0RX-xLog_Feature_Comparison_2026-10-16.xlsx
+++ b/outputs/feature-matrix-2026-10-16/OM0RX-xLog_Feature_Comparison_2026-10-16.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Matrix" sheetId="1" r:id="R1f707880367140ec"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Outstanding" sheetId="2" r:id="R84853679dc0f4c08"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enhancement Review" sheetId="3" r:id="R93b4f8c4afda4f89"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="4" r:id="Ra6c2289a0db44ed6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Matrix" sheetId="1" r:id="R769cd6cdc2f342d1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Outstanding" sheetId="2" r:id="R8939dabb8b62478b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enhancement Review" sheetId="3" r:id="Rd3fa8452d55d4dc3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="4" r:id="R35f3bc2b727a4647"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -370,431 +370,7 @@
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
-  <x:dxfs count="50">
-    <x:dxf>
-      <x:font>
-        <x:color rgb="FF087A68"/>
-      </x:font>
-      <x:fill>
-        <x:patternFill>
-          <x:bgColor rgb="FFE7F6F1"/>
-        </x:patternFill>
-      </x:fill>
-    </x:dxf>
-    <x:dxf>
-      <x:font>
-        <x:color rgb="FF087A68"/>
-      </x:font>
-      <x:fill>
-        <x:patternFill>
-          <x:bgColor rgb="FFE7F6F1"/>
-        </x:patternFill>
-      </x:fill>
-    </x:dxf>
-    <x:dxf>
-      <x:font>
-        <x:color rgb="FF163A5F"/>
-      </x:font>
-      <x:fill>
-        <x:patternFill>
-          <x:bgColor rgb="FFEAF4FB"/>
-        </x:patternFill>
-      </x:fill>
-    </x:dxf>
-    <x:dxf>
-      <x:font>
-        <x:b/>
-        <x:color rgb="FF8A5A00"/>
-      </x:font>
-      <x:fill>
-        <x:patternFill>
-          <x:bgColor rgb="FFFFF4D6"/>
-        </x:patternFill>
-      </x:fill>
-    </x:dxf>
-    <x:dxf>
-      <x:font>
-        <x:color rgb="FF8A5A00"/>
-      </x:font>
-      <x:fill>
-        <x:patternFill>
-          <x:bgColor rgb="FFFFF4D6"/>
-        </x:patternFill>
-      </x:fill>
-    </x:dxf>
-    <x:dxf>
-      <x:font>
-        <x:b/>
-        <x:color rgb="FFA61B1B"/>
-      </x:font>
-      <x:fill>
-        <x:patternFill>
-          <x:bgColor rgb="FFFCE8E6"/>
-        </x:patternFill>
-      </x:fill>
-    </x:dxf>
-    <x:dxf>
-      <x:font>
-        <x:b/>
-        <x:color rgb="FFA61B1B"/>
-      </x:font>
-      <x:fill>
-        <x:patternFill>
-          <x:bgColor rgb="FFFCE8E6"/>
-        </x:patternFill>
-      </x:fill>
-    </x:dxf>
-    <x:dxf>
-      <x:font>
-        <x:b/>
-        <x:color rgb="FF8A5A00"/>
-      </x:font>
-      <x:fill>
-        <x:patternFill>
-          <x:bgColor rgb="FFFFF4D6"/>
-        </x:patternFill>
-      </x:fill>
-    </x:dxf>
-    <x:dxf>
-      <x:font>
-        <x:b/>
-        <x:color rgb="FFA61B1B"/>
-      </x:font>
-      <x:fill>
-        <x:patternFill>
-          <x:bgColor rgb="FFFCE8E6"/>
-        </x:patternFill>
-      </x:fill>
-    </x:dxf>
-    <x:dxf>
-      <x:font>
-        <x:b/>
-        <x:color rgb="FF8A5A00"/>
-      </x:font>
-      <x:fill>
-        <x:patternFill>
-          <x:bgColor rgb="FFFFF4D6"/>
-        </x:patternFill>
-      </x:fill>
-    </x:dxf>
-    <x:dxf>
-      <x:font>
-        <x:color rgb="FF087A68"/>
-      </x:font>
-      <x:fill>
-        <x:patternFill>
-          <x:bgColor rgb="FFE7F6F1"/>
-        </x:patternFill>
-      </x:fill>
-    </x:dxf>
-    <x:dxf>
-      <x:font>
-        <x:color rgb="FF087A68"/>
-      </x:font>
-      <x:fill>
-        <x:patternFill>
-          <x:bgColor rgb="FFE7F6F1"/>
-        </x:patternFill>
-      </x:fill>
-    </x:dxf>
-    <x:dxf>
-      <x:font>
-        <x:color rgb="FF163A5F"/>
-      </x:font>
-      <x:fill>
-        <x:patternFill>
-          <x:bgColor rgb="FFEAF4FB"/>
-        </x:patternFill>
-      </x:fill>
-    </x:dxf>
-    <x:dxf>
-      <x:font>
-        <x:b/>
-        <x:color rgb="FF8A5A00"/>
-      </x:font>
-      <x:fill>
-        <x:patternFill>
-          <x:bgColor rgb="FFFFF4D6"/>
-        </x:patternFill>
-      </x:fill>
-    </x:dxf>
-    <x:dxf>
-      <x:font>
-        <x:color rgb="FF8A5A00"/>
-      </x:font>
-      <x:fill>
-        <x:patternFill>
-          <x:bgColor rgb="FFFFF4D6"/>
-        </x:patternFill>
-      </x:fill>
-    </x:dxf>
-    <x:dxf>
-      <x:font>
-        <x:b/>
-        <x:color rgb="FFA61B1B"/>
-      </x:font>
-      <x:fill>
-        <x:patternFill>
-          <x:bgColor rgb="FFFCE8E6"/>
-        </x:patternFill>
-      </x:fill>
-    </x:dxf>
-    <x:dxf>
-      <x:font>
-        <x:b/>
-        <x:color rgb="FFA61B1B"/>
-      </x:font>
-      <x:fill>
-        <x:patternFill>
-          <x:bgColor rgb="FFFCE8E6"/>
-        </x:patternFill>
-      </x:fill>
-    </x:dxf>
-    <x:dxf>
-      <x:font>
-        <x:b/>
-        <x:color rgb="FF8A5A00"/>
-      </x:font>
-      <x:fill>
-        <x:patternFill>
-          <x:bgColor rgb="FFFFF4D6"/>
-        </x:patternFill>
-      </x:fill>
-    </x:dxf>
-    <x:dxf>
-      <x:font>
-        <x:b/>
-        <x:color rgb="FFA61B1B"/>
-      </x:font>
-      <x:fill>
-        <x:patternFill>
-          <x:bgColor rgb="FFFCE8E6"/>
-        </x:patternFill>
-      </x:fill>
-    </x:dxf>
-    <x:dxf>
-      <x:font>
-        <x:b/>
-        <x:color rgb="FF8A5A00"/>
-      </x:font>
-      <x:fill>
-        <x:patternFill>
-          <x:bgColor rgb="FFFFF4D6"/>
-        </x:patternFill>
-      </x:fill>
-    </x:dxf>
-    <x:dxf>
-      <x:font>
-        <x:color rgb="FF087A68"/>
-      </x:font>
-      <x:fill>
-        <x:patternFill>
-          <x:bgColor rgb="FFE7F6F1"/>
-        </x:patternFill>
-      </x:fill>
-    </x:dxf>
-    <x:dxf>
-      <x:font>
-        <x:color rgb="FF087A68"/>
-      </x:font>
-      <x:fill>
-        <x:patternFill>
-          <x:bgColor rgb="FFE7F6F1"/>
-        </x:patternFill>
-      </x:fill>
-    </x:dxf>
-    <x:dxf>
-      <x:font>
-        <x:color rgb="FF163A5F"/>
-      </x:font>
-      <x:fill>
-        <x:patternFill>
-          <x:bgColor rgb="FFEAF4FB"/>
-        </x:patternFill>
-      </x:fill>
-    </x:dxf>
-    <x:dxf>
-      <x:font>
-        <x:b/>
-        <x:color rgb="FF8A5A00"/>
-      </x:font>
-      <x:fill>
-        <x:patternFill>
-          <x:bgColor rgb="FFFFF4D6"/>
-        </x:patternFill>
-      </x:fill>
-    </x:dxf>
-    <x:dxf>
-      <x:font>
-        <x:color rgb="FF8A5A00"/>
-      </x:font>
-      <x:fill>
-        <x:patternFill>
-          <x:bgColor rgb="FFFFF4D6"/>
-        </x:patternFill>
-      </x:fill>
-    </x:dxf>
-    <x:dxf>
-      <x:font>
-        <x:b/>
-        <x:color rgb="FFA61B1B"/>
-      </x:font>
-      <x:fill>
-        <x:patternFill>
-          <x:bgColor rgb="FFFCE8E6"/>
-        </x:patternFill>
-      </x:fill>
-    </x:dxf>
-    <x:dxf>
-      <x:font>
-        <x:b/>
-        <x:color rgb="FFA61B1B"/>
-      </x:font>
-      <x:fill>
-        <x:patternFill>
-          <x:bgColor rgb="FFFCE8E6"/>
-        </x:patternFill>
-      </x:fill>
-    </x:dxf>
-    <x:dxf>
-      <x:font>
-        <x:b/>
-        <x:color rgb="FF8A5A00"/>
-      </x:font>
-      <x:fill>
-        <x:patternFill>
-          <x:bgColor rgb="FFFFF4D6"/>
-        </x:patternFill>
-      </x:fill>
-    </x:dxf>
-    <x:dxf>
-      <x:font>
-        <x:b/>
-        <x:color rgb="FFA61B1B"/>
-      </x:font>
-      <x:fill>
-        <x:patternFill>
-          <x:bgColor rgb="FFFCE8E6"/>
-        </x:patternFill>
-      </x:fill>
-    </x:dxf>
-    <x:dxf>
-      <x:font>
-        <x:b/>
-        <x:color rgb="FF8A5A00"/>
-      </x:font>
-      <x:fill>
-        <x:patternFill>
-          <x:bgColor rgb="FFFFF4D6"/>
-        </x:patternFill>
-      </x:fill>
-    </x:dxf>
-    <x:dxf>
-      <x:font>
-        <x:color rgb="FF087A68"/>
-      </x:font>
-      <x:fill>
-        <x:patternFill>
-          <x:bgColor rgb="FFE7F6F1"/>
-        </x:patternFill>
-      </x:fill>
-    </x:dxf>
-    <x:dxf>
-      <x:font>
-        <x:color rgb="FF087A68"/>
-      </x:font>
-      <x:fill>
-        <x:patternFill>
-          <x:bgColor rgb="FFE7F6F1"/>
-        </x:patternFill>
-      </x:fill>
-    </x:dxf>
-    <x:dxf>
-      <x:font>
-        <x:color rgb="FF163A5F"/>
-      </x:font>
-      <x:fill>
-        <x:patternFill>
-          <x:bgColor rgb="FFEAF4FB"/>
-        </x:patternFill>
-      </x:fill>
-    </x:dxf>
-    <x:dxf>
-      <x:font>
-        <x:b/>
-        <x:color rgb="FF8A5A00"/>
-      </x:font>
-      <x:fill>
-        <x:patternFill>
-          <x:bgColor rgb="FFFFF4D6"/>
-        </x:patternFill>
-      </x:fill>
-    </x:dxf>
-    <x:dxf>
-      <x:font>
-        <x:color rgb="FF8A5A00"/>
-      </x:font>
-      <x:fill>
-        <x:patternFill>
-          <x:bgColor rgb="FFFFF4D6"/>
-        </x:patternFill>
-      </x:fill>
-    </x:dxf>
-    <x:dxf>
-      <x:font>
-        <x:b/>
-        <x:color rgb="FFA61B1B"/>
-      </x:font>
-      <x:fill>
-        <x:patternFill>
-          <x:bgColor rgb="FFFCE8E6"/>
-        </x:patternFill>
-      </x:fill>
-    </x:dxf>
-    <x:dxf>
-      <x:font>
-        <x:b/>
-        <x:color rgb="FFA61B1B"/>
-      </x:font>
-      <x:fill>
-        <x:patternFill>
-          <x:bgColor rgb="FFFCE8E6"/>
-        </x:patternFill>
-      </x:fill>
-    </x:dxf>
-    <x:dxf>
-      <x:font>
-        <x:b/>
-        <x:color rgb="FF8A5A00"/>
-      </x:font>
-      <x:fill>
-        <x:patternFill>
-          <x:bgColor rgb="FFFFF4D6"/>
-        </x:patternFill>
-      </x:fill>
-    </x:dxf>
-    <x:dxf>
-      <x:font>
-        <x:b/>
-        <x:color rgb="FFA61B1B"/>
-      </x:font>
-      <x:fill>
-        <x:patternFill>
-          <x:bgColor rgb="FFFCE8E6"/>
-        </x:patternFill>
-      </x:fill>
-    </x:dxf>
-    <x:dxf>
-      <x:font>
-        <x:b/>
-        <x:color rgb="FF8A5A00"/>
-      </x:font>
-      <x:fill>
-        <x:patternFill>
-          <x:bgColor rgb="FFFFF4D6"/>
-        </x:patternFill>
-      </x:fill>
-    </x:dxf>
+  <x:dxfs count="10">
     <x:dxf>
       <x:font>
         <x:color rgb="FF087A68"/>
@@ -906,19 +482,20 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="FeatureComparisonTable" displayName="FeatureComparisonTable" ref="A6:D53" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:tableColumns count="4">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="FeatureComparisonTable" displayName="FeatureComparisonTable" ref="A6:E53" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="5">
     <x:tableColumn id="1" name="Feature"/>
     <x:tableColumn id="2" name="OM0RX-xLog"/>
     <x:tableColumn id="3" name="RUMlogNG"/>
     <x:tableColumn id="4" name="QLog"/>
+    <x:tableColumn id="5" name="OpsLog"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="OutstandingWorkTable" displayName="OutstandingWorkTable" ref="A6:F27" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="OutstandingWorkTable" displayName="OutstandingWorkTable" ref="A6:F29" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="6">
     <x:tableColumn id="1" name="Priority"/>
     <x:tableColumn id="2" name="Feature or decision"/>
@@ -945,7 +522,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="SourcesTable" displayName="SourcesTable" ref="A6:D18" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="SourcesTable" displayName="SourcesTable" ref="A6:D22" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="4">
     <x:tableColumn id="1" name="Product"/>
     <x:tableColumn id="2" name="Source or evidence"/>
@@ -1158,6 +735,7 @@
     <x:col min="2" max="2" width="64" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="54" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="54" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="54" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="15" hidden="0" customHeight="1">
@@ -1175,17 +753,17 @@
       <x:c r="B2" s="61"/>
       <x:c r="C2" s="61"/>
       <x:c r="D2" s="61"/>
-      <x:c r="E2" s="59"/>
+      <x:c r="E2" s="61"/>
       <x:c r="F2" s="59"/>
     </x:row>
     <x:row r="3" ht="15" hidden="0" customHeight="1">
       <x:c r="A3" s="62" t="str">
-        <x:v>As of 16 October 2026. OM0RX-xLog states distinguish source implementation, installed/package acceptance and live hardware/service proof. RUMlogNG and QLog entries are limited to the verified sources listed on the Sources sheet.</x:v>
+        <x:v>As of 16 October 2026. OM0RX-xLog states distinguish source implementation, installed/package acceptance and live hardware/service proof. External references: RUMlogNG #1, QLog #2, OpsLog #3. OpsLog v0.51.10 is documented supplementary only, not current-source/license verified; Sources records the access gap.</x:v>
       </x:c>
       <x:c r="B3" s="63"/>
       <x:c r="C3" s="63"/>
       <x:c r="D3" s="63"/>
-      <x:c r="E3" s="59"/>
+      <x:c r="E3" s="63"/>
       <x:c r="F3" s="59"/>
     </x:row>
     <x:row r="4" ht="15" hidden="0" customHeight="1">
@@ -1222,10 +800,12 @@
       <x:c r="C6" s="30" t="str">
         <x:v>RUMlogNG</x:v>
       </x:c>
-      <x:c r="D6" s="31" t="str">
+      <x:c r="D6" s="30" t="str">
         <x:v>QLog</x:v>
       </x:c>
-      <x:c r="E6" s="59"/>
+      <x:c r="E6" s="31" t="str">
+        <x:v>OpsLog</x:v>
+      </x:c>
       <x:c r="F6" s="59"/>
     </x:row>
     <x:row r="7" ht="24" hidden="0" customHeight="1">
@@ -1241,7 +821,9 @@
       <x:c r="D7" s="65" t="str">
         <x:v>Documented — local SQLite backend on Linux and Windows.</x:v>
       </x:c>
-      <x:c r="E7" s="59"/>
+      <x:c r="E7" s="65" t="str">
+        <x:v>Documented — local SQLite logbook or optional per-profile shared MySQL; configuration remains local SQLite.</x:v>
+      </x:c>
       <x:c r="F7" s="59"/>
     </x:row>
     <x:row r="8" ht="36" hidden="0" customHeight="1">
@@ -1257,7 +839,9 @@
       <x:c r="D8" s="67" t="str">
         <x:v>Documented — general-purpose QSO logging; customizable interface.</x:v>
       </x:c>
-      <x:c r="E8" s="59"/>
+      <x:c r="E8" s="67" t="str">
+        <x:v>Documented — single-strip entry and configurable panes. A matching Simple/Full editor contract was not established.</x:v>
+      </x:c>
       <x:c r="F8" s="59"/>
     </x:row>
     <x:row r="9" ht="48" hidden="0" customHeight="1">
@@ -1273,7 +857,9 @@
       <x:c r="D9" s="67" t="str">
         <x:v>Documented — log management and custom QSO filters; arbitrary-field editor breadth was not established in the reviewed README.</x:v>
       </x:c>
-      <x:c r="E9" s="59"/>
+      <x:c r="E9" s="67" t="str">
+        <x:v>Documented — QSO editing, generic ADIF extras and duplicate deletion choices. Matching revision/undo guarantees were not established.</x:v>
+      </x:c>
       <x:c r="F9" s="59"/>
     </x:row>
     <x:row r="10" ht="264" hidden="0" customHeight="1">
@@ -1289,7 +875,9 @@
       <x:c r="D10" s="67" t="str">
         <x:v>Documented — log management and service reconciliation; comparable field-provenance findings were not established.</x:v>
       </x:c>
-      <x:c r="E10" s="59"/>
+      <x:c r="E10" s="67" t="str">
+        <x:v>Documented — dated CTY/ClubLog resolution, preservation of deleted DXCC entities and per-row RDA disagreement choices. Matching field-origin provenance was not established.</x:v>
+      </x:c>
       <x:c r="F10" s="59"/>
     </x:row>
     <x:row r="11" ht="156" hidden="0" customHeight="1">
@@ -1305,7 +893,9 @@
       <x:c r="D11" s="67" t="str">
         <x:v>Documented — ADIF-oriented logbook and online-service interchange; unknown-field preservation was not established in the reviewed README.</x:v>
       </x:c>
-      <x:c r="E11" s="59"/>
+      <x:c r="E11" s="67" t="str">
+        <x:v>Documented — ADIF 3.1.7 dictionary, promoted columns, generic extras and standard/all export modes. Round-trip fidelity is not independently verified.</x:v>
+      </x:c>
       <x:c r="F11" s="59"/>
     </x:row>
     <x:row r="12" ht="24" hidden="0" customHeight="1">
@@ -1321,7 +911,9 @@
       <x:c r="D12" s="67" t="str">
         <x:v>Documented — import and service reconciliation are present; exact duplicate/update review behavior was not established in the reviewed README.</x:v>
       </x:c>
-      <x:c r="E12" s="59"/>
+      <x:c r="E12" s="67" t="str">
+        <x:v>Documented — skip/update/import-anyway choices, optional field mapping and duplicate tools.</x:v>
+      </x:c>
       <x:c r="F12" s="59"/>
     </x:row>
     <x:row r="13" ht="24" hidden="0" customHeight="1">
@@ -1337,7 +929,9 @@
       <x:c r="D13" s="67" t="str">
         <x:v>Documented — log and service integrations imply interchange; exact selected/filtered export behavior was not established in the reviewed README.</x:v>
       </x:c>
-      <x:c r="E13" s="59"/>
+      <x:c r="E13" s="67" t="str">
+        <x:v>Documented — filter builder and filtered/selected ADIF export, plus standard/all export modes.</x:v>
+      </x:c>
       <x:c r="F13" s="59"/>
     </x:row>
     <x:row r="14" ht="24" hidden="0" customHeight="1">
@@ -1353,7 +947,9 @@
       <x:c r="D14" s="67" t="str">
         <x:v>Documented — customizable GUI and saved table state patterns.</x:v>
       </x:c>
-      <x:c r="E14" s="59"/>
+      <x:c r="E14" s="67" t="str">
+        <x:v>Not established in reviewed v0.51.10 documentation as equivalent selectable Logbook columns.</x:v>
+      </x:c>
       <x:c r="F14" s="59"/>
     </x:row>
     <x:row r="15" ht="24" hidden="0" customHeight="1">
@@ -1369,7 +965,9 @@
       <x:c r="D15" s="67" t="str">
         <x:v>Documented — movable/visible columns are used in QLog tables; exact persistence varies by view.</x:v>
       </x:c>
-      <x:c r="E15" s="59"/>
+      <x:c r="E15" s="67" t="str">
+        <x:v>Not established in reviewed v0.51.10 documentation as equivalent persisted Logbook column widths.</x:v>
+      </x:c>
       <x:c r="F15" s="59"/>
     </x:row>
     <x:row r="16" ht="48" hidden="0" customHeight="1">
@@ -1385,7 +983,9 @@
       <x:c r="D16" s="67" t="str">
         <x:v>Not established in reviewed evidence as a dedicated independent window.</x:v>
       </x:c>
-      <x:c r="E16" s="59"/>
+      <x:c r="E16" s="67" t="str">
+        <x:v>Documented — recent QSOs and worked-before band/mode matrix. Independent native-window behavior was not established.</x:v>
+      </x:c>
       <x:c r="F16" s="59"/>
     </x:row>
     <x:row r="17" ht="60" hidden="0" customHeight="1">
@@ -1401,7 +1001,9 @@
       <x:c r="D17" s="67" t="str">
         <x:v>Documented — QRZ.com and HamQTH callbook integration plus club-member lookup.</x:v>
       </x:c>
-      <x:c r="E17" s="59"/>
+      <x:c r="E17" s="67" t="str">
+        <x:v>Documented — QRZ/HamQTH lookup, offline CTY, call-area handling and dated ClubLog exceptions.</x:v>
+      </x:c>
       <x:c r="F17" s="59"/>
     </x:row>
     <x:row r="18" ht="60" hidden="0" customHeight="1">
@@ -1417,7 +1019,9 @@
       <x:c r="D18" s="67" t="str">
         <x:v>Documented — alerts, custom filters and award tracking; the reviewed evidence did not establish the same shared goal model.</x:v>
       </x:c>
-      <x:c r="E18" s="59"/>
+      <x:c r="E18" s="67" t="str">
+        <x:v>Documented — award/reference detection and POTA-tagged spots. An equivalent shared goal/opportunity model was not established.</x:v>
+      </x:c>
       <x:c r="F18" s="59"/>
     </x:row>
     <x:row r="19" ht="72" hidden="0" customHeight="1">
@@ -1433,7 +1037,9 @@
       <x:c r="D19" s="67" t="str">
         <x:v>Not established as a comparable product surface in reviewed primary evidence.</x:v>
       </x:c>
-      <x:c r="E19" s="59"/>
+      <x:c r="E19" s="67" t="str">
+        <x:v>Not established in reviewed v0.51.10 documentation as an equivalent redacted diagnostic/support surface.</x:v>
+      </x:c>
       <x:c r="F19" s="59"/>
     </x:row>
     <x:row r="20" ht="72" hidden="0" customHeight="1">
@@ -1449,7 +1055,9 @@
       <x:c r="D20" s="67" t="str">
         <x:v>Documented — Cloudlog/Wavelog integration.</x:v>
       </x:c>
-      <x:c r="E20" s="59"/>
+      <x:c r="E20" s="67" t="str">
+        <x:v>Documented — Cloudlog/Wavelog upload and confirmation download. Matching conflict-safe two-way reconciliation was not established.</x:v>
+      </x:c>
       <x:c r="F20" s="59"/>
     </x:row>
     <x:row r="21" ht="72" hidden="0" customHeight="1">
@@ -1465,7 +1073,9 @@
       <x:c r="D21" s="67" t="str">
         <x:v>Documented — LoTW, eQSL, QRZ.com, Club Log, HRDLog.net and Cloudlog/Wavelog integrations.</x:v>
       </x:c>
-      <x:c r="E21" s="59"/>
+      <x:c r="E21" s="67" t="str">
+        <x:v>Documented — ClubLog/LoTW/QRZ/eQSL/Cloudlog/Wavelog/HAMLOG confirmations refresh award statistics.</x:v>
+      </x:c>
       <x:c r="F21" s="59"/>
     </x:row>
     <x:row r="22" ht="24" hidden="0" customHeight="1">
@@ -1481,7 +1091,9 @@
       <x:c r="D22" s="67" t="str">
         <x:v>Documented — QRZ.com callbook integration.</x:v>
       </x:c>
-      <x:c r="E22" s="59"/>
+      <x:c r="E22" s="67" t="str">
+        <x:v>Documented — QRZ.com lookup with photo and contact-field autofill.</x:v>
+      </x:c>
       <x:c r="F22" s="59"/>
     </x:row>
     <x:row r="23" ht="24" hidden="0" customHeight="1">
@@ -1497,7 +1109,9 @@
       <x:c r="D23" s="67" t="str">
         <x:v>Documented — QRZ.com online-log integration.</x:v>
       </x:c>
-      <x:c r="E23" s="59"/>
+      <x:c r="E23" s="67" t="str">
+        <x:v>Documented — QRZ.com upload and confirmation workflows; account/runtime acceptance not independently verified.</x:v>
+      </x:c>
       <x:c r="F23" s="59"/>
     </x:row>
     <x:row r="24" ht="24" hidden="0" customHeight="1">
@@ -1513,7 +1127,9 @@
       <x:c r="D24" s="67" t="str">
         <x:v>Documented — Club Log integration.</x:v>
       </x:c>
-      <x:c r="E24" s="59"/>
+      <x:c r="E24" s="67" t="str">
+        <x:v>Documented — batched ADIF upload and confirmation download.</x:v>
+      </x:c>
       <x:c r="F24" s="59"/>
     </x:row>
     <x:row r="25" ht="84" hidden="0" customHeight="1">
@@ -1529,7 +1145,9 @@
       <x:c r="D25" s="67" t="str">
         <x:v>Documented online-log integrations; exact evidence boundaries were not audited.</x:v>
       </x:c>
-      <x:c r="E25" s="59"/>
+      <x:c r="E25" s="67" t="str">
+        <x:v>Documented — confirmation download and award refresh. Equivalent provider acceptance/match ages and sponsor-credit semantics were not established.</x:v>
+      </x:c>
       <x:c r="F25" s="59"/>
     </x:row>
     <x:row r="26" ht="24" hidden="0" customHeight="1">
@@ -1545,7 +1163,9 @@
       <x:c r="D26" s="67" t="str">
         <x:v>Documented — HRDLog.net integration.</x:v>
       </x:c>
-      <x:c r="E26" s="59"/>
+      <x:c r="E26" s="67" t="str">
+        <x:v>Not established in reviewed v0.51.10 documentation.</x:v>
+      </x:c>
       <x:c r="F26" s="59"/>
     </x:row>
     <x:row r="27" ht="24" hidden="0" customHeight="1">
@@ -1561,7 +1181,9 @@
       <x:c r="D27" s="67" t="str">
         <x:v>Documented — LoTW and eQSL integration; TQSL is optional for LoTW and eQSL can download QSL pictures.</x:v>
       </x:c>
-      <x:c r="E27" s="59"/>
+      <x:c r="E27" s="67" t="str">
+        <x:v>Documented — direct LoTW and eQSL upload/confirmation workflows.</x:v>
+      </x:c>
       <x:c r="F27" s="59"/>
     </x:row>
     <x:row r="28" ht="24" hidden="0" customHeight="1">
@@ -1577,7 +1199,9 @@
       <x:c r="D28" s="67" t="str">
         <x:v>Documented — WSJT-X integration; source audit shows one configurable unicast/multicast receiver and QSO Logged/Logged ADIF parsing.</x:v>
       </x:c>
-      <x:c r="E28" s="59"/>
+      <x:c r="E28" s="67" t="str">
+        <x:v>Documented — WSJT-X/JTDX/MSHV UDP decodes and outbound logged-QSO ADIF. Matching inbound Logged ADIF safety contract was not established.</x:v>
+      </x:c>
       <x:c r="F28" s="59"/>
     </x:row>
     <x:row r="29" ht="24" hidden="0" customHeight="1">
@@ -1593,7 +1217,9 @@
       <x:c r="D29" s="67" t="str">
         <x:v>Documented — WSJT-X activity can feed its alert evaluator.</x:v>
       </x:c>
-      <x:c r="E29" s="59"/>
+      <x:c r="E29" s="67" t="str">
+        <x:v>Documented — UDP decodes feed band maps, alerts and Flex spots; v0.51.10 notes a direct-reply filtering fix.</x:v>
+      </x:c>
       <x:c r="F29" s="59"/>
     </x:row>
     <x:row r="30" ht="24" hidden="0" customHeight="1">
@@ -1609,7 +1235,9 @@
       <x:c r="D30" s="67" t="str">
         <x:v>Documented — DX cluster integration.</x:v>
       </x:c>
-      <x:c r="E30" s="59"/>
+      <x:c r="E30" s="67" t="str">
+        <x:v>Documented — multiple clusters, reconnect, shared filters and new/new-band/new-slot/worked status.</x:v>
+      </x:c>
       <x:c r="F30" s="59"/>
     </x:row>
     <x:row r="31" ht="24" hidden="0" customHeight="1">
@@ -1625,7 +1253,9 @@
       <x:c r="D31" s="67" t="str">
         <x:v>Documented alert/history tables; exact long-term raw report retention was not established in the reviewed README.</x:v>
       </x:c>
-      <x:c r="E31" s="59"/>
+      <x:c r="E31" s="67" t="str">
+        <x:v>Not established in reviewed v0.51.10 documentation as an equivalent retained report/history store.</x:v>
+      </x:c>
       <x:c r="F31" s="59"/>
     </x:row>
     <x:row r="32" ht="48" hidden="0" customHeight="1">
@@ -1641,7 +1271,9 @@
       <x:c r="D32" s="67" t="str">
         <x:v>Documented — named cloneable rules combining source, callsign, entity, novelty, geography, comment, band, mode, memberships and activity references.</x:v>
       </x:c>
-      <x:c r="E32" s="59"/>
+      <x:c r="E32" s="67" t="str">
+        <x:v>Documented — call/country/band/mode/spotter alert rules and WSJT-X/JTDX/MSHV activity.</x:v>
+      </x:c>
       <x:c r="F32" s="59"/>
     </x:row>
     <x:row r="33" ht="24" hidden="0" customHeight="1">
@@ -1657,7 +1289,9 @@
       <x:c r="D33" s="67" t="str">
         <x:v>Documented — optional bell and outbound UDP; QLog may also tune/reply from alert UI, which OM0RX-xLog intentionally does not copy.</x:v>
       </x:c>
-      <x:c r="E33" s="59"/>
+      <x:c r="E33" s="67" t="str">
+        <x:v>Documented — sound, visual and email alerts. Equivalent no-action/no-RF authority guarantees were not established.</x:v>
+      </x:c>
       <x:c r="F33" s="59"/>
     </x:row>
     <x:row r="34" ht="24" hidden="0" customHeight="1">
@@ -1673,7 +1307,9 @@
       <x:c r="D34" s="67" t="str">
         <x:v>Documented — online and offline map.</x:v>
       </x:c>
-      <x:c r="E34" s="59"/>
+      <x:c r="E34" s="67" t="str">
+        <x:v>Documented — great-circle and locator maps, basemaps, distance/bearing and antenna lobes. Grayline was not established.</x:v>
+      </x:c>
       <x:c r="F34" s="59"/>
     </x:row>
     <x:row r="35" ht="24" hidden="0" customHeight="1">
@@ -1689,7 +1325,9 @@
       <x:c r="D35" s="67" t="str">
         <x:v>Documented — bandmap.</x:v>
       </x:c>
-      <x:c r="E35" s="59"/>
+      <x:c r="E35" s="67" t="str">
+        <x:v>Documented — multi-band panadapter-style strips and worked-status filtering.</x:v>
+      </x:c>
       <x:c r="F35" s="59"/>
     </x:row>
     <x:row r="36" ht="36" hidden="0" customHeight="1">
@@ -1705,7 +1343,9 @@
       <x:c r="D36" s="67" t="str">
         <x:v>Documented — customizable GUI and saved layout profiles; macOS is experimental.</x:v>
       </x:c>
-      <x:c r="E36" s="59"/>
+      <x:c r="E36" s="67" t="str">
+        <x:v>Documented — configurable per-profile panes and independent per-tab persistence in v0.51.10. Equivalent detached lifecycle was not established.</x:v>
+      </x:c>
       <x:c r="F36" s="59"/>
     </x:row>
     <x:row r="37" ht="60" hidden="0" customHeight="1">
@@ -1721,7 +1361,9 @@
       <x:c r="D37" s="67" t="str">
         <x:v>Recommended resolution is 1920×1080; cross-platform GUI is customizable, but compact-window behavior was not established.</x:v>
       </x:c>
-      <x:c r="E37" s="59"/>
+      <x:c r="E37" s="67" t="str">
+        <x:v>Not independently verified. Release notes mention window sizing; exact compact/mixed-display acceptance was not established.</x:v>
+      </x:c>
       <x:c r="F37" s="59"/>
     </x:row>
     <x:row r="38" ht="24" hidden="0" customHeight="1">
@@ -1737,7 +1379,9 @@
       <x:c r="D38" s="67" t="str">
         <x:v>Documented saved layout profiles; exact freeform canvas resize interaction differs.</x:v>
       </x:c>
-      <x:c r="E38" s="59"/>
+      <x:c r="E38" s="67" t="str">
+        <x:v>Documented — configurable panes and dockable/reorderable Station Control. Equivalent freeform canvas resize was not established.</x:v>
+      </x:c>
       <x:c r="F38" s="59"/>
     </x:row>
     <x:row r="39" ht="24" hidden="0" customHeight="1">
@@ -1753,7 +1397,9 @@
       <x:c r="D39" s="67" t="str">
         <x:v>Documented — Hamlib, OmniRig, TCI and FLRig.</x:v>
       </x:c>
-      <x:c r="E39" s="59"/>
+      <x:c r="E39" s="67" t="str">
+        <x:v>Documented — OmniRig, Flex TCP/UDP, Icom CI-V USB/network, Kenwood/Elecraft, Yaesu and TCI.</x:v>
+      </x:c>
       <x:c r="F39" s="59"/>
     </x:row>
     <x:row r="40" ht="300" hidden="0" customHeight="1">
@@ -1769,7 +1415,9 @@
       <x:c r="D40" s="67" t="str">
         <x:v>Documented — QLog supports all TCI-compatible rigs through its native TCI provider.</x:v>
       </x:c>
-      <x:c r="E40" s="59"/>
+      <x:c r="E40" s="67" t="str">
+        <x:v>Documented — push-driven TCI console, bidirectional audio, recorder and DVK. Source, key/release safety, physical calibration and RF acceptance are not independently verified.</x:v>
+      </x:c>
       <x:c r="F40" s="59"/>
     </x:row>
     <x:row r="41" ht="24" hidden="0" customHeight="1">
@@ -1785,7 +1433,9 @@
       <x:c r="D41" s="67" t="str">
         <x:v>Documented — rig control and cluster/bandmap integration; safety contract was not audited.</x:v>
       </x:c>
-      <x:c r="E41" s="59"/>
+      <x:c r="E41" s="67" t="str">
+        <x:v>Documented — tune/PTT controls and frequency/mode actions. Equivalent no-replay, abort and durable readback guarantees were not established.</x:v>
+      </x:c>
       <x:c r="F41" s="59"/>
     </x:row>
     <x:row r="42" ht="48" hidden="0" customHeight="1">
@@ -1801,7 +1451,9 @@
       <x:c r="D42" s="67" t="str">
         <x:v>No comparable amplifier owner was established in reviewed evidence.</x:v>
       </x:c>
-      <x:c r="E42" s="59"/>
+      <x:c r="E42" s="67" t="str">
+        <x:v>Documented — multiple amplifier controls/status/meters for PGXL, SPE, Acom and Elecraft families.</x:v>
+      </x:c>
       <x:c r="F42" s="59"/>
     </x:row>
     <x:row r="43" ht="24" hidden="0" customHeight="1">
@@ -1817,7 +1469,9 @@
       <x:c r="D43" s="67" t="str">
         <x:v>Documented — Hamlib and PSTRotator control.</x:v>
       </x:c>
-      <x:c r="E43" s="59"/>
+      <x:c r="E43" s="67" t="str">
+        <x:v>Documented — PstRotator UDP, Rotator Genius TCP, ARCO LAN/USB and Ultrabeam direction context.</x:v>
+      </x:c>
       <x:c r="F43" s="59"/>
     </x:row>
     <x:row r="44" ht="24" hidden="0" customHeight="1">
@@ -1833,7 +1487,9 @@
       <x:c r="D44" s="67" t="str">
         <x:v>Documented — CWDaemon, FLDigi, Morse over CAT, WinKey v1/v2 and CW Console.</x:v>
       </x:c>
-      <x:c r="E44" s="59"/>
+      <x:c r="E44" s="67" t="str">
+        <x:v>Documented — macros/F-keys via WinKeyer, Flex CWX, Icom or TCI; DVK and QSO audio recording.</x:v>
+      </x:c>
       <x:c r="F44" s="59"/>
     </x:row>
     <x:row r="45" ht="24" hidden="0" customHeight="1">
@@ -1849,7 +1505,9 @@
       <x:c r="D45" s="67" t="str">
         <x:v>Not highlighted in reviewed primary feature listing.</x:v>
       </x:c>
-      <x:c r="E45" s="59"/>
+      <x:c r="E45" s="67" t="str">
+        <x:v>Not established in reviewed v0.51.10 documentation as an equivalent propagation display.</x:v>
+      </x:c>
       <x:c r="F45" s="59"/>
     </x:row>
     <x:row r="46" ht="84" hidden="0" customHeight="1">
@@ -1865,7 +1523,9 @@
       <x:c r="D46" s="67" t="str">
         <x:v>Documented — basic awards and station statistics.</x:v>
       </x:c>
-      <x:c r="E46" s="59"/>
+      <x:c r="E46" s="67" t="str">
+        <x:v>Documented — configurable awards/references, worked/confirmed/validated band-mode matrices, reference import/rescan and statistics; sponsor-rule correctness is not verified.</x:v>
+      </x:c>
       <x:c r="F46" s="59"/>
     </x:row>
     <x:row r="47" ht="24" hidden="0" customHeight="1">
@@ -1881,7 +1541,9 @@
       <x:c r="D47" s="67" t="str">
         <x:v>Documented — basic contest support; QLog states contests are not its current focus.</x:v>
       </x:c>
-      <x:c r="E47" s="59"/>
+      <x:c r="E47" s="67" t="str">
+        <x:v>Documented — contest selection/exchange, dupe flags and scoreboard. Not independently source/runtime verified.</x:v>
+      </x:c>
       <x:c r="F47" s="59"/>
     </x:row>
     <x:row r="48" ht="24" hidden="0" customHeight="1">
@@ -1897,7 +1559,9 @@
       <x:c r="D48" s="67" t="str">
         <x:v>No paper-label workflow established in the reviewed README.</x:v>
       </x:c>
-      <x:c r="E48" s="59"/>
+      <x:c r="E48" s="67" t="str">
+        <x:v>Documented — QSL management and QSL-card designer/email eQSL. Equivalent paper-label printing was not established.</x:v>
+      </x:c>
       <x:c r="F48" s="59"/>
     </x:row>
     <x:row r="49" ht="24" hidden="0" customHeight="1">
@@ -1913,7 +1577,9 @@
       <x:c r="D49" s="67" t="str">
         <x:v>Documented — station location profile support.</x:v>
       </x:c>
-      <x:c r="E49" s="59"/>
+      <x:c r="E49" s="67" t="str">
+        <x:v>Documented — per-profile settings/logbook selection and optional shared MySQL.</x:v>
+      </x:c>
       <x:c r="F49" s="59"/>
     </x:row>
     <x:row r="50" ht="24" hidden="0" customHeight="1">
@@ -1929,7 +1595,9 @@
       <x:c r="D50" s="67" t="str">
         <x:v>Documented — system keyring/credential store support on Linux, Windows and macOS.</x:v>
       </x:c>
-      <x:c r="E50" s="59"/>
+      <x:c r="E50" s="67" t="str">
+        <x:v>Documented — opt-in passphrase vault using AES-GCM/PBKDF2. Implementation/security not independently source-verified.</x:v>
+      </x:c>
       <x:c r="F50" s="59"/>
     </x:row>
     <x:row r="51" ht="24" hidden="0" customHeight="1">
@@ -1945,7 +1613,9 @@
       <x:c r="D51" s="67" t="str">
         <x:v>Not established in reviewed primary feature listing.</x:v>
       </x:c>
-      <x:c r="E51" s="59"/>
+      <x:c r="E51" s="67" t="str">
+        <x:v>Documented — optional database/ADIF backup at shutdown. Equivalent verified recovery/restore guarantees were not established.</x:v>
+      </x:c>
       <x:c r="F51" s="59"/>
     </x:row>
     <x:row r="52" ht="24" hidden="0" customHeight="1">
@@ -1961,7 +1631,9 @@
       <x:c r="D52" s="67" t="str">
         <x:v>Linux and Windows supported; macOS is documented as experimental/developer-only.</x:v>
       </x:c>
-      <x:c r="E52" s="59"/>
+      <x:c r="E52" s="67" t="str">
+        <x:v>Documented as a Windows logger. Cross-platform delivery was not established.</x:v>
+      </x:c>
       <x:c r="F52" s="59"/>
     </x:row>
     <x:row r="53" ht="24" hidden="0" customHeight="1">
@@ -1977,7 +1649,9 @@
       <x:c r="D53" s="67" t="str">
         <x:v>Documented — no ads, user tracking or hidden telemetry.</x:v>
       </x:c>
-      <x:c r="E53" s="59"/>
+      <x:c r="E53" s="67" t="str">
+        <x:v>Documented — daily anonymous installation/version/OS telemetry with opt-out. No privacy/runtime verification performed.</x:v>
+      </x:c>
       <x:c r="F53" s="59"/>
     </x:row>
     <x:row r="54" ht="15" hidden="0" customHeight="1">
@@ -3158,19 +2832,19 @@
     </x:row>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="A3:D3"/>
+    <x:mergeCell ref="A3:E3"/>
   </x:mergeCells>
   <x:conditionalFormatting sqref="B7:B53">
-    <x:cfRule type="beginsWith" dxfId="40" priority="1" operator="beginsWith" text="Installed"/>
-    <x:cfRule type="beginsWith" dxfId="41" priority="2" operator="beginsWith" text="Implemented"/>
-    <x:cfRule type="beginsWith" dxfId="42" priority="3" operator="beginsWith" text="Source complete"/>
-    <x:cfRule type="beginsWith" dxfId="43" priority="4" operator="beginsWith" text="Active"/>
-    <x:cfRule type="beginsWith" dxfId="44" priority="5" operator="beginsWith" text="Partial"/>
-    <x:cfRule type="beginsWith" dxfId="45" priority="6" operator="beginsWith" text="Outstanding"/>
+    <x:cfRule type="beginsWith" dxfId="0" priority="1" operator="beginsWith" text="Installed"/>
+    <x:cfRule type="beginsWith" dxfId="1" priority="2" operator="beginsWith" text="Implemented"/>
+    <x:cfRule type="beginsWith" dxfId="2" priority="3" operator="beginsWith" text="Source complete"/>
+    <x:cfRule type="beginsWith" dxfId="3" priority="4" operator="beginsWith" text="Active"/>
+    <x:cfRule type="beginsWith" dxfId="4" priority="5" operator="beginsWith" text="Partial"/>
+    <x:cfRule type="beginsWith" dxfId="5" priority="6" operator="beginsWith" text="Outstanding"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rff5f82e80c5d4779"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R255c860418eb4f16"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3674,21 +3348,45 @@
         <x:v>QLog cross-platform distribution</x:v>
       </x:c>
     </x:row>
-    <x:row r="28" ht="15" hidden="0" customHeight="1">
-      <x:c r="A28" s="59"/>
-      <x:c r="B28" s="59"/>
-      <x:c r="C28" s="59"/>
-      <x:c r="D28" s="59"/>
-      <x:c r="E28" s="59"/>
-      <x:c r="F28" s="59"/>
-    </x:row>
-    <x:row r="29" ht="15" hidden="0" customHeight="1">
-      <x:c r="A29" s="59"/>
-      <x:c r="B29" s="59"/>
-      <x:c r="C29" s="59"/>
-      <x:c r="D29" s="59"/>
-      <x:c r="E29" s="59"/>
-      <x:c r="F29" s="59"/>
+    <x:row r="28" ht="48" hidden="0" customHeight="1">
+      <x:c r="A28" s="66" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="B28" s="67" t="str">
+        <x:v>OpsLog source/licence access</x:v>
+      </x:c>
+      <x:c r="C28" s="67" t="str">
+        <x:v>Documentation-only supplementary reference</x:v>
+      </x:c>
+      <x:c r="D28" s="67" t="str">
+        <x:v>Obtain legitimate access to actual versioned Gitea application source and explicit application licensing before any source audit or reuse. Public v0.51.10 mirror contains only README.md/README.fr.md; current source is auth-gated (Git credentials, web/archive login, API 403). No direct code copied.</x:v>
+      </x:c>
+      <x:c r="E28" s="67" t="str">
+        <x:v>Versioned application source and licence; no runtime/live acceptance inferred</x:v>
+      </x:c>
+      <x:c r="F28" s="67" t="str">
+        <x:v>RUMlogNG #1, QLog #2, OpsLog #3; OpsLog audit</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29" ht="48" hidden="0" customHeight="1">
+      <x:c r="A29" s="66" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="B29" s="67" t="str">
+        <x:v>Independent cross-surface acceptance</x:v>
+      </x:c>
+      <x:c r="C29" s="67" t="str">
+        <x:v>Planning; existing owners only</x:v>
+      </x:c>
+      <x:c r="D29" s="67" t="str">
+        <x:v>Separate standard ADIF/full-backup export; one award/spot-status projection across refresh; revision-checked caches; capability/transport/observed/action separation; TCI endpoint/key-release validation; per-map persistence/resize-after-layout; preserve user award customizations across catalogue upgrades.</x:v>
+      </x:c>
+      <x:c r="E29" s="67" t="str">
+        <x:v>Focused owner tests, exact-package/native/copied-log acceptance, then explicitly authorized device/provider/RF proof</x:v>
+      </x:c>
+      <x:c r="F29" s="67" t="str">
+        <x:v>OpsLog v0.51.10 README/release as supplementary behavior only</x:v>
+      </x:c>
     </x:row>
     <x:row r="30" ht="15" hidden="0" customHeight="1">
       <x:c r="A30" s="59"/>
@@ -5062,17 +4760,17 @@
   <x:mergeCells>
     <x:mergeCell ref="A3:F3"/>
   </x:mergeCells>
-  <x:conditionalFormatting sqref="A7:A27">
-    <x:cfRule type="cellIs" dxfId="46" priority="1" operator="equal">
+  <x:conditionalFormatting sqref="A7:A29">
+    <x:cfRule type="cellIs" dxfId="6" priority="1" operator="equal">
       <x:formula>"P0"</x:formula>
     </x:cfRule>
-    <x:cfRule type="cellIs" dxfId="47" priority="2" operator="equal">
+    <x:cfRule type="cellIs" dxfId="7" priority="2" operator="equal">
       <x:formula>"P1"</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R54539ca392bc42bf"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7510d9d0b576408b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6950,16 +6648,16 @@
     <x:mergeCell ref="A3:E3"/>
   </x:mergeCells>
   <x:conditionalFormatting sqref="B7:B30">
-    <x:cfRule type="cellIs" dxfId="48" priority="1" operator="equal">
+    <x:cfRule type="cellIs" dxfId="8" priority="1" operator="equal">
       <x:formula>"P0"</x:formula>
     </x:cfRule>
-    <x:cfRule type="cellIs" dxfId="49" priority="2" operator="equal">
+    <x:cfRule type="cellIs" dxfId="9" priority="2" operator="equal">
       <x:formula>"P1"</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R16285621e4c84f4a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3e938aa2b7c14a82"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7215,7 +6913,7 @@
         <x:v>Comparison method</x:v>
       </x:c>
       <x:c r="B18" s="67" t="str">
-        <x:v>RUMLOG_WORKFLOW_GAP_AUDIT_2026-10-14.md and QLOG_WORKFLOW_GAP_AUDIT_2026-10-15.md</x:v>
+        <x:v>RUMLOG_WORKFLOW_GAP_AUDIT_2026-10-14.md; QLOG_WORKFLOW_GAP_AUDIT_2026-10-15.md; OPSLOG_REFERENCE_AUDIT_2026-10-16.md</x:v>
       </x:c>
       <x:c r="C18" s="67" t="str">
         <x:v>2026-10-16</x:v>
@@ -7226,35 +6924,67 @@
       <x:c r="E18" s="59"/>
       <x:c r="F18" s="59"/>
     </x:row>
-    <x:row r="19" ht="15" hidden="0" customHeight="1">
-      <x:c r="A19" s="59"/>
-      <x:c r="B19" s="59"/>
-      <x:c r="C19" s="59"/>
-      <x:c r="D19" s="59"/>
+    <x:row r="19" ht="36" hidden="0" customHeight="1">
+      <x:c r="A19" s="66" t="str">
+        <x:v>Reference order</x:v>
+      </x:c>
+      <x:c r="B19" s="67" t="str">
+        <x:v>RUMlogNG #1; QLog #2; OpsLog #3</x:v>
+      </x:c>
+      <x:c r="C19" s="67" t="str">
+        <x:v>2026-10-16</x:v>
+      </x:c>
+      <x:c r="D19" s="67" t="str">
+        <x:v>OpsLog is documented supplementary only until current source and application licensing can be reviewed. Existing xLog checkpoint/test/acceptance limits remain unchanged. See docs/OPSLOG_REFERENCE_AUDIT_2026-10-16.md.</x:v>
+      </x:c>
       <x:c r="E19" s="59"/>
       <x:c r="F19" s="59"/>
     </x:row>
-    <x:row r="20" ht="15" hidden="0" customHeight="1">
-      <x:c r="A20" s="59"/>
-      <x:c r="B20" s="59"/>
-      <x:c r="C20" s="59"/>
-      <x:c r="D20" s="59"/>
+    <x:row r="20" ht="24" hidden="0" customHeight="1">
+      <x:c r="A20" s="66" t="str">
+        <x:v>OpsLog (#3)</x:v>
+      </x:c>
+      <x:c r="B20" s="67" t="str">
+        <x:v>https://github.com/GregTroar/OpsLog/releases/tag/v0.51.10</x:v>
+      </x:c>
+      <x:c r="C20" s="67" t="str">
+        <x:v>2026-10-16</x:v>
+      </x:c>
+      <x:c r="D20" s="67" t="str">
+        <x:v>Official release published 2026-10-15. Mirror tag SHA b30bd55c3de979edc76a965034e8d2f7fd5fdc12. Release notes supply acceptance ideas, not independent runtime/source verification.</x:v>
+      </x:c>
       <x:c r="E20" s="59"/>
       <x:c r="F20" s="59"/>
     </x:row>
-    <x:row r="21" ht="15" hidden="0" customHeight="1">
-      <x:c r="A21" s="59"/>
-      <x:c r="B21" s="59"/>
-      <x:c r="C21" s="59"/>
-      <x:c r="D21" s="59"/>
+    <x:row r="21" ht="36" hidden="0" customHeight="1">
+      <x:c r="A21" s="66" t="str">
+        <x:v>OpsLog (#3)</x:v>
+      </x:c>
+      <x:c r="B21" s="67" t="str">
+        <x:v>https://github.com/GregTroar/OpsLog/blob/b30bd55c3de979edc76a965034e8d2f7fd5fdc12/README.md</x:v>
+      </x:c>
+      <x:c r="C21" s="67" t="str">
+        <x:v>2026-10-16</x:v>
+      </x:c>
+      <x:c r="D21" s="67" t="str">
+        <x:v>Public tag contains README.md and README.fr.md only. Documented Wails 2.11/Go/React/TypeScript/Vite, SQLite configuration and optional shared MySQL log; feature statements in OpsLog column are documentation claims.</x:v>
+      </x:c>
       <x:c r="E21" s="59"/>
       <x:c r="F21" s="59"/>
     </x:row>
-    <x:row r="22" ht="15" hidden="0" customHeight="1">
-      <x:c r="A22" s="59"/>
-      <x:c r="B22" s="59"/>
-      <x:c r="C22" s="59"/>
-      <x:c r="D22" s="59"/>
+    <x:row r="22" ht="36" hidden="0" customHeight="1">
+      <x:c r="A22" s="66" t="str">
+        <x:v>OpsLog (#3)</x:v>
+      </x:c>
+      <x:c r="B22" s="67" t="str">
+        <x:v>https://git.rouggy.com/rouggy/OpsLog</x:v>
+      </x:c>
+      <x:c r="C22" s="67" t="str">
+        <x:v>2026-10-16</x:v>
+      </x:c>
+      <x:c r="D22" s="67" t="str">
+        <x:v>Actual source authority is authentication-gated: Git credentials, web/archive sign-in and API 403 in access audit. GitHub API license:null; no app source licence found. Not current-source-reviewed or licence-verified; no code copied.</x:v>
+      </x:c>
       <x:c r="E22" s="59"/>
       <x:c r="F22" s="59"/>
     </x:row>
@@ -8688,7 +8418,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdfb797c89d93414b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6d33e553516340c0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Refresh RUMlog-first feature comparison
</commit_message>
<xml_diff>
--- a/outputs/feature-matrix-2026-10-16/OM0RX-xLog_Feature_Comparison_2026-10-16.xlsx
+++ b/outputs/feature-matrix-2026-10-16/OM0RX-xLog_Feature_Comparison_2026-10-16.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Matrix" sheetId="1" r:id="R769cd6cdc2f342d1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Outstanding" sheetId="2" r:id="R8939dabb8b62478b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enhancement Review" sheetId="3" r:id="Rd3fa8452d55d4dc3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="4" r:id="R35f3bc2b727a4647"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Matrix" sheetId="1" r:id="R2886a8031864445c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Outstanding" sheetId="2" r:id="R874a728c194047cd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enhancement Review" sheetId="3" r:id="Rb3783e94713b4296"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="4" r:id="R44a768b7c6a04541"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -522,7 +522,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="SourcesTable" displayName="SourcesTable" ref="A6:D22" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="SourcesTable" displayName="SourcesTable" ref="A6:D24" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="4">
     <x:tableColumn id="1" name="Product"/>
     <x:tableColumn id="2" name="Source or evidence"/>
@@ -867,7 +867,7 @@
         <x:v>QSO data quality findings</x:v>
       </x:c>
       <x:c r="B10" s="67" t="str">
-        <x:v>Source complete for read-only findings, exact-contact route, Details UI and bounded duplicate review. c6ada81 reuses native exact call/band/primary-mode case-insensitive +/-600-second matching, self/deleted excluded, cap 5 plus lookahead with complete/truncated/unknown states. No semantic/frequency/submode/portable-callsign inference or mutation. Existing validation, dated CTY comparisons and retained power provenance remain review evidence; CTY version/date unknown and stored/manual values authoritative. Agent core 8/8, route/regression 6/6, frontend 19/19, tsc/build/window gates; root route 3/3, duplicate 3/3, frontend 19/19 pass. Native/package/live/full-coverage/correction/provider gates stay open; no award/sync delta. Installed alpha.31 unchanged. 33e5eb4 adds a pure bounded contact-update validation/raw field-diff prerequisite reused by canonical apply without changing receipts/revision/save semantics. Explicit invalid/stale/protected-identity failures; literal arbitrary fields preserve absent/empty distinction; cap 128 changes and 24,576 bytes/input with truncated/unavailable states. New 6/6 plus route/contact 15/15 and root focused 6/6 pass, including DB/WAL/SHM/journal purity. Not a saved-value simulation or correction-preview route/UI; correction UI/apply/undo remain open. 8ccffe7 adds read-only CTY DXCC-only correction preview, exact-contact/generation/revision/current-comparison-evidence fenced, using the canonical finding and pure review owner (root 2/2 plus data-quality regression). Unknown source/version/date facts stay unknown; stored/manual values are unchanged. No apply/undo/UI, operation ID, receipt, journal, provider correction or live acceptance. 327648c adds compact read-only CTY DXCC preview inside existing Logbook Details only, validating exact scope/evidence (Swift 2/2, UI/bridge 22/22, tsc). No apply/undo, operation ID, receipt, journal or provider correction; package/native/copied-log/live acceptance stays open.</x:v>
+        <x:v>Source complete for read-only findings, exact-contact route, Details UI and bounded duplicate review. c6ada81 reuses native exact call/band/primary-mode case-insensitive +/-600-second matching, self/deleted excluded, cap 5 plus lookahead with complete/truncated/unknown states. No semantic/frequency/submode/portable-callsign inference or mutation. Existing validation, dated CTY comparisons and retained power provenance remain review evidence; CTY version/date unknown and stored/manual values authoritative. Agent core 8/8, route/regression 6/6, frontend 19/19, tsc/build/window gates; root route 3/3, duplicate 3/3, frontend 19/19 pass. Native/package/live/full-coverage/correction/provider gates stay open; no award/sync delta. Installed alpha.32 is exact source e270ab5; later findings work remains source-only. 33e5eb4 adds a pure bounded contact-update validation/raw field-diff prerequisite reused by canonical apply without changing receipts/revision/save semantics. Explicit invalid/stale/protected-identity failures; literal arbitrary fields preserve absent/empty distinction; cap 128 changes and 24,576 bytes/input with truncated/unavailable states. New 6/6 plus route/contact 15/15 and root focused 6/6 pass, including DB/WAL/SHM/journal purity. Not a saved-value simulation or correction-preview route/UI; correction UI/apply/undo remain open. 8ccffe7 adds read-only CTY DXCC-only correction preview, exact-contact/generation/revision/current-comparison-evidence fenced, using the canonical finding and pure review owner (root 2/2 plus data-quality regression). Unknown source/version/date facts stay unknown; stored/manual values are unchanged. No apply/undo/UI, operation ID, receipt, journal, provider correction or live acceptance. 327648c adds compact read-only CTY DXCC preview inside existing Logbook Details only, validating exact scope/evidence (Swift 2/2, UI/bridge 22/22, tsc). No apply/undo, operation ID, receipt, journal or provider correction; package/native/copied-log/live acceptance stays open.</x:v>
       </x:c>
       <x:c r="C10" s="67" t="str">
         <x:v>Documented — QSO editing and DXCC/QSL workflows; comparable field-provenance findings were not established.</x:v>
@@ -934,12 +934,12 @@
       </x:c>
       <x:c r="F13" s="59"/>
     </x:row>
-    <x:row r="14" ht="24" hidden="0" customHeight="1">
+    <x:row r="14" ht="36" hidden="0" customHeight="1">
       <x:c r="A14" s="66" t="str">
         <x:v>Logbook table — selectable columns</x:v>
       </x:c>
       <x:c r="B14" s="67" t="str">
-        <x:v>Source complete — normal Logbook columns are available in dedicated, detached and map-split views with separate visibility preferences.</x:v>
+        <x:v>Source complete — normal Logbook columns are available in dedicated, detached and map-split views; visibility and keyboard-accessible ordering persist independently per presentation context. Packaged visual acceptance remains open.</x:v>
       </x:c>
       <x:c r="C14" s="67" t="str">
         <x:v>Documented / locally observed — configurable Logbook columns and table sizing.</x:v>
@@ -1168,12 +1168,12 @@
       </x:c>
       <x:c r="F26" s="59"/>
     </x:row>
-    <x:row r="27" ht="24" hidden="0" customHeight="1">
+    <x:row r="27" ht="60" hidden="0" customHeight="1">
       <x:c r="A27" s="66" t="str">
         <x:v>Direct LoTW and eQSL workflows</x:v>
       </x:c>
       <x:c r="B27" s="67" t="str">
-        <x:v>Outstanding as independent providers — confirmation fields and Wavelog refresh are supported, but direct credential/upload/download owners remain separate programmes.</x:v>
+        <x:v>Partial — LoTW parser foundation source complete: a dedicated bounded confirmation-report parser preserves report count, watermark, optional mode and LoTW-only evidence without generic ADIF import, paper-QSL mapping, credentials, network calls or database mutation. Fixed-origin download, frozen matching/apply, TQSL upload and all eQSL owners remain outstanding.</x:v>
       </x:c>
       <x:c r="C27" s="67" t="str">
         <x:v>Documented — direct upload/download, QSL statistics and paper-QSL workflows.</x:v>
@@ -1240,12 +1240,12 @@
       </x:c>
       <x:c r="F30" s="59"/>
     </x:row>
-    <x:row r="31" ht="24" hidden="0" customHeight="1">
+    <x:row r="31" ht="36" hidden="0" customHeight="1">
       <x:c r="A31" s="66" t="str">
         <x:v>Spot History</x:v>
       </x:c>
       <x:c r="B31" s="67" t="str">
-        <x:v>Source complete — separate retained local reports, search/filter/statistics and read-only review. Detached column controls exist; packaged/live retention acceptance remains open.</x:v>
+        <x:v>Source complete — separate retained local reports, search/filter/statistics and read-only review. Detached visibility, width and keyboard-accessible column ordering persist while headers, cells and widths move together; packaged/live retention acceptance remains open.</x:v>
       </x:c>
       <x:c r="C31" s="67" t="str">
         <x:v>Documented — incoming cluster data and spot/search workflows; exact retained-history model differs.</x:v>
@@ -1258,12 +1258,12 @@
       </x:c>
       <x:c r="F31" s="59"/>
     </x:row>
-    <x:row r="32" ht="48" hidden="0" customHeight="1">
+    <x:row r="32" ht="60" hidden="0" customHeight="1">
       <x:c r="A32" s="66" t="str">
         <x:v>Named DX/WSJT-X alert rules</x:v>
       </x:c>
       <x:c r="B32" s="67" t="str">
-        <x:v>Source complete — independently enabled structured rules, all matching names, bounded dedup/rate limiting and passive recent-alert dashboard. Each retained event explains its call/DXCC/band/mode/special evidence and first-to-last report history; compact windows use cards instead of horizontal scrolling.</x:v>
+        <x:v>Source complete — independently enabled structured rules, all matching names, bounded dedup/rate limiting and passive recent-alert dashboard. Retained events explain evidence/history, sort deterministically, and support exact-UUID selective clearing that preserves rules, source baselines, delivery limits and no-replay state; compact windows use cards instead of horizontal scrolling.</x:v>
       </x:c>
       <x:c r="C32" s="67" t="str">
         <x:v>Documented — DXCC/band/mode/IOTA novelty, confirmation source choices, wildcard station watches and optional spoken delivery.</x:v>
@@ -1402,12 +1402,12 @@
       </x:c>
       <x:c r="F39" s="59"/>
     </x:row>
-    <x:row r="40" ht="300" hidden="0" customHeight="1">
+    <x:row r="40" ht="96" hidden="0" customHeight="1">
       <x:c r="A40" s="66" t="str">
         <x:v>TCI rig control — SunSDR/ExpertSDR and compatible servers</x:v>
       </x:c>
       <x:c r="B40" s="67" t="str">
-        <x:v>Source complete for receive tune/filter, passive configured-TRX split/TX-frequency, APP_FOCUS, addressed/legacy spot clicks, receipt-only CW_MACROS_EMPTY/CALLSIGN_SEND, per-address VFO_LOCK, RX_CHANNEL_SENSORS, separate deprecated RX_SENSORS, formal-five-field TX_SENSORS, global MUTE/VOLUME and receiver RX_MUTE observations. Independent raw tokens/producer receipts do not establish physical power/calibration, queue-empty, contact identity, command correlation, configured freshness/readiness, control, TX completion or RF authority. 4a34eb4 adds passive RX_VOLUME exact raw [-60,0] dB per receiver/channel (agent 107/107; root focused 6/6). 63ef8b2 separately adds RX_BALANCE exact raw [-40,40] dB per receiver/channel (agent 113/113; root focused 6/6). Both have independent receipts, discovery-shrink pruning and reconnect clearing; no global mute/volume relationships, measured stereo output, audibility or streaming inference. Existing no-replay/readback owner is unchanged. Recurring testDroppingLastSessionReferenceClosesPendingConnection closeCount 0 vs 1 failure remains open; passing focused checks are not a lifecycle fix. Transmit/PTT, split/TX-VFO controls, outbound spots, audio/IQ and package/native/live station/provider/network/RF acceptance remain open. Earlier source/test history is retained in project tracking docs. Installed alpha.31 unchanged. d2b2d24 adds independent passive global MON_VOLUME exact raw [-60,0] dB with its own receipt/reconnect reset (agent 118/118; root focused 5/5). No relationship to other audio/mute and no monitoring/TX/readiness/RF inference; package/native/live acceptance stays open. c54cc0f adds passive global MON_ENABLE exact boolean token plus parsed setting, independent receipt/reset (agent 123/123; root focused 5/5). Independent of MON_VOLUME; no monitoring/audibility/streaming/TX/readiness/control/RF inference. b1691a5 adds passive receiver AGC_MODE normal/fast/off exact token plus typed mode, independent receipt, TRX pruning/reconnect reset (agent 129/129; root focused 6/6). No gain/modulation/receiver-enable/audio/readiness/control/RF inference.</x:v>
+        <x:v>Source complete for receive tune/filter and bounded passive telemetry, including configured-TRX split/TX-frequency, spots, sensors, locks, mute/volume/balance, monitor state, AGC mode, RX_BIN_ENABLE and RX_NR_ENABLE. Independent exact tokens and producer receipts are pruned/reset with discovery/lifecycle changes and never establish audibility, capability, configured readiness, control, TX completion or RF authority. Existing no-replay/readback owner is unchanged. Transmit/PTT, split/TX-VFO controls, outbound spots, audio/IQ and package/native/live station/provider/network/RF acceptance remain open. Installed alpha.32 is exact source e270ab5; later TCI observations are source-only.</x:v>
       </x:c>
       <x:c r="C40" s="67" t="str">
         <x:v>Not established in the reviewed primary RUMlogNG evidence.</x:v>
@@ -2844,7 +2844,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R255c860418eb4f16"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R23dc6c14c958421a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3068,7 +3068,7 @@
         <x:v>Official/date-qualified CTY rules</x:v>
       </x:c>
     </x:row>
-    <x:row r="14" ht="312" hidden="0" customHeight="1">
+    <x:row r="14" ht="288" hidden="0" customHeight="1">
       <x:c r="A14" s="66" t="str">
         <x:v>P1</x:v>
       </x:c>
@@ -3076,7 +3076,7 @@
         <x:v>Full TCI radio provider</x:v>
       </x:c>
       <x:c r="C14" s="67" t="str">
-        <x:v>Receive tune/filter and bounded passive telemetry source complete; full history/counts in project docs and Feature Matrix. Independent RX_VOLUME/RX_BALANCE, global MON_VOLUME (d2b2d24: 118/118 + root 5/5) and MON_ENABLE (c54cc0f: 123/123 + root 5/5) receipts/reset confer no audio/monitoring authority. AGC_MODE b1691a5: receiver normal/fast/off exact token/typed mode, independent receipt, TRX pruning/reset; agent 129/129 + root 6/6. No gain/modulation/receiver-enable/audio/readiness/control/RF inference. closeCount 0 vs 1 lifecycle failure and package/native/live station/provider/network/RF gates remain open.</x:v>
+        <x:v>Receive tune/filter and bounded passive telemetry source complete; full history/counts in project docs and Feature Matrix. Independent RX_VOLUME/RX_BALANCE, MON_VOLUME/MON_ENABLE, AGC_MODE, RX_BIN_ENABLE and RX_NR_ENABLE receipts/reset confer no audio, audibility, capability, configured readiness, control or RF authority. RX_BIN_ENABLE fd12703: 147/147 focused; RX_NR_ENABLE 7fe73ea: 153/153 focused. The closeCount lifecycle failure and package/native/live station/provider/network/RF gates remain open.</x:v>
       </x:c>
       <x:c r="D14" s="67" t="str">
         <x:v>Extend the existing no-replay owner with separately reviewed split/TX-VFO controls, urgent release and optional audio/IQ slices; passive notifications never become configured evidence/inventory or CW/RF authority. Transmit/PTT keeps its own explicit authority.</x:v>
@@ -3108,7 +3108,7 @@
         <x:v>RUMlogNG entity/QSO search surfaces</x:v>
       </x:c>
     </x:row>
-    <x:row r="16" ht="24" hidden="0" customHeight="1">
+    <x:row r="16" ht="36" hidden="0" customHeight="1">
       <x:c r="A16" s="66" t="str">
         <x:v>P1</x:v>
       </x:c>
@@ -3116,16 +3116,16 @@
         <x:v>Direct LoTW/eQSL</x:v>
       </x:c>
       <x:c r="C16" s="67" t="str">
-        <x:v>Outstanding</x:v>
+        <x:v>LoTW report parser source foundation complete</x:v>
       </x:c>
       <x:c r="D16" s="67" t="str">
-        <x:v>Design separate vault, receipt, reconciliation and no-replay owners; do not piggyback on Wavelog credentials.</x:v>
+        <x:v>Add a fixed-origin manual LoTW download, frozen match/change preview and confirmation-only revision-fenced apply with no outbox; keep TQSL signing/upload and eQSL as separate provider owners. Never piggyback on Wavelog credentials.</x:v>
       </x:c>
       <x:c r="E16" s="67" t="str">
-        <x:v>Provider sandbox/live-account acceptance</x:v>
+        <x:v>Parser 12/12; remaining provider sandbox/live-account, exact-package and no-outbox acceptance</x:v>
       </x:c>
       <x:c r="F16" s="67" t="str">
-        <x:v>RUMlogNG and QLog service workflows</x:v>
+        <x:v>RUMlogNG and QLog service workflows; official ARRL LoTW query/TQSL contracts</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="24" hidden="0" customHeight="1">
@@ -3179,7 +3179,7 @@
         <x:v>Source complete</x:v>
       </x:c>
       <x:c r="D19" s="67" t="str">
-        <x:v>Verify popup, optional sound, expiry, clear and suppression counters from real retained cluster/WSJT-X traffic.</x:v>
+        <x:v>Verify popup, optional sound, expiry, deterministic sorting, selective/all clearing and suppression counters from real retained cluster/WSJT-X traffic.</x:v>
       </x:c>
       <x:c r="E19" s="67" t="str">
         <x:v>Installed live-cluster evidence</x:v>
@@ -3199,7 +3199,7 @@
         <x:v>Source complete</x:v>
       </x:c>
       <x:c r="D20" s="67" t="str">
-        <x:v>Package-test Save/Apply/Clone/Rename/Delete against the canonical query and verify keyboard/focus behavior across window contexts.</x:v>
+        <x:v>Package-test Save/Apply/Clone/Rename/Update/Delete against the canonical query and verify keyboard/focus behavior across window contexts.</x:v>
       </x:c>
       <x:c r="E20" s="67" t="str">
         <x:v>Exact-source package, UX and persistence acceptance</x:v>
@@ -4770,7 +4770,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7510d9d0b576408b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re68ecfc3f806416b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4941,7 +4941,7 @@
       </x:c>
       <x:c r="F11" s="59"/>
     </x:row>
-    <x:row r="12" ht="24" hidden="0" customHeight="1">
+    <x:row r="12" ht="36" hidden="0" customHeight="1">
       <x:c r="A12" s="66" t="str">
         <x:v>R06</x:v>
       </x:c>
@@ -4955,7 +4955,7 @@
         <x:v>Opportunity feeds, spots, alerts, awards and history</x:v>
       </x:c>
       <x:c r="E12" s="67" t="str">
-        <x:v>Package-test 52010e3; retain explicit cluster-provenance exclusion.</x:v>
+        <x:v>Package-test 52010e3 plus Spot History ordering 82bcbee and deterministic/selective Alerts f517d9a/685f468; retain explicit cluster-provenance exclusion and no station actions.</x:v>
       </x:c>
       <x:c r="F12" s="59"/>
     </x:row>
@@ -4977,7 +4977,7 @@
       </x:c>
       <x:c r="F13" s="59"/>
     </x:row>
-    <x:row r="14" ht="15" hidden="0" customHeight="1">
+    <x:row r="14" ht="36" hidden="0" customHeight="1">
       <x:c r="A14" s="66" t="str">
         <x:v>R08</x:v>
       </x:c>
@@ -4985,13 +4985,13 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="C14" s="67" t="str">
-        <x:v>Existing service programme</x:v>
+        <x:v>LoTW report parser source foundation complete</x:v>
       </x:c>
       <x:c r="D14" s="67" t="str">
-        <x:v>Vault plus durable claim/receipt patterns</x:v>
+        <x:v>Dedicated LoTW envelope parser plus vault and durable claim/receipt patterns</x:v>
       </x:c>
       <x:c r="E14" s="67" t="str">
-        <x:v>Direct LoTW/TQSL station/certificate/upload/download owner.</x:v>
+        <x:v>3c6f26f parses bounded LoTW-only confirmation evidence (12/12) without network/DB action. Add fixed-origin download, frozen preview and no-outbox apply; keep TQSL signing/upload and eQSL separate.</x:v>
       </x:c>
       <x:c r="F14" s="59"/>
     </x:row>
@@ -5117,7 +5117,7 @@
         <x:v>Logbook query snapshot and canonical detached history context</x:v>
       </x:c>
       <x:c r="E21" s="67" t="str">
-        <x:v>Package-test native history plus cloneable canonical filters.</x:v>
+        <x:v>2f00a55 adds query-only Update with no implicit Apply. Package-test native history plus Save/Apply/Clone/Rename/Update/Delete persistence.</x:v>
       </x:c>
       <x:c r="F21" s="59"/>
     </x:row>
@@ -6657,7 +6657,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3e938aa2b7c14a82"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rea818cf0049f43e6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6732,34 +6732,34 @@
       <x:c r="E6" s="59"/>
       <x:c r="F6" s="59"/>
     </x:row>
-    <x:row r="7" ht="36" hidden="0" customHeight="1">
+    <x:row r="7" ht="48" hidden="0" customHeight="1">
       <x:c r="A7" s="64" t="str">
         <x:v>OM0RX-xLog</x:v>
       </x:c>
       <x:c r="B7" s="65" t="str">
-        <x:v>Current implementation checkpoint b1691a5712ef9e8bbcd29038f12ade0954334735</x:v>
+        <x:v>Current implementation checkpoint 3c6f26fbf9d213090ebf4e759c64b281c640d488</x:v>
       </x:c>
       <x:c r="C7" s="65" t="str">
         <x:v>2026-10-16</x:v>
       </x:c>
       <x:c r="D7" s="65" t="str">
-        <x:v>PROJECT_STATUS.md, PROJECT_BOARD.md, operator-feedback tracker and enhancement-recommendations reconciliation. Source/test/browser results remain separate from package/native/live/hardware acceptance; installed alpha.31 is unchanged.</x:v>
+        <x:v>PROJECT_STATUS.md, PROJECT_BOARD.md, operator-feedback tracker and enhancement-recommendations reconciliation. Source/test/browser results remain separate from package/native/live/hardware acceptance. Installed alpha.32 is the separately accepted exact source e270ab5; later commits are not claimed inside that bundle.</x:v>
       </x:c>
       <x:c r="E7" s="59"/>
       <x:c r="F7" s="59"/>
     </x:row>
-    <x:row r="8" ht="228" hidden="0" customHeight="1">
+    <x:row r="8" ht="60" hidden="0" customHeight="1">
       <x:c r="A8" s="66" t="str">
         <x:v>OM0RX-xLog</x:v>
       </x:c>
       <x:c r="B8" s="67" t="str">
-        <x:v>https://github.com/oliverbross/OM0RX-xLog/commit/b1691a5712ef9e8bbcd29038f12ade0954334735</x:v>
+        <x:v>https://github.com/oliverbross/OM0RX-xLog/commit/3c6f26fbf9d213090ebf4e759c64b281c640d488</x:v>
       </x:c>
       <x:c r="C8" s="67" t="str">
         <x:v>2026-10-16</x:v>
       </x:c>
       <x:c r="D8" s="67" t="str">
-        <x:v>Accepted source increments after tracking 3acfc4d: RX_VOLUME 4a34eb4 (107/107 + root 6/6); PSKAM31 90f7a3e (Swift 18/18, frontend 1,218/1,218, tsc); PSKAM50 e34a094 (Swift 18/18, frontend 1,234/1,234, tsc); pure contact-update validation/diff 33e5eb4 (new 6/6 + regressions 15/15, root 6/6); RX_BALANCE 63ef8b2 (113/113 + root 6/6). Focused/source-level evidence only. Installed alpha.31 and ADIF_VER 3.1.7 unchanged; recurring closeCount lifecycle failure, correction UI/apply/undo, package/native/live station/provider/network/RF acceptance remain open. Later increments: PSKFEC31 8c43ef5 (Swift 18/18, frontend 1,250/1,250, tsc); MON_VOLUME d2b2d24 (118/118 + root 5/5); exact-evidence-fenced CTY DXCC-only correction preview 8ccffe7 (root 2/2 plus data-quality regression), without apply/undo/UI/operation ID/receipt/journal/provider correction or live acceptance. New source increments: Details-only CTY DXCC preview UI 327648c (Swift 2/2, UI/bridge 22/22, tsc; no apply/undo); PSKHELL 9e8b97b import-only to HELL (Swift 18/18, frontend 1,266/1,266, tsc; root reviewed/diff checked); passive MON_ENABLE c54cc0f (123/123 + root 5/5), independent setting/receipt/reset with no monitoring/audibility/streaming/TX/readiness/control/RF inference. ADIF_VER remains 3.1.7; installed alpha.31 unchanged. Since c54cc0f: synthetic Wavelog confirmation-refresh regression 7adb008 (1/1; preserved local-only fields, no outbox/conflict, idempotent second sync; no live provider); QPSK31 8934ab6 import-only to PSK (agent Swift 18/18, frontend 1,282/1,282, tsc; root frontend 1,282/1,282, tsc/diff); passive receiver AGC_MODE b1691a5 (129/129 + root 6/6; exact token/typed mode, independent receipt/TRX pruning/reset; no gain/modulation/receiver-enable/audio/readiness/control/RF inference). All existing acceptance limits remain open.</x:v>
+        <x:v>Current RUMlog-first/QLog-second source increments after installed alpha.32: Logbook ordering 544b763; Alerts sorting f517d9a; passive TCI RX_BIN_ENABLE fd12703; Spot History ordering 82bcbee; passive TCI RX_NR_ENABLE 7fe73ea; selective Alerts clearing 685f468; saved-filter query Update 2f00a55; bounded LoTW confirmation-envelope parser 3c6f26f (12/12). Focused/source evidence only; package/native/live provider/station/network/RF acceptance remains open.</x:v>
       </x:c>
       <x:c r="E8" s="59"/>
       <x:c r="F8" s="59"/>
@@ -6894,113 +6894,129 @@
     </x:row>
     <x:row r="17" ht="24" hidden="0" customHeight="1">
       <x:c r="A17" s="66" t="str">
-        <x:v>TCI protocol</x:v>
+        <x:v>LoTW</x:v>
       </x:c>
       <x:c r="B17" s="67" t="str">
-        <x:v>https://github.com/ExpertSDR3/TCI/tree/b081213ff97150fd29f669c633f060f93c81a286</x:v>
+        <x:v>https://lotw.arrl.org/lotw-help/developer-query-qsos-qsls/</x:v>
       </x:c>
       <x:c r="C17" s="67" t="str">
         <x:v>2026-10-16</x:v>
       </x:c>
       <x:c r="D17" s="67" t="str">
-        <x:v>Pinned official ExpertSDR3 MIT protocol source for the original codec/reducer implementation; no QLog implementation code was copied.</x:v>
+        <x:v>Official ARRL GET/report contract used for the dedicated confirmation-envelope parser and download plan; no account request or credential use was performed.</x:v>
       </x:c>
       <x:c r="E17" s="59"/>
       <x:c r="F17" s="59"/>
     </x:row>
     <x:row r="18" ht="24" hidden="0" customHeight="1">
       <x:c r="A18" s="66" t="str">
-        <x:v>Comparison method</x:v>
+        <x:v>LoTW/TQSL</x:v>
       </x:c>
       <x:c r="B18" s="67" t="str">
-        <x:v>RUMLOG_WORKFLOW_GAP_AUDIT_2026-10-14.md; QLOG_WORKFLOW_GAP_AUDIT_2026-10-15.md; OPSLOG_REFERENCE_AUDIT_2026-10-16.md</x:v>
+        <x:v>https://lotw.arrl.org/lotw-help/developer-submit-qsos/</x:v>
       </x:c>
       <x:c r="C18" s="67" t="str">
         <x:v>2026-10-16</x:v>
       </x:c>
       <x:c r="D18" s="67" t="str">
-        <x:v>Behavioral inspiration only. No third-party source, artwork, settings, credentials or logbook data is copied into OM0RX-xLog.</x:v>
+        <x:v>Official ARRL submission boundary: certificate/station-location signing and upload remain separate from report download and are not implemented by the parser stage.</x:v>
       </x:c>
       <x:c r="E18" s="59"/>
       <x:c r="F18" s="59"/>
     </x:row>
-    <x:row r="19" ht="36" hidden="0" customHeight="1">
+    <x:row r="19" ht="24" hidden="0" customHeight="1">
       <x:c r="A19" s="66" t="str">
-        <x:v>Reference order</x:v>
+        <x:v>TCI protocol</x:v>
       </x:c>
       <x:c r="B19" s="67" t="str">
-        <x:v>RUMlogNG #1; QLog #2; OpsLog #3</x:v>
+        <x:v>https://github.com/ExpertSDR3/TCI/tree/b081213ff97150fd29f669c633f060f93c81a286</x:v>
       </x:c>
       <x:c r="C19" s="67" t="str">
         <x:v>2026-10-16</x:v>
       </x:c>
       <x:c r="D19" s="67" t="str">
-        <x:v>OpsLog is documented supplementary only until current source and application licensing can be reviewed. Existing xLog checkpoint/test/acceptance limits remain unchanged. See docs/OPSLOG_REFERENCE_AUDIT_2026-10-16.md.</x:v>
+        <x:v>Pinned official ExpertSDR3 MIT protocol source for the original codec/reducer implementation; no QLog implementation code was copied.</x:v>
       </x:c>
       <x:c r="E19" s="59"/>
       <x:c r="F19" s="59"/>
     </x:row>
     <x:row r="20" ht="24" hidden="0" customHeight="1">
       <x:c r="A20" s="66" t="str">
-        <x:v>OpsLog (#3)</x:v>
+        <x:v>Comparison method</x:v>
       </x:c>
       <x:c r="B20" s="67" t="str">
-        <x:v>https://github.com/GregTroar/OpsLog/releases/tag/v0.51.10</x:v>
+        <x:v>RUMLOG_WORKFLOW_GAP_AUDIT_2026-10-14.md; QLOG_WORKFLOW_GAP_AUDIT_2026-10-15.md; OPSLOG_REFERENCE_AUDIT_2026-10-16.md</x:v>
       </x:c>
       <x:c r="C20" s="67" t="str">
         <x:v>2026-10-16</x:v>
       </x:c>
       <x:c r="D20" s="67" t="str">
-        <x:v>Official release published 2026-10-15. Mirror tag SHA b30bd55c3de979edc76a965034e8d2f7fd5fdc12. Release notes supply acceptance ideas, not independent runtime/source verification.</x:v>
+        <x:v>Behavioral inspiration only. No third-party source, artwork, settings, credentials or logbook data is copied into OM0RX-xLog.</x:v>
       </x:c>
       <x:c r="E20" s="59"/>
       <x:c r="F20" s="59"/>
     </x:row>
     <x:row r="21" ht="36" hidden="0" customHeight="1">
       <x:c r="A21" s="66" t="str">
-        <x:v>OpsLog (#3)</x:v>
+        <x:v>Reference order</x:v>
       </x:c>
       <x:c r="B21" s="67" t="str">
-        <x:v>https://github.com/GregTroar/OpsLog/blob/b30bd55c3de979edc76a965034e8d2f7fd5fdc12/README.md</x:v>
+        <x:v>RUMlogNG #1; QLog #2; OpsLog #3</x:v>
       </x:c>
       <x:c r="C21" s="67" t="str">
         <x:v>2026-10-16</x:v>
       </x:c>
       <x:c r="D21" s="67" t="str">
-        <x:v>Public tag contains README.md and README.fr.md only. Documented Wails 2.11/Go/React/TypeScript/Vite, SQLite configuration and optional shared MySQL log; feature statements in OpsLog column are documentation claims.</x:v>
+        <x:v>OpsLog is documented supplementary only until current source and application licensing can be reviewed. Existing xLog checkpoint/test/acceptance limits remain unchanged. See docs/OPSLOG_REFERENCE_AUDIT_2026-10-16.md.</x:v>
       </x:c>
       <x:c r="E21" s="59"/>
       <x:c r="F21" s="59"/>
     </x:row>
-    <x:row r="22" ht="36" hidden="0" customHeight="1">
+    <x:row r="22" ht="24" hidden="0" customHeight="1">
       <x:c r="A22" s="66" t="str">
         <x:v>OpsLog (#3)</x:v>
       </x:c>
       <x:c r="B22" s="67" t="str">
-        <x:v>https://git.rouggy.com/rouggy/OpsLog</x:v>
+        <x:v>https://github.com/GregTroar/OpsLog/releases/tag/v0.51.10</x:v>
       </x:c>
       <x:c r="C22" s="67" t="str">
         <x:v>2026-10-16</x:v>
       </x:c>
       <x:c r="D22" s="67" t="str">
-        <x:v>Actual source authority is authentication-gated: Git credentials, web/archive sign-in and API 403 in access audit. GitHub API license:null; no app source licence found. Not current-source-reviewed or licence-verified; no code copied.</x:v>
+        <x:v>Official release published 2026-10-15. Mirror tag SHA b30bd55c3de979edc76a965034e8d2f7fd5fdc12. Release notes supply acceptance ideas, not independent runtime/source verification.</x:v>
       </x:c>
       <x:c r="E22" s="59"/>
       <x:c r="F22" s="59"/>
     </x:row>
-    <x:row r="23" ht="15" hidden="0" customHeight="1">
-      <x:c r="A23" s="59"/>
-      <x:c r="B23" s="59"/>
-      <x:c r="C23" s="59"/>
-      <x:c r="D23" s="59"/>
+    <x:row r="23" ht="36" hidden="0" customHeight="1">
+      <x:c r="A23" s="66" t="str">
+        <x:v>OpsLog (#3)</x:v>
+      </x:c>
+      <x:c r="B23" s="67" t="str">
+        <x:v>https://github.com/GregTroar/OpsLog/blob/b30bd55c3de979edc76a965034e8d2f7fd5fdc12/README.md</x:v>
+      </x:c>
+      <x:c r="C23" s="67" t="str">
+        <x:v>2026-10-16</x:v>
+      </x:c>
+      <x:c r="D23" s="67" t="str">
+        <x:v>Public tag contains README.md and README.fr.md only. Documented Wails 2.11/Go/React/TypeScript/Vite, SQLite configuration and optional shared MySQL log; feature statements in OpsLog column are documentation claims.</x:v>
+      </x:c>
       <x:c r="E23" s="59"/>
       <x:c r="F23" s="59"/>
     </x:row>
-    <x:row r="24" ht="15" hidden="0" customHeight="1">
-      <x:c r="A24" s="59"/>
-      <x:c r="B24" s="59"/>
-      <x:c r="C24" s="59"/>
-      <x:c r="D24" s="59"/>
+    <x:row r="24" ht="36" hidden="0" customHeight="1">
+      <x:c r="A24" s="66" t="str">
+        <x:v>OpsLog (#3)</x:v>
+      </x:c>
+      <x:c r="B24" s="67" t="str">
+        <x:v>https://git.rouggy.com/rouggy/OpsLog</x:v>
+      </x:c>
+      <x:c r="C24" s="67" t="str">
+        <x:v>2026-10-16</x:v>
+      </x:c>
+      <x:c r="D24" s="67" t="str">
+        <x:v>Actual source authority is authentication-gated: Git credentials, web/archive sign-in and API 403 in access audit. GitHub API license:null; no app source licence found. Not current-source-reviewed or licence-verified; no code copied.</x:v>
+      </x:c>
       <x:c r="E24" s="59"/>
       <x:c r="F24" s="59"/>
     </x:row>
@@ -8418,7 +8434,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6d33e553516340c0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5abb3661bd2a4ff5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Track LoTW preview and alert columns
</commit_message>
<xml_diff>
--- a/outputs/feature-matrix-2026-10-16/OM0RX-xLog_Feature_Comparison_2026-10-16.xlsx
+++ b/outputs/feature-matrix-2026-10-16/OM0RX-xLog_Feature_Comparison_2026-10-16.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Matrix" sheetId="1" r:id="R2886a8031864445c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Outstanding" sheetId="2" r:id="R874a728c194047cd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enhancement Review" sheetId="3" r:id="Rb3783e94713b4296"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="4" r:id="R44a768b7c6a04541"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Matrix" sheetId="1" r:id="R10038eb1e0574bce"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Outstanding" sheetId="2" r:id="Rd9d609b25ade475d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enhancement Review" sheetId="3" r:id="Re353701f90224821"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="4" r:id="R117ce6e1e46c4834"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1168,12 +1168,12 @@
       </x:c>
       <x:c r="F26" s="59"/>
     </x:row>
-    <x:row r="27" ht="60" hidden="0" customHeight="1">
+    <x:row r="27" ht="84" hidden="0" customHeight="1">
       <x:c r="A27" s="66" t="str">
         <x:v>Direct LoTW and eQSL workflows</x:v>
       </x:c>
       <x:c r="B27" s="67" t="str">
-        <x:v>Partial — LoTW parser foundation source complete: a dedicated bounded confirmation-report parser preserves report count, watermark, optional mode and LoTW-only evidence without generic ADIF import, paper-QSL mapping, credentials, network calls or database mutation. Fixed-origin download, frozen matching/apply, TQSL upload and all eQSL owners remain outstanding.</x:v>
+        <x:v>Partial — dedicated bounded LoTW parser plus fixed-origin GET plan, strict response validation and frozen station/generation/revision-fenced match/change preview are source complete (25/25 combined Swift). Mode only disambiguates multiple date/time/band/call matches; minute-only times retain minute precision, unmatched records are not inserted and positive confirmations are never downgraded. No credentials, network request or database action occurred. Redirect-disabled streaming transport, confirmation-only no-outbox apply, TQSL upload and all eQSL owners remain outstanding.</x:v>
       </x:c>
       <x:c r="C27" s="67" t="str">
         <x:v>Documented — direct upload/download, QSL statistics and paper-QSL workflows.</x:v>
@@ -1258,12 +1258,12 @@
       </x:c>
       <x:c r="F31" s="59"/>
     </x:row>
-    <x:row r="32" ht="60" hidden="0" customHeight="1">
+    <x:row r="32" ht="72" hidden="0" customHeight="1">
       <x:c r="A32" s="66" t="str">
         <x:v>Named DX/WSJT-X alert rules</x:v>
       </x:c>
       <x:c r="B32" s="67" t="str">
-        <x:v>Source complete — independently enabled structured rules, all matching names, bounded dedup/rate limiting and passive recent-alert dashboard. Retained events explain evidence/history, sort deterministically, and support exact-UUID selective clearing that preserves rules, source baselines, delivery limits and no-replay state; compact windows use cards instead of horizontal scrolling.</x:v>
+        <x:v>Source complete — independently enabled structured rules, all matching names, bounded dedup/rate limiting and passive recent-alert dashboard. Retained events explain evidence/history, sort deterministically, support exact-UUID selective clearing, and persist operator-selected table columns while Select/Call remain mandatory; compact cards retain all evidence. Presentation changes preserve rules, UUID selection, source baselines, delivery limits and no-replay state.</x:v>
       </x:c>
       <x:c r="C32" s="67" t="str">
         <x:v>Documented — DXCC/band/mode/IOTA novelty, confirmation source choices, wildcard station watches and optional spoken delivery.</x:v>
@@ -2844,7 +2844,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R23dc6c14c958421a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdbfee512ac9f4e04"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3116,13 +3116,13 @@
         <x:v>Direct LoTW/eQSL</x:v>
       </x:c>
       <x:c r="C16" s="67" t="str">
-        <x:v>LoTW report parser source foundation complete</x:v>
+        <x:v>LoTW request and frozen preview source foundation complete</x:v>
       </x:c>
       <x:c r="D16" s="67" t="str">
-        <x:v>Add a fixed-origin manual LoTW download, frozen match/change preview and confirmation-only revision-fenced apply with no outbox; keep TQSL signing/upload and eQSL as separate provider owners. Never piggyback on Wavelog credentials.</x:v>
+        <x:v>Add redirect-disabled bounded streaming transport and confirmation-only revision-fenced apply with no outbox; keep TQSL signing/upload and eQSL as separate provider owners. Never log GET credentials or piggyback on Wavelog credentials.</x:v>
       </x:c>
       <x:c r="E16" s="67" t="str">
-        <x:v>Parser 12/12; remaining provider sandbox/live-account, exact-package and no-outbox acceptance</x:v>
+        <x:v>Parser/request/preview 25/25; remaining transport/apply, provider sandbox/live-account, exact-package and no-outbox acceptance</x:v>
       </x:c>
       <x:c r="F16" s="67" t="str">
         <x:v>RUMlogNG and QLog service workflows; official ARRL LoTW query/TQSL contracts</x:v>
@@ -3168,7 +3168,7 @@
         <x:v>QLog and RUMlogNG UDP workflows</x:v>
       </x:c>
     </x:row>
-    <x:row r="19" ht="24" hidden="0" customHeight="1">
+    <x:row r="19" ht="36" hidden="0" customHeight="1">
       <x:c r="A19" s="66" t="str">
         <x:v>P1</x:v>
       </x:c>
@@ -3179,13 +3179,13 @@
         <x:v>Source complete</x:v>
       </x:c>
       <x:c r="D19" s="67" t="str">
-        <x:v>Verify popup, optional sound, expiry, deterministic sorting, selective/all clearing and suppression counters from real retained cluster/WSJT-X traffic.</x:v>
+        <x:v>Verify popup, optional sound, expiry, deterministic sorting, persisted column visibility, selective/all clearing and suppression counters from real retained cluster/WSJT-X traffic.</x:v>
       </x:c>
       <x:c r="E19" s="67" t="str">
-        <x:v>Installed live-cluster evidence</x:v>
+        <x:v>Installed live-cluster and compact/wide column-presentation evidence</x:v>
       </x:c>
       <x:c r="F19" s="67" t="str">
-        <x:v>QLog rule table and RUMlogNG novelty alarms</x:v>
+        <x:v>QLog rule table/columns and RUMlogNG novelty alarms</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="24" hidden="0" customHeight="1">
@@ -4770,7 +4770,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re68ecfc3f806416b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1461852dca36438b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4955,7 +4955,7 @@
         <x:v>Opportunity feeds, spots, alerts, awards and history</x:v>
       </x:c>
       <x:c r="E12" s="67" t="str">
-        <x:v>Package-test 52010e3 plus Spot History ordering 82bcbee and deterministic/selective Alerts f517d9a/685f468; retain explicit cluster-provenance exclusion and no station actions.</x:v>
+        <x:v>Package-test 52010e3 plus Spot History ordering 82bcbee and deterministic/selective/configurable-column Alerts f517d9a/685f468/27354a3; retain explicit cluster-provenance exclusion and no station actions.</x:v>
       </x:c>
       <x:c r="F12" s="59"/>
     </x:row>
@@ -4977,7 +4977,7 @@
       </x:c>
       <x:c r="F13" s="59"/>
     </x:row>
-    <x:row r="14" ht="36" hidden="0" customHeight="1">
+    <x:row r="14" ht="48" hidden="0" customHeight="1">
       <x:c r="A14" s="66" t="str">
         <x:v>R08</x:v>
       </x:c>
@@ -4985,13 +4985,13 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="C14" s="67" t="str">
-        <x:v>LoTW report parser source foundation complete</x:v>
+        <x:v>LoTW request and frozen preview source foundation complete</x:v>
       </x:c>
       <x:c r="D14" s="67" t="str">
-        <x:v>Dedicated LoTW envelope parser plus vault and durable claim/receipt patterns</x:v>
+        <x:v>Dedicated LoTW parser/request/preview plus vault and durable claim/receipt patterns</x:v>
       </x:c>
       <x:c r="E14" s="67" t="str">
-        <x:v>3c6f26f parses bounded LoTW-only confirmation evidence (12/12) without network/DB action. Add fixed-origin download, frozen preview and no-outbox apply; keep TQSL signing/upload and eQSL separate.</x:v>
+        <x:v>3c6f26f parses bounded LoTW-only evidence; 8a45a73 adds fixed-origin GET planning, response validation and frozen match/change preview (25/25 combined) without live request or DB action. Add redirect-disabled streaming transport and revision-fenced no-outbox apply; keep TQSL signing/upload and eQSL separate.</x:v>
       </x:c>
       <x:c r="F14" s="59"/>
     </x:row>
@@ -6657,7 +6657,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rea818cf0049f43e6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2feef3f1eb474692"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6737,7 +6737,7 @@
         <x:v>OM0RX-xLog</x:v>
       </x:c>
       <x:c r="B7" s="65" t="str">
-        <x:v>Current implementation checkpoint 3c6f26fbf9d213090ebf4e759c64b281c640d488</x:v>
+        <x:v>Current implementation checkpoint 27354a36f062f3790b2ee8f7b8ea4570d1b8d015</x:v>
       </x:c>
       <x:c r="C7" s="65" t="str">
         <x:v>2026-10-16</x:v>
@@ -6748,18 +6748,18 @@
       <x:c r="E7" s="59"/>
       <x:c r="F7" s="59"/>
     </x:row>
-    <x:row r="8" ht="60" hidden="0" customHeight="1">
+    <x:row r="8" ht="72" hidden="0" customHeight="1">
       <x:c r="A8" s="66" t="str">
         <x:v>OM0RX-xLog</x:v>
       </x:c>
       <x:c r="B8" s="67" t="str">
-        <x:v>https://github.com/oliverbross/OM0RX-xLog/commit/3c6f26fbf9d213090ebf4e759c64b281c640d488</x:v>
+        <x:v>https://github.com/oliverbross/OM0RX-xLog/commit/27354a36f062f3790b2ee8f7b8ea4570d1b8d015</x:v>
       </x:c>
       <x:c r="C8" s="67" t="str">
         <x:v>2026-10-16</x:v>
       </x:c>
       <x:c r="D8" s="67" t="str">
-        <x:v>Current RUMlog-first/QLog-second source increments after installed alpha.32: Logbook ordering 544b763; Alerts sorting f517d9a; passive TCI RX_BIN_ENABLE fd12703; Spot History ordering 82bcbee; passive TCI RX_NR_ENABLE 7fe73ea; selective Alerts clearing 685f468; saved-filter query Update 2f00a55; bounded LoTW confirmation-envelope parser 3c6f26f (12/12). Focused/source evidence only; package/native/live provider/station/network/RF acceptance remains open.</x:v>
+        <x:v>Current RUMlog-first/QLog-second source increments after installed alpha.32: Logbook ordering 544b763; Alerts sorting f517d9a; passive TCI RX_BIN_ENABLE fd12703; Spot History ordering 82bcbee; passive TCI RX_NR_ENABLE 7fe73ea; selective Alerts clearing 685f468; saved-filter query Update 2f00a55; bounded LoTW parser 3c6f26f; fixed-origin request/frozen preview 8a45a73 (25/25 combined); persisted Alerts columns 27354a3 (28/28 plus build). Focused/source evidence only; package/native/live provider/station/network/RF acceptance remains open.</x:v>
       </x:c>
       <x:c r="E8" s="59"/>
       <x:c r="F8" s="59"/>
@@ -8434,7 +8434,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5abb3661bd2a4ff5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re7b80c45bbce43c5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>